<commit_message>
Explore Pants: tela en almacén + Shorts R1 + uso total kg
- Existencias reales TH (985.8 kg) repartidas Explore ~2900 und + Shorts R1 ≥1500
- Shorts Negro/Gris CAB 0.14 · DAMA 0.12 kg/und
- Ranking color/talla dashboard; KIDS ~585; CAB 2XL mín. 8 por color
- Verificación: delta kg ≈ 0 por color (Explore + Shorts)

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/EXPLORE_PANTS_Proyeccion_Produccion.xlsx
+++ b/EXPLORE_PANTS_Proyeccion_Produccion.xlsx
@@ -12,16 +12,17 @@
     <sheet name="Cantidades por Colores" sheetId="3" r:id="rId3"/>
     <sheet name="Producción por Talla" sheetId="4" r:id="rId4"/>
     <sheet name="Verificación Tela" sheetId="5" r:id="rId5"/>
-    <sheet name="Compra en 2 Órdenes" sheetId="6" r:id="rId6"/>
-    <sheet name="Producción Color × Talla" sheetId="7" r:id="rId7"/>
-    <sheet name="Metodología" sheetId="8" r:id="rId8"/>
+    <sheet name="Shorts R1" sheetId="6" r:id="rId6"/>
+    <sheet name="Compra en 2 Órdenes" sheetId="7" r:id="rId7"/>
+    <sheet name="Producción Color × Talla" sheetId="8" r:id="rId8"/>
+    <sheet name="Metodología" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="115">
   <si>
     <t>EXPLORE PANTS — PROYECCIÓN ANCLADA A JUSTIFICACIÓN NOVAKTEX</t>
   </si>
@@ -29,7 +30,7 @@
     <t>Fuente: DATA_JUSTIFICACI_N_COMPRA_TELA_NOVAKTEX_REPEl_c4ef.xlsx</t>
   </si>
   <si>
-    <t>Producción objetivo (80% pendiente): 2,908 und</t>
+    <t>Meta Explore Pants: 2,900 und · Shorts R1 ≥ 1,500 und</t>
   </si>
   <si>
     <t>Demanda proyectada Jul–Dic: 2,228 und</t>
@@ -38,16 +39,16 @@
     <t>Stock referencia justificación: 2,988 und (1,636 tiendas + 1,352 taller)</t>
   </si>
   <si>
-    <t>Stock actual dashboard: 3,249 und</t>
-  </si>
-  <si>
-    <t>Tela ya comprada (referencia): 1089 kg Explore</t>
-  </si>
-  <si>
-    <t>Pedido total archivo (Explore + Shorts): 1088 kg · split 65% / 35%</t>
-  </si>
-  <si>
-    <t>Color/talla: ranking dashboard por género, ajustado a tela comprada (sin déficit kg)</t>
+    <t>Stock actual dashboard: 2,988 und</t>
+  </si>
+  <si>
+    <t>Tela en almacén (existencias): 985.8 kg · uso total Explore + Shorts</t>
+  </si>
+  <si>
+    <t>Shorts R1: Negro/Gris · CAB 0.14 · DAMA 0.12 kg/und</t>
+  </si>
+  <si>
+    <t>Color/talla Explore: ranking dashboard · CAB 2XL mín. 8 und por color</t>
   </si>
   <si>
     <t>KIDS 550–620 und · CAB sin 3XL</t>
@@ -134,15 +135,15 @@
     <t>% ventas dash.</t>
   </si>
   <si>
+    <t>Gris Oscuro</t>
+  </si>
+  <si>
+    <t>Kaki</t>
+  </si>
+  <si>
     <t>Negro</t>
   </si>
   <si>
-    <t>Gris Oscuro</t>
-  </si>
-  <si>
-    <t>Kaki</t>
-  </si>
-  <si>
     <t>Azul Marino</t>
   </si>
   <si>
@@ -224,22 +225,28 @@
     <t>EXPLORE PANTS — VERIFICACIÓN TELA NOVAKTEX REPEL COMPRADA</t>
   </si>
   <si>
-    <t>Compara und a producir vs kg de tela ya pedida por color.</t>
-  </si>
-  <si>
-    <t>Und</t>
-  </si>
-  <si>
-    <t>% compra</t>
-  </si>
-  <si>
-    <t>Kg necesario</t>
-  </si>
-  <si>
-    <t>Kg neto compra</t>
-  </si>
-  <si>
-    <t>Delta kg</t>
+    <t>Explore + Shorts R1 vs kg en existencias (objetivo: delta ≈ 0).</t>
+  </si>
+  <si>
+    <t>Und Explore</t>
+  </si>
+  <si>
+    <t>Kg Explore</t>
+  </si>
+  <si>
+    <t>Kg Shorts</t>
+  </si>
+  <si>
+    <t>Kg total</t>
+  </si>
+  <si>
+    <t>Kg existencia</t>
+  </si>
+  <si>
+    <t>Delta</t>
+  </si>
+  <si>
+    <t>Shorts R1 total: 1,689 und · 219.36 kg</t>
   </si>
   <si>
     <t>Consumo referencial por género (kg/und)</t>
@@ -248,6 +255,21 @@
     <t>Consumo ref.</t>
   </si>
   <si>
+    <t>SHORT SPORT R1 — NEGRO / GRIS OSCURO (CAB · DAMA)</t>
+  </si>
+  <si>
+    <t>Color tela</t>
+  </si>
+  <si>
+    <t>Total und</t>
+  </si>
+  <si>
+    <t>CAB</t>
+  </si>
+  <si>
+    <t>Kg tela</t>
+  </si>
+  <si>
     <t>PROPUESTA COMPRA 65% AHORA / 35% SEPTIEMBRE (archivo justificación)</t>
   </si>
   <si>
@@ -326,19 +348,19 @@
     <t>METODOLOGÍA — EXPLORE PANTS</t>
   </si>
   <si>
-    <t>1. TOTAL a producir: 2,908 und (80% pendiente, justificación Novaktex). La tela ya está comprada.</t>
-  </si>
-  <si>
-    <t>2. COLOR y TALLA: ranking del dashboard por género; se ajusta iterativamente para no exceder kg de tela comprada.</t>
-  </si>
-  <si>
-    <t>3. KIDS 550–620 und (meta 585); CAB/DAMA reparten el resto por ventas.</t>
-  </si>
-  <si>
-    <t>4. CAB sin 3XL · KIDS sin talla 1 · Gris (ventas) → Gris Oscuro (producción).</t>
-  </si>
-  <si>
-    <t>5. Verificación tela: kg necesario ≤ kg neto comprado por color (consumo ref. CAB 0.3 · DAMA 0.25 · KIDS 0.22).</t>
+    <t>1. Tela en almacén: 985.8 kg — se usa completa (Explore + Shorts R1).</t>
+  </si>
+  <si>
+    <t>2. Explore Pants meta ~2,900 und · Shorts R1 ≥ 1,500 und (Negro/Gris, CAB/DAMA).</t>
+  </si>
+  <si>
+    <t>3. COLOR/TALLA Explore: ranking dashboard; KIDS meta 585; CAB 2XL mín. 8 und por color.</t>
+  </si>
+  <si>
+    <t>4. Shorts: CAB 0.14 kg/und · DAMA 0.12 kg/und.</t>
+  </si>
+  <si>
+    <t>5. Explore: CAB 0.3 · DAMA 0.25 · KIDS 0.22 kg/und.</t>
   </si>
   <si>
     <t>6. Demanda Jul–Dic (2,228 und) y escenarios mensuales del archivo de justificación.</t>
@@ -895,7 +917,7 @@
         <v>760</v>
       </c>
       <c r="C26" s="4">
-        <v>1021</v>
+        <v>760</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -906,7 +928,7 @@
         <v>3668</v>
       </c>
       <c r="C27" s="4">
-        <v>3929</v>
+        <v>3660</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -925,10 +947,10 @@
         <v>28</v>
       </c>
       <c r="B30">
-        <v>1185</v>
+        <v>1145</v>
       </c>
       <c r="C30">
-        <v>1270</v>
+        <v>1227</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -936,10 +958,10 @@
         <v>29</v>
       </c>
       <c r="B31">
-        <v>1138</v>
+        <v>1174</v>
       </c>
       <c r="C31">
-        <v>1221</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -947,10 +969,10 @@
         <v>30</v>
       </c>
       <c r="B32">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="C32">
-        <v>633</v>
+        <v>635</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -958,10 +980,10 @@
         <v>31</v>
       </c>
       <c r="B33" s="5">
-        <v>2908</v>
+        <v>2905</v>
       </c>
       <c r="C33" s="5">
-        <v>3124</v>
+        <v>3117</v>
       </c>
     </row>
   </sheetData>
@@ -1006,13 +1028,13 @@
         <v>37</v>
       </c>
       <c r="B5" s="4">
-        <v>457</v>
+        <v>325</v>
       </c>
       <c r="C5" s="6">
-        <v>0.3856540084388186</v>
+        <v>0.2838427947598253</v>
       </c>
       <c r="D5" s="6">
-        <v>0.272</v>
+        <v>0.06900000000000001</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -1020,13 +1042,13 @@
         <v>38</v>
       </c>
       <c r="B6" s="4">
-        <v>328</v>
+        <v>282</v>
       </c>
       <c r="C6" s="6">
-        <v>0.2767932489451477</v>
+        <v>0.2462882096069869</v>
       </c>
       <c r="D6" s="6">
-        <v>0.196</v>
+        <v>0.211</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -1034,13 +1056,13 @@
         <v>39</v>
       </c>
       <c r="B7" s="4">
-        <v>218</v>
+        <v>263</v>
       </c>
       <c r="C7" s="6">
-        <v>0.1839662447257384</v>
+        <v>0.2296943231441048</v>
       </c>
       <c r="D7" s="6">
-        <v>0.21</v>
+        <v>0.252</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -1048,13 +1070,13 @@
         <v>40</v>
       </c>
       <c r="B8" s="4">
-        <v>103</v>
+        <v>201</v>
       </c>
       <c r="C8" s="6">
-        <v>0.08691983122362869</v>
+        <v>0.1755458515283843</v>
       </c>
       <c r="D8" s="6">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -1062,13 +1084,13 @@
         <v>41</v>
       </c>
       <c r="B9" s="4">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C9" s="6">
-        <v>0.06666666666666667</v>
+        <v>0.06462882096069869</v>
       </c>
       <c r="D9" s="6">
-        <v>0.162</v>
+        <v>0.164</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -1076,7 +1098,7 @@
         <v>31</v>
       </c>
       <c r="B10" s="4">
-        <v>1185</v>
+        <v>1145</v>
       </c>
       <c r="C10" s="7">
         <v>1</v>
@@ -1103,16 +1125,16 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B14" s="4">
-        <v>466</v>
+        <v>339</v>
       </c>
       <c r="C14" s="6">
-        <v>0.4094903339191564</v>
+        <v>0.2887563884156729</v>
       </c>
       <c r="D14" s="6">
-        <v>0.298</v>
+        <v>0.306</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -1120,27 +1142,27 @@
         <v>38</v>
       </c>
       <c r="B15" s="4">
-        <v>308</v>
+        <v>298</v>
       </c>
       <c r="C15" s="6">
-        <v>0.2706502636203866</v>
+        <v>0.2538330494037478</v>
       </c>
       <c r="D15" s="6">
-        <v>0.198</v>
+        <v>0.209</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B16" s="4">
-        <v>217</v>
+        <v>295</v>
       </c>
       <c r="C16" s="6">
-        <v>0.1906854130052724</v>
+        <v>0.2512776831345826</v>
       </c>
       <c r="D16" s="6">
-        <v>0.223</v>
+        <v>0.058</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -1148,13 +1170,13 @@
         <v>40</v>
       </c>
       <c r="B17" s="4">
-        <v>87</v>
+        <v>174</v>
       </c>
       <c r="C17" s="6">
-        <v>0.07644991212653779</v>
+        <v>0.1482112436115843</v>
       </c>
       <c r="D17" s="6">
-        <v>0.145</v>
+        <v>0.139</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -1162,13 +1184,13 @@
         <v>41</v>
       </c>
       <c r="B18" s="4">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="C18" s="6">
-        <v>0.05272407732864675</v>
+        <v>0.05792163543441227</v>
       </c>
       <c r="D18" s="6">
-        <v>0.136</v>
+        <v>0.142</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -1176,7 +1198,7 @@
         <v>31</v>
       </c>
       <c r="B19" s="4">
-        <v>1138</v>
+        <v>1174</v>
       </c>
       <c r="C19" s="7">
         <v>1</v>
@@ -1203,72 +1225,72 @@
     </row>
     <row r="23" spans="1:4">
       <c r="A23" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B23" s="4">
-        <v>214</v>
+        <v>255</v>
       </c>
       <c r="C23" s="6">
-        <v>0.3658119658119658</v>
+        <v>0.4351535836177474</v>
       </c>
       <c r="D23" s="6">
-        <v>0.225</v>
+        <v>0.298</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B24" s="4">
-        <v>146</v>
+        <v>170</v>
       </c>
       <c r="C24" s="6">
-        <v>0.2495726495726496</v>
+        <v>0.2901023890784983</v>
       </c>
       <c r="D24" s="6">
-        <v>0.154</v>
+        <v>0.225</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B25" s="4">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="C25" s="6">
-        <v>0.1777777777777778</v>
+        <v>0.1518771331058021</v>
       </c>
       <c r="D25" s="6">
-        <v>0.284</v>
+        <v>0.269</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B26" s="4">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="C26" s="6">
-        <v>0.1213675213675214</v>
+        <v>0.07508532423208192</v>
       </c>
       <c r="D26" s="6">
-        <v>0.253</v>
+        <v>0.045</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B27" s="4">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="C27" s="6">
-        <v>0.08547008547008547</v>
+        <v>0.04778156996587031</v>
       </c>
       <c r="D27" s="6">
-        <v>0.08400000000000001</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -1276,7 +1298,7 @@
         <v>31</v>
       </c>
       <c r="B28" s="4">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="C28" s="7">
         <v>1</v>
@@ -1316,53 +1338,53 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B4" s="4">
-        <v>1137</v>
+        <v>772</v>
       </c>
       <c r="C4" s="6">
-        <v>0.390990371389271</v>
+        <v>0.2657487091222031</v>
       </c>
       <c r="D4" s="6">
-        <v>0.3801652892561984</v>
+        <v>0.3223210782341178</v>
       </c>
       <c r="E4" s="8">
-        <v>414</v>
+        <v>317.7556</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B5" s="4">
-        <v>782</v>
+        <v>648</v>
       </c>
       <c r="C5" s="6">
-        <v>0.2689133425034388</v>
+        <v>0.2230636833046472</v>
       </c>
       <c r="D5" s="6">
-        <v>0.3314967860422406</v>
+        <v>0.2844671001033621</v>
       </c>
       <c r="E5" s="8">
-        <v>361</v>
+        <v>280.4378</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B6" s="4">
-        <v>485</v>
+        <v>624</v>
       </c>
       <c r="C6" s="6">
-        <v>0.1667812929848693</v>
+        <v>0.2148020654044751</v>
       </c>
       <c r="D6" s="6">
-        <v>0.1441689623507805</v>
+        <v>0.1713177091328877</v>
       </c>
       <c r="E6" s="8">
-        <v>157</v>
+        <v>168.8911</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -1370,16 +1392,16 @@
         <v>40</v>
       </c>
       <c r="B7" s="4">
-        <v>294</v>
+        <v>630</v>
       </c>
       <c r="C7" s="6">
-        <v>0.1011004126547455</v>
+        <v>0.2168674698795181</v>
       </c>
       <c r="D7" s="6">
-        <v>0.08356290174471992</v>
+        <v>0.1622064538507951</v>
       </c>
       <c r="E7" s="8">
-        <v>91</v>
+        <v>159.9089</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -1387,16 +1409,16 @@
         <v>41</v>
       </c>
       <c r="B8" s="4">
-        <v>210</v>
+        <v>231</v>
       </c>
       <c r="C8" s="6">
-        <v>0.07221458046767538</v>
+        <v>0.07951807228915662</v>
       </c>
       <c r="D8" s="6">
-        <v>0.06060606060606061</v>
+        <v>0.05968765867883735</v>
       </c>
       <c r="E8" s="8">
-        <v>66</v>
+        <v>58.84222</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -1404,7 +1426,7 @@
         <v>31</v>
       </c>
       <c r="B9" s="4">
-        <v>2908</v>
+        <v>2905</v>
       </c>
       <c r="C9" s="7">
         <v>1</v>
@@ -1413,7 +1435,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="8">
-        <v>1089</v>
+        <v>985.8356199999999</v>
       </c>
     </row>
   </sheetData>
@@ -1458,16 +1480,16 @@
         <v>52</v>
       </c>
       <c r="B5" s="6">
-        <v>0.1451476793248945</v>
+        <v>0.1248908296943231</v>
       </c>
       <c r="C5" s="6">
-        <v>0.141</v>
+        <v>0.136</v>
       </c>
       <c r="D5" s="4">
-        <v>172</v>
+        <v>143</v>
       </c>
       <c r="E5" s="4">
-        <v>185</v>
+        <v>154</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -1475,16 +1497,16 @@
         <v>53</v>
       </c>
       <c r="B6" s="6">
-        <v>0.329957805907173</v>
+        <v>0.3301310043668123</v>
       </c>
       <c r="C6" s="6">
-        <v>0.334</v>
+        <v>0.339</v>
       </c>
       <c r="D6" s="4">
-        <v>391</v>
+        <v>378</v>
       </c>
       <c r="E6" s="4">
-        <v>418</v>
+        <v>404</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -1492,16 +1514,16 @@
         <v>54</v>
       </c>
       <c r="B7" s="6">
-        <v>0.3341772151898734</v>
+        <v>0.3310043668122271</v>
       </c>
       <c r="C7" s="6">
-        <v>0.336</v>
+        <v>0.346</v>
       </c>
       <c r="D7" s="4">
-        <v>396</v>
+        <v>379</v>
       </c>
       <c r="E7" s="4">
-        <v>423</v>
+        <v>404</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -1509,16 +1531,16 @@
         <v>55</v>
       </c>
       <c r="B8" s="6">
-        <v>0.1763713080168776</v>
+        <v>0.1790393013100437</v>
       </c>
       <c r="C8" s="6">
-        <v>0.178</v>
+        <v>0.179</v>
       </c>
       <c r="D8" s="4">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="E8" s="4">
-        <v>224</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -1526,16 +1548,16 @@
         <v>56</v>
       </c>
       <c r="B9" s="6">
-        <v>0.01434599156118144</v>
+        <v>0.03493449781659388</v>
       </c>
       <c r="C9" s="6">
-        <v>0.011</v>
+        <v>0</v>
       </c>
       <c r="D9" s="4">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="E9" s="4">
-        <v>20</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -1549,7 +1571,7 @@
         <v>1</v>
       </c>
       <c r="D10" s="4">
-        <v>1185</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -1579,16 +1601,16 @@
         <v>58</v>
       </c>
       <c r="B14" s="6">
-        <v>0.1300527240773287</v>
+        <v>0.100511073253833</v>
       </c>
       <c r="C14" s="6">
-        <v>0.122</v>
+        <v>0.112</v>
       </c>
       <c r="D14" s="4">
-        <v>148</v>
+        <v>118</v>
       </c>
       <c r="E14" s="4">
-        <v>160</v>
+        <v>127</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -1596,16 +1618,16 @@
         <v>52</v>
       </c>
       <c r="B15" s="6">
-        <v>0.2478031634446397</v>
+        <v>0.2163543441226576</v>
       </c>
       <c r="C15" s="6">
-        <v>0.244</v>
+        <v>0.237</v>
       </c>
       <c r="D15" s="4">
-        <v>282</v>
+        <v>254</v>
       </c>
       <c r="E15" s="4">
-        <v>301</v>
+        <v>270</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -1613,16 +1635,16 @@
         <v>53</v>
       </c>
       <c r="B16" s="6">
-        <v>0.3014059753954306</v>
+        <v>0.3194207836456559</v>
       </c>
       <c r="C16" s="6">
-        <v>0.305</v>
+        <v>0.304</v>
       </c>
       <c r="D16" s="4">
-        <v>343</v>
+        <v>375</v>
       </c>
       <c r="E16" s="4">
-        <v>367</v>
+        <v>399</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -1630,16 +1652,16 @@
         <v>54</v>
       </c>
       <c r="B17" s="6">
-        <v>0.1704745166959578</v>
+        <v>0.1890971039182283</v>
       </c>
       <c r="C17" s="6">
-        <v>0.176</v>
+        <v>0.181</v>
       </c>
       <c r="D17" s="4">
-        <v>194</v>
+        <v>222</v>
       </c>
       <c r="E17" s="4">
-        <v>208</v>
+        <v>238</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -1647,16 +1669,16 @@
         <v>55</v>
       </c>
       <c r="B18" s="6">
-        <v>0.1493848857644991</v>
+        <v>0.1737649063032368</v>
       </c>
       <c r="C18" s="6">
-        <v>0.153</v>
+        <v>0.165</v>
       </c>
       <c r="D18" s="4">
-        <v>170</v>
+        <v>204</v>
       </c>
       <c r="E18" s="4">
-        <v>183</v>
+        <v>219</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -1664,7 +1686,7 @@
         <v>56</v>
       </c>
       <c r="B19" s="6">
-        <v>0.0008787346221441124</v>
+        <v>0.0008517887563884157</v>
       </c>
       <c r="C19" s="6">
         <v>0.001</v>
@@ -1687,7 +1709,7 @@
         <v>1</v>
       </c>
       <c r="D20" s="4">
-        <v>1138</v>
+        <v>1174</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -1717,16 +1739,16 @@
         <v>60</v>
       </c>
       <c r="B24" s="6">
-        <v>0.105982905982906</v>
+        <v>0.08532423208191127</v>
       </c>
       <c r="C24" s="6">
-        <v>0.09300000000000001</v>
+        <v>0.095</v>
       </c>
       <c r="D24" s="4">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="E24" s="4">
-        <v>68</v>
+        <v>56</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -1734,16 +1756,16 @@
         <v>61</v>
       </c>
       <c r="B25" s="6">
-        <v>0.1316239316239316</v>
+        <v>0.1518771331058021</v>
       </c>
       <c r="C25" s="6">
-        <v>0.131</v>
+        <v>0.139</v>
       </c>
       <c r="D25" s="4">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="E25" s="4">
-        <v>84</v>
+        <v>97</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -1751,16 +1773,16 @@
         <v>62</v>
       </c>
       <c r="B26" s="6">
-        <v>0.1076923076923077</v>
+        <v>0.09556313993174062</v>
       </c>
       <c r="C26" s="6">
-        <v>0.115</v>
+        <v>0.101</v>
       </c>
       <c r="D26" s="4">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="E26" s="4">
-        <v>69</v>
+        <v>61</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -1768,16 +1790,16 @@
         <v>63</v>
       </c>
       <c r="B27" s="6">
-        <v>0.2034188034188034</v>
+        <v>0.1860068259385665</v>
       </c>
       <c r="C27" s="6">
-        <v>0.198</v>
+        <v>0.202</v>
       </c>
       <c r="D27" s="4">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="E27" s="4">
-        <v>129</v>
+        <v>118</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -1785,16 +1807,16 @@
         <v>64</v>
       </c>
       <c r="B28" s="6">
-        <v>0.2205128205128205</v>
+        <v>0.2150170648464164</v>
       </c>
       <c r="C28" s="6">
-        <v>0.215</v>
+        <v>0.22</v>
       </c>
       <c r="D28" s="4">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="E28" s="4">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -1802,16 +1824,16 @@
         <v>65</v>
       </c>
       <c r="B29" s="6">
-        <v>0.2307692307692308</v>
+        <v>0.2662116040955632</v>
       </c>
       <c r="C29" s="6">
-        <v>0.248</v>
+        <v>0.244</v>
       </c>
       <c r="D29" s="4">
-        <v>135</v>
+        <v>156</v>
       </c>
       <c r="E29" s="4">
-        <v>145</v>
+        <v>167</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -1825,7 +1847,7 @@
         <v>1</v>
       </c>
       <c r="D30" s="4">
-        <v>585</v>
+        <v>586</v>
       </c>
     </row>
   </sheetData>
@@ -1835,7 +1857,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -1856,88 +1878,88 @@
         <v>68</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>35</v>
+        <v>69</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B6" s="4">
-        <v>1137</v>
-      </c>
-      <c r="C6" s="6">
-        <v>0.391</v>
-      </c>
-      <c r="D6" s="6">
-        <v>0.38</v>
+        <v>772</v>
+      </c>
+      <c r="C6" s="8">
+        <v>201.05</v>
+      </c>
+      <c r="D6" s="8">
+        <v>116.52</v>
       </c>
       <c r="E6" s="8">
-        <v>300.7</v>
+        <v>317.57</v>
       </c>
       <c r="F6" s="8">
-        <v>345</v>
+        <v>317.76</v>
       </c>
       <c r="G6" s="8">
-        <v>44.3</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B7" s="4">
-        <v>782</v>
-      </c>
-      <c r="C7" s="6">
-        <v>0.269</v>
-      </c>
-      <c r="D7" s="6">
-        <v>0.331</v>
+        <v>648</v>
+      </c>
+      <c r="C7" s="8">
+        <v>177.41</v>
+      </c>
+      <c r="D7" s="8">
+        <v>102.84</v>
       </c>
       <c r="E7" s="8">
-        <v>207.5</v>
+        <v>280.25</v>
       </c>
       <c r="F7" s="8">
-        <v>300.8</v>
+        <v>280.44</v>
       </c>
       <c r="G7" s="8">
-        <v>93.3</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B8" s="4">
-        <v>485</v>
-      </c>
-      <c r="C8" s="6">
-        <v>0.167</v>
-      </c>
-      <c r="D8" s="6">
-        <v>0.144</v>
+        <v>624</v>
+      </c>
+      <c r="C8" s="8">
+        <v>168.78</v>
+      </c>
+      <c r="D8" s="8">
+        <v>0</v>
       </c>
       <c r="E8" s="8">
-        <v>130.6</v>
+        <v>168.78</v>
       </c>
       <c r="F8" s="8">
-        <v>130.8</v>
+        <v>168.89</v>
       </c>
       <c r="G8" s="8">
-        <v>0.2</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -1945,22 +1967,22 @@
         <v>40</v>
       </c>
       <c r="B9" s="4">
-        <v>294</v>
-      </c>
-      <c r="C9" s="6">
-        <v>0.101</v>
-      </c>
-      <c r="D9" s="6">
-        <v>0.08400000000000001</v>
+        <v>630</v>
+      </c>
+      <c r="C9" s="8">
+        <v>159.9</v>
+      </c>
+      <c r="D9" s="8">
+        <v>0</v>
       </c>
       <c r="E9" s="8">
-        <v>75.5</v>
+        <v>159.9</v>
       </c>
       <c r="F9" s="8">
-        <v>75.8</v>
+        <v>159.91</v>
       </c>
       <c r="G9" s="8">
-        <v>0.3</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -1968,22 +1990,22 @@
         <v>41</v>
       </c>
       <c r="B10" s="4">
-        <v>210</v>
-      </c>
-      <c r="C10" s="6">
-        <v>0.07200000000000001</v>
-      </c>
-      <c r="D10" s="6">
-        <v>0.061</v>
+        <v>231</v>
+      </c>
+      <c r="C10" s="8">
+        <v>58.78</v>
+      </c>
+      <c r="D10" s="8">
+        <v>0</v>
       </c>
       <c r="E10" s="8">
-        <v>54.3</v>
+        <v>58.78</v>
       </c>
       <c r="F10" s="8">
-        <v>55</v>
+        <v>58.84</v>
       </c>
       <c r="G10" s="8">
-        <v>0.7</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -1991,52 +2013,57 @@
         <v>31</v>
       </c>
       <c r="B11" s="4">
-        <v>2908</v>
+        <v>2905</v>
       </c>
       <c r="E11" s="8">
-        <v>768.6</v>
+        <v>985.28</v>
       </c>
       <c r="F11" s="8">
-        <v>907.4</v>
+        <v>985.84</v>
       </c>
       <c r="G11" s="8">
-        <v>138.8</v>
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="2" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
-      <c r="A14" s="3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="3" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7">
-      <c r="A15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
-      <c r="A16" t="s">
-        <v>29</v>
-      </c>
-      <c r="B16">
-        <v>0.25</v>
+      <c r="B16" s="3" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
+        <v>28</v>
+      </c>
+      <c r="B17">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" t="s">
+        <v>29</v>
+      </c>
+      <c r="B18">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" t="s">
         <v>30</v>
       </c>
-      <c r="B17">
+      <c r="B19">
         <v>0.22</v>
       </c>
     </row>
@@ -2047,156 +2074,74 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B4" s="3" t="s">
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="B3" s="3" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="5" spans="1:3">
+      <c r="C3" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4">
+        <v>897</v>
+      </c>
+      <c r="C4">
+        <v>443</v>
+      </c>
+      <c r="D4">
+        <v>454</v>
+      </c>
+      <c r="E4">
+        <v>116.52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>80</v>
-      </c>
-      <c r="B5" s="8">
-        <v>361.2</v>
-      </c>
-      <c r="C5" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>82</v>
-      </c>
-      <c r="B6" s="8">
-        <v>125.1</v>
-      </c>
-      <c r="C6" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
-        <v>83</v>
-      </c>
-      <c r="B7" s="8">
-        <v>157</v>
-      </c>
-      <c r="C7" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="s">
-        <v>85</v>
-      </c>
-      <c r="B8" s="8">
-        <v>62.8</v>
-      </c>
-      <c r="C8" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="B9" s="8">
-        <v>706.1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11" s="2" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3">
-      <c r="A12" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3">
-      <c r="A13" t="s">
-        <v>90</v>
-      </c>
-      <c r="B13" s="8">
-        <v>157</v>
-      </c>
-      <c r="C13" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3">
-      <c r="A14" t="s">
-        <v>92</v>
-      </c>
-      <c r="B14" s="8">
-        <v>94.2</v>
-      </c>
-      <c r="C14" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3">
-      <c r="A15" t="s">
-        <v>93</v>
-      </c>
-      <c r="B15" s="8">
-        <v>65.59999999999999</v>
-      </c>
-      <c r="C15" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3">
-      <c r="A16" t="s">
-        <v>94</v>
-      </c>
-      <c r="B16" s="8">
-        <v>65.5</v>
-      </c>
-      <c r="C16" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2">
-      <c r="A17" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="B17" s="8">
-        <v>382.3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2">
-      <c r="A19" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="B19" s="8">
-        <v>1088.4</v>
+        <v>37</v>
+      </c>
+      <c r="B5">
+        <v>792</v>
+      </c>
+      <c r="C5">
+        <v>391</v>
+      </c>
+      <c r="D5">
+        <v>401</v>
+      </c>
+      <c r="E5">
+        <v>102.84</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="4">
+        <v>1689</v>
+      </c>
+      <c r="E6" s="8">
+        <v>219.36</v>
       </c>
     </row>
   </sheetData>
@@ -2206,477 +2151,156 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B5" s="8">
+        <v>361.2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>89</v>
+      </c>
+      <c r="B6" s="8">
+        <v>125.1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>90</v>
+      </c>
+      <c r="B7" s="8">
+        <v>157</v>
+      </c>
+      <c r="C7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>92</v>
+      </c>
+      <c r="B8" s="8">
+        <v>62.8</v>
+      </c>
+      <c r="C8" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B9" s="8">
+        <v>706.1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="3" spans="1:8">
-      <c r="A3" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" s="3" t="s">
+      <c r="B13" s="8">
+        <v>157</v>
+      </c>
+      <c r="C13" t="s">
         <v>98</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="G4" s="3" t="s">
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" t="s">
-        <v>37</v>
-      </c>
-      <c r="B5">
-        <v>60</v>
-      </c>
-      <c r="C5">
-        <v>151</v>
-      </c>
-      <c r="D5">
-        <v>153</v>
-      </c>
-      <c r="E5">
-        <v>81</v>
-      </c>
-      <c r="F5">
-        <v>12</v>
-      </c>
-      <c r="G5">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="A6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B6">
-        <v>55</v>
-      </c>
-      <c r="C6">
-        <v>105</v>
-      </c>
-      <c r="D6">
-        <v>113</v>
-      </c>
-      <c r="E6">
-        <v>53</v>
-      </c>
-      <c r="F6">
-        <v>2</v>
-      </c>
-      <c r="G6">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
-      <c r="A7" t="s">
-        <v>39</v>
-      </c>
-      <c r="B7">
-        <v>35</v>
-      </c>
-      <c r="C7">
-        <v>72</v>
-      </c>
-      <c r="D7">
-        <v>67</v>
-      </c>
-      <c r="E7">
-        <v>41</v>
-      </c>
-      <c r="F7">
-        <v>3</v>
-      </c>
-      <c r="G7">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" t="s">
-        <v>40</v>
-      </c>
-      <c r="B8">
-        <v>13</v>
-      </c>
-      <c r="C8">
-        <v>36</v>
-      </c>
-      <c r="D8">
-        <v>35</v>
-      </c>
-      <c r="E8">
-        <v>19</v>
-      </c>
-      <c r="F8">
-        <v>0</v>
-      </c>
-      <c r="G8">
+      <c r="B14" s="8">
+        <v>94.2</v>
+      </c>
+      <c r="C14" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" t="s">
+        <v>100</v>
+      </c>
+      <c r="B15" s="8">
+        <v>65.59999999999999</v>
+      </c>
+      <c r="C15" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" t="s">
+        <v>101</v>
+      </c>
+      <c r="B16" s="8">
+        <v>65.5</v>
+      </c>
+      <c r="C16" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="B17" s="8">
+        <v>382.3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" s="5" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="9" spans="1:8">
-      <c r="A9" t="s">
-        <v>41</v>
-      </c>
-      <c r="B9">
-        <v>9</v>
-      </c>
-      <c r="C9">
-        <v>27</v>
-      </c>
-      <c r="D9">
-        <v>28</v>
-      </c>
-      <c r="E9">
-        <v>15</v>
-      </c>
-      <c r="F9">
-        <v>0</v>
-      </c>
-      <c r="G9">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="A11" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8">
-      <c r="A12" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8">
-      <c r="A13" t="s">
-        <v>37</v>
-      </c>
-      <c r="B13">
-        <v>73</v>
-      </c>
-      <c r="C13">
-        <v>116</v>
-      </c>
-      <c r="D13">
-        <v>138</v>
-      </c>
-      <c r="E13">
-        <v>70</v>
-      </c>
-      <c r="F13">
-        <v>69</v>
-      </c>
-      <c r="G13">
-        <v>0</v>
-      </c>
-      <c r="H13">
-        <v>466</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8">
-      <c r="A14" t="s">
-        <v>38</v>
-      </c>
-      <c r="B14">
-        <v>37</v>
-      </c>
-      <c r="C14">
-        <v>78</v>
-      </c>
-      <c r="D14">
-        <v>90</v>
-      </c>
-      <c r="E14">
-        <v>56</v>
-      </c>
-      <c r="F14">
-        <v>47</v>
-      </c>
-      <c r="G14">
-        <v>0</v>
-      </c>
-      <c r="H14">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8">
-      <c r="A15" t="s">
-        <v>39</v>
-      </c>
-      <c r="B15">
-        <v>24</v>
-      </c>
-      <c r="C15">
-        <v>56</v>
-      </c>
-      <c r="D15">
-        <v>68</v>
-      </c>
-      <c r="E15">
-        <v>41</v>
-      </c>
-      <c r="F15">
-        <v>28</v>
-      </c>
-      <c r="G15">
-        <v>0</v>
-      </c>
-      <c r="H15">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8">
-      <c r="A16" t="s">
-        <v>40</v>
-      </c>
-      <c r="B16">
-        <v>7</v>
-      </c>
-      <c r="C16">
-        <v>17</v>
-      </c>
-      <c r="D16">
-        <v>30</v>
-      </c>
-      <c r="E16">
-        <v>15</v>
-      </c>
-      <c r="F16">
-        <v>17</v>
-      </c>
-      <c r="G16">
-        <v>1</v>
-      </c>
-      <c r="H16">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8">
-      <c r="A17" t="s">
-        <v>41</v>
-      </c>
-      <c r="B17">
-        <v>7</v>
-      </c>
-      <c r="C17">
-        <v>15</v>
-      </c>
-      <c r="D17">
-        <v>17</v>
-      </c>
-      <c r="E17">
-        <v>12</v>
-      </c>
-      <c r="F17">
-        <v>9</v>
-      </c>
-      <c r="G17">
-        <v>0</v>
-      </c>
-      <c r="H17">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8">
-      <c r="A19" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8">
-      <c r="A20" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="H20" s="3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8">
-      <c r="A21" t="s">
-        <v>37</v>
-      </c>
-      <c r="B21">
-        <v>30</v>
-      </c>
-      <c r="C21">
-        <v>28</v>
-      </c>
-      <c r="D21">
-        <v>23</v>
-      </c>
-      <c r="E21">
-        <v>40</v>
-      </c>
-      <c r="F21">
-        <v>50</v>
-      </c>
-      <c r="G21">
-        <v>43</v>
-      </c>
-      <c r="H21">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8">
-      <c r="A22" t="s">
-        <v>38</v>
-      </c>
-      <c r="B22">
-        <v>15</v>
-      </c>
-      <c r="C22">
-        <v>18</v>
-      </c>
-      <c r="D22">
-        <v>12</v>
-      </c>
-      <c r="E22">
-        <v>40</v>
-      </c>
-      <c r="F22">
-        <v>31</v>
-      </c>
-      <c r="G22">
-        <v>30</v>
-      </c>
-      <c r="H22">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8">
-      <c r="A23" t="s">
-        <v>40</v>
-      </c>
-      <c r="B23">
-        <v>8</v>
-      </c>
-      <c r="C23">
-        <v>14</v>
-      </c>
-      <c r="D23">
-        <v>10</v>
-      </c>
-      <c r="E23">
-        <v>19</v>
-      </c>
-      <c r="F23">
-        <v>23</v>
-      </c>
-      <c r="G23">
-        <v>30</v>
-      </c>
-      <c r="H23">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8">
-      <c r="A24" t="s">
-        <v>41</v>
-      </c>
-      <c r="B24">
-        <v>5</v>
-      </c>
-      <c r="C24">
-        <v>8</v>
-      </c>
-      <c r="D24">
-        <v>11</v>
-      </c>
-      <c r="E24">
-        <v>14</v>
-      </c>
-      <c r="F24">
-        <v>14</v>
-      </c>
-      <c r="G24">
-        <v>19</v>
-      </c>
-      <c r="H24">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8">
-      <c r="A25" t="s">
-        <v>39</v>
-      </c>
-      <c r="B25">
-        <v>4</v>
-      </c>
-      <c r="C25">
-        <v>9</v>
-      </c>
-      <c r="D25">
-        <v>7</v>
-      </c>
-      <c r="E25">
-        <v>6</v>
-      </c>
-      <c r="F25">
-        <v>11</v>
-      </c>
-      <c r="G25">
-        <v>13</v>
-      </c>
-      <c r="H25">
-        <v>50</v>
+      <c r="B19" s="8">
+        <v>1088.4</v>
       </c>
     </row>
   </sheetData>
@@ -2685,6 +2309,486 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5">
+        <v>31</v>
+      </c>
+      <c r="C5">
+        <v>113</v>
+      </c>
+      <c r="D5">
+        <v>115</v>
+      </c>
+      <c r="E5">
+        <v>58</v>
+      </c>
+      <c r="F5">
+        <v>8</v>
+      </c>
+      <c r="G5">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6">
+        <v>43</v>
+      </c>
+      <c r="C6">
+        <v>87</v>
+      </c>
+      <c r="D6">
+        <v>89</v>
+      </c>
+      <c r="E6">
+        <v>55</v>
+      </c>
+      <c r="F6">
+        <v>8</v>
+      </c>
+      <c r="G6">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7">
+        <v>35</v>
+      </c>
+      <c r="C7">
+        <v>91</v>
+      </c>
+      <c r="D7">
+        <v>87</v>
+      </c>
+      <c r="E7">
+        <v>42</v>
+      </c>
+      <c r="F7">
+        <v>8</v>
+      </c>
+      <c r="G7">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8">
+        <v>25</v>
+      </c>
+      <c r="C8">
+        <v>69</v>
+      </c>
+      <c r="D8">
+        <v>63</v>
+      </c>
+      <c r="E8">
+        <v>36</v>
+      </c>
+      <c r="F8">
+        <v>8</v>
+      </c>
+      <c r="G8">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9">
+        <v>9</v>
+      </c>
+      <c r="C9">
+        <v>18</v>
+      </c>
+      <c r="D9">
+        <v>25</v>
+      </c>
+      <c r="E9">
+        <v>14</v>
+      </c>
+      <c r="F9">
+        <v>8</v>
+      </c>
+      <c r="G9">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13">
+        <v>49</v>
+      </c>
+      <c r="C13">
+        <v>83</v>
+      </c>
+      <c r="D13">
+        <v>98</v>
+      </c>
+      <c r="E13">
+        <v>53</v>
+      </c>
+      <c r="F13">
+        <v>56</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14">
+        <v>28</v>
+      </c>
+      <c r="C14">
+        <v>75</v>
+      </c>
+      <c r="D14">
+        <v>97</v>
+      </c>
+      <c r="E14">
+        <v>56</v>
+      </c>
+      <c r="F14">
+        <v>42</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" t="s">
+        <v>37</v>
+      </c>
+      <c r="B15">
+        <v>19</v>
+      </c>
+      <c r="C15">
+        <v>49</v>
+      </c>
+      <c r="D15">
+        <v>99</v>
+      </c>
+      <c r="E15">
+        <v>68</v>
+      </c>
+      <c r="F15">
+        <v>60</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" t="s">
+        <v>40</v>
+      </c>
+      <c r="B16">
+        <v>15</v>
+      </c>
+      <c r="C16">
+        <v>31</v>
+      </c>
+      <c r="D16">
+        <v>61</v>
+      </c>
+      <c r="E16">
+        <v>31</v>
+      </c>
+      <c r="F16">
+        <v>35</v>
+      </c>
+      <c r="G16">
+        <v>1</v>
+      </c>
+      <c r="H16">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="A17" t="s">
+        <v>41</v>
+      </c>
+      <c r="B17">
+        <v>7</v>
+      </c>
+      <c r="C17">
+        <v>16</v>
+      </c>
+      <c r="D17">
+        <v>20</v>
+      </c>
+      <c r="E17">
+        <v>14</v>
+      </c>
+      <c r="F17">
+        <v>11</v>
+      </c>
+      <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
+      <c r="A19" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
+      <c r="A21" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21">
+        <v>17</v>
+      </c>
+      <c r="C21">
+        <v>34</v>
+      </c>
+      <c r="D21">
+        <v>27</v>
+      </c>
+      <c r="E21">
+        <v>49</v>
+      </c>
+      <c r="F21">
+        <v>55</v>
+      </c>
+      <c r="G21">
+        <v>73</v>
+      </c>
+      <c r="H21">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22" t="s">
+        <v>39</v>
+      </c>
+      <c r="B22">
+        <v>25</v>
+      </c>
+      <c r="C22">
+        <v>25</v>
+      </c>
+      <c r="D22">
+        <v>17</v>
+      </c>
+      <c r="E22">
+        <v>31</v>
+      </c>
+      <c r="F22">
+        <v>39</v>
+      </c>
+      <c r="G22">
+        <v>33</v>
+      </c>
+      <c r="H22">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" t="s">
+        <v>41</v>
+      </c>
+      <c r="B23">
+        <v>6</v>
+      </c>
+      <c r="C23">
+        <v>10</v>
+      </c>
+      <c r="D23">
+        <v>12</v>
+      </c>
+      <c r="E23">
+        <v>18</v>
+      </c>
+      <c r="F23">
+        <v>19</v>
+      </c>
+      <c r="G23">
+        <v>24</v>
+      </c>
+      <c r="H23">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
+      <c r="A24" t="s">
+        <v>38</v>
+      </c>
+      <c r="B24">
+        <v>2</v>
+      </c>
+      <c r="C24">
+        <v>13</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
+        <v>4</v>
+      </c>
+      <c r="F24">
+        <v>13</v>
+      </c>
+      <c r="G24">
+        <v>12</v>
+      </c>
+      <c r="H24">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
+      <c r="A25" t="s">
+        <v>37</v>
+      </c>
+      <c r="B25">
+        <v>0</v>
+      </c>
+      <c r="C25">
+        <v>7</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25">
+        <v>7</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+      <c r="G25">
+        <v>14</v>
+      </c>
+      <c r="H25">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A9"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2694,42 +2798,42 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Explore Pants: KIDS Gris/Azul curva completa, rangos MÍN/MÁX y ranking tela
Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/EXPLORE_PANTS_Proyeccion_Produccion.xlsx
+++ b/EXPLORE_PANTS_Proyeccion_Produccion.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="139">
   <si>
     <t>EXPLORE PANTS — PROYECCIÓN ANCLADA A JUSTIFICACIÓN NOVAKTEX</t>
   </si>
@@ -127,10 +127,16 @@
     <t>EXPLORE PANTS — COLOR POR GÉNERO (PRODUCCIÓN vs VENTAS)</t>
   </si>
   <si>
+    <t># ventas</t>
+  </si>
+  <si>
     <t>Color</t>
   </si>
   <si>
-    <t>Und producir</t>
+    <t>Und Mín</t>
+  </si>
+  <si>
+    <t>Und Máx</t>
   </si>
   <si>
     <t>% prod.</t>
@@ -181,201 +187,231 @@
     <t>Rango</t>
   </si>
   <si>
-    <t>CABALLERO — COLOR × TALLA (MÍN)</t>
+    <t>CABALLERO — RANGO MÍN / MÁX POR COLOR</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>M</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>XL</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Negro — MÍN</t>
+  </si>
+  <si>
+    <t>Negro — MÁX</t>
+  </si>
+  <si>
+    <t>Kaki — MÍN</t>
+  </si>
+  <si>
+    <t>Kaki — MÁX</t>
+  </si>
+  <si>
+    <t>Azul Marino — MÍN</t>
+  </si>
+  <si>
+    <t>Azul Marino — MÁX</t>
+  </si>
+  <si>
+    <t>Verde Militar — MÍN</t>
+  </si>
+  <si>
+    <t>Verde Militar — MÁX</t>
+  </si>
+  <si>
+    <t>Gris Oscuro — MÍN</t>
+  </si>
+  <si>
+    <t>Gris Oscuro — MÁX</t>
+  </si>
+  <si>
+    <t>TOTAL — MÍN</t>
+  </si>
+  <si>
+    <t>TOTAL — MÁX</t>
+  </si>
+  <si>
+    <t>DAMA — RANGO MÍN / MÁX POR COLOR</t>
+  </si>
+  <si>
+    <t>XS</t>
+  </si>
+  <si>
+    <t>KIDS — RANGO MÍN / MÁX POR COLOR</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>EXPLORE PANTS — CURVA DE TALLA POR GÉNERO (vs dashboard)</t>
+  </si>
+  <si>
+    <t>CABALLERO — TALLAS</t>
+  </si>
+  <si>
+    <t>Talla</t>
+  </si>
+  <si>
+    <t>Mínimo</t>
+  </si>
+  <si>
+    <t>Máximo</t>
+  </si>
+  <si>
+    <t>DAMA — TALLAS</t>
+  </si>
+  <si>
+    <t>KIDS — TALLAS</t>
+  </si>
+  <si>
+    <t>EXPLORE PANTS — VERIFICACIÓN TELA NOVAKTEX REPEL COMPRADA</t>
+  </si>
+  <si>
+    <t>Explore + Shorts R1 vs kg en existencias (objetivo: delta ≈ 0).</t>
+  </si>
+  <si>
+    <t>Und Explore</t>
+  </si>
+  <si>
+    <t>Kg Explore</t>
+  </si>
+  <si>
+    <t>Kg Shorts</t>
+  </si>
+  <si>
+    <t>Kg total</t>
+  </si>
+  <si>
+    <t>Kg existencia</t>
+  </si>
+  <si>
+    <t>Delta</t>
+  </si>
+  <si>
+    <t>Shorts R1 total: 1,697 und · 220.4 kg</t>
+  </si>
+  <si>
+    <t>Consumo referencial por género (kg/und)</t>
+  </si>
+  <si>
+    <t>Consumo ref.</t>
+  </si>
+  <si>
+    <t>SHORT SPORT R1 — NEGRO / GRIS OSCURO (CAB · DAMA)</t>
+  </si>
+  <si>
+    <t>Color tela</t>
+  </si>
+  <si>
+    <t>Total und</t>
+  </si>
+  <si>
+    <t>CAB</t>
+  </si>
+  <si>
+    <t>Kg tela</t>
+  </si>
+  <si>
+    <t>PROPUESTA COMPRA 65% AHORA / 35% SEPTIEMBRE (archivo justificación)</t>
+  </si>
+  <si>
+    <t>ORDEN 1 — INMEDIATA (65%)</t>
+  </si>
+  <si>
+    <t>Ítem</t>
+  </si>
+  <si>
+    <t>Kg</t>
+  </si>
+  <si>
+    <t>Prioridad</t>
+  </si>
+  <si>
+    <t>Gris Oscuro — TODO (Explore + Shorts)</t>
+  </si>
+  <si>
+    <t>CRÍTICA</t>
+  </si>
+  <si>
+    <t>Tela de Shorts — Negro y Azul (completa)</t>
+  </si>
+  <si>
+    <t>Negro Explore — mitad</t>
+  </si>
+  <si>
+    <t>ALTA</t>
+  </si>
+  <si>
+    <t>Kaki Explore — parte</t>
+  </si>
+  <si>
+    <t>MEDIA</t>
+  </si>
+  <si>
+    <t>SUBTOTAL ORDEN 1</t>
+  </si>
+  <si>
+    <t>ORDEN 2 — COMIENZOS SEPTIEMBRE (35%)</t>
+  </si>
+  <si>
+    <t>Riesgo</t>
+  </si>
+  <si>
+    <t>Negro Explore — la otra mitad</t>
+  </si>
+  <si>
+    <t>BAJO</t>
+  </si>
+  <si>
+    <t>Kaki Explore — resto</t>
+  </si>
+  <si>
+    <t>Verde Militar — TODO</t>
+  </si>
+  <si>
+    <t>Azul Marino Explore — TODO</t>
+  </si>
+  <si>
+    <t>SUBTOTAL ORDEN 2</t>
+  </si>
+  <si>
+    <t>TELA TOTAL (Explore + Shorts)</t>
+  </si>
+  <si>
+    <t>EXPLORE PANTS — MATRIZ COLOR × TALLA</t>
   </si>
   <si>
     <t>Color / Talla</t>
   </si>
   <si>
-    <t>S</t>
-  </si>
-  <si>
-    <t>M</t>
-  </si>
-  <si>
-    <t>L</t>
-  </si>
-  <si>
-    <t>XL</t>
-  </si>
-  <si>
-    <t>Total Mín</t>
-  </si>
-  <si>
-    <t>Total Máx</t>
-  </si>
-  <si>
-    <t>DAMA — COLOR × TALLA (MÍN)</t>
-  </si>
-  <si>
-    <t>XS</t>
-  </si>
-  <si>
-    <t>KIDS — COLOR × TALLA (MÍN)</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>EXPLORE PANTS — CURVA DE TALLA POR GÉNERO (vs dashboard)</t>
-  </si>
-  <si>
-    <t>CABALLERO — TALLAS</t>
-  </si>
-  <si>
-    <t>Talla</t>
-  </si>
-  <si>
-    <t>Mínimo</t>
-  </si>
-  <si>
-    <t>Máximo</t>
-  </si>
-  <si>
-    <t>DAMA — TALLAS</t>
-  </si>
-  <si>
-    <t>KIDS — TALLAS</t>
-  </si>
-  <si>
-    <t>EXPLORE PANTS — VERIFICACIÓN TELA NOVAKTEX REPEL COMPRADA</t>
-  </si>
-  <si>
-    <t>Explore + Shorts R1 vs kg en existencias (objetivo: delta ≈ 0).</t>
-  </si>
-  <si>
-    <t>Und Explore</t>
-  </si>
-  <si>
-    <t>Kg Explore</t>
-  </si>
-  <si>
-    <t>Kg Shorts</t>
-  </si>
-  <si>
-    <t>Kg total</t>
-  </si>
-  <si>
-    <t>Kg existencia</t>
-  </si>
-  <si>
-    <t>Delta</t>
-  </si>
-  <si>
-    <t>Shorts R1 total: 1,689 und · 219.36 kg</t>
-  </si>
-  <si>
-    <t>Consumo referencial por género (kg/und)</t>
-  </si>
-  <si>
-    <t>Consumo ref.</t>
-  </si>
-  <si>
-    <t>SHORT SPORT R1 — NEGRO / GRIS OSCURO (CAB · DAMA)</t>
-  </si>
-  <si>
-    <t>Color tela</t>
-  </si>
-  <si>
-    <t>Total und</t>
-  </si>
-  <si>
-    <t>CAB</t>
-  </si>
-  <si>
-    <t>Kg tela</t>
-  </si>
-  <si>
-    <t>PROPUESTA COMPRA 65% AHORA / 35% SEPTIEMBRE (archivo justificación)</t>
-  </si>
-  <si>
-    <t>ORDEN 1 — INMEDIATA (65%)</t>
-  </si>
-  <si>
-    <t>Ítem</t>
-  </si>
-  <si>
-    <t>Kg</t>
-  </si>
-  <si>
-    <t>Prioridad</t>
-  </si>
-  <si>
-    <t>Gris Oscuro — TODO (Explore + Shorts)</t>
-  </si>
-  <si>
-    <t>CRÍTICA</t>
-  </si>
-  <si>
-    <t>Tela de Shorts — Negro y Azul (completa)</t>
-  </si>
-  <si>
-    <t>Negro Explore — mitad</t>
-  </si>
-  <si>
-    <t>ALTA</t>
-  </si>
-  <si>
-    <t>Kaki Explore — parte</t>
-  </si>
-  <si>
-    <t>MEDIA</t>
-  </si>
-  <si>
-    <t>SUBTOTAL ORDEN 1</t>
-  </si>
-  <si>
-    <t>ORDEN 2 — COMIENZOS SEPTIEMBRE (35%)</t>
-  </si>
-  <si>
-    <t>Riesgo</t>
-  </si>
-  <si>
-    <t>Negro Explore — la otra mitad</t>
-  </si>
-  <si>
-    <t>BAJO</t>
-  </si>
-  <si>
-    <t>Kaki Explore — resto</t>
-  </si>
-  <si>
-    <t>Verde Militar — TODO</t>
-  </si>
-  <si>
-    <t>Azul Marino Explore — TODO</t>
-  </si>
-  <si>
-    <t>SUBTOTAL ORDEN 2</t>
-  </si>
-  <si>
-    <t>TELA TOTAL (Explore + Shorts)</t>
-  </si>
-  <si>
-    <t>EXPLORE PANTS — MATRIZ COLOR × TALLA</t>
-  </si>
-  <si>
-    <t>Total</t>
-  </si>
-  <si>
     <t>METODOLOGÍA — EXPLORE PANTS</t>
   </si>
   <si>
@@ -388,10 +424,10 @@
     <t>3. Rango MÍN/MÁX Explore: factor temporada alta ×1.2.</t>
   </si>
   <si>
-    <t>4. COLOR: ranking ventas por género (ajustado a tela). TALLA: curva dashboard.</t>
-  </si>
-  <si>
-    <t>5. KIDS Gris/Azul: al menos 1 und por talla 2–14. CAB sin 3XL · DAMA sin 2XL.</t>
+    <t>4. COLOR: ranking ventas por género; si CAB Negro queda bajo vs Gris es por kg Negro/Gris en Shorts R1 + consumo de existencia Gris (no por mezcla de compra).</t>
+  </si>
+  <si>
+    <t>5. KIDS Gris/Azul: presencia 2–14 con curva talla dashboard; Gris piso ~48 und. CAB sin 3XL · DAMA sin 2XL.</t>
   </si>
   <si>
     <t>6. Shorts R1: CAB 0.14 · DAMA 0.12 kg/und.</t>
@@ -989,10 +1025,10 @@
         <v>29</v>
       </c>
       <c r="B31">
-        <v>1145</v>
+        <v>1143</v>
       </c>
       <c r="C31">
-        <v>1381</v>
+        <v>1379</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -1000,10 +1036,10 @@
         <v>30</v>
       </c>
       <c r="B32">
-        <v>1174</v>
+        <v>1172</v>
       </c>
       <c r="C32">
-        <v>1420</v>
+        <v>1418</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -1011,10 +1047,10 @@
         <v>31</v>
       </c>
       <c r="B33">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="C33">
-        <v>715</v>
+        <v>714</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -1022,10 +1058,10 @@
         <v>32</v>
       </c>
       <c r="B34" s="5">
-        <v>2905</v>
+        <v>2900</v>
       </c>
       <c r="C34" s="5">
-        <v>3516</v>
+        <v>3511</v>
       </c>
     </row>
   </sheetData>
@@ -1046,52 +1082,52 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>118</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" t="s">
-        <v>123</v>
+        <v>135</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" t="s">
-        <v>124</v>
+        <v>136</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -1101,20 +1137,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:6">
       <c r="A3" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:6">
       <c r="A4" s="3" t="s">
         <v>34</v>
       </c>
@@ -1127,94 +1163,130 @@
       <c r="D4" s="3" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" t="s">
+      <c r="E4" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="4">
-        <v>263</v>
-      </c>
-      <c r="C5" s="6">
-        <v>0.2296943231441048</v>
-      </c>
-      <c r="D5" s="6">
+      <c r="F4" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5" s="4">
+        <v>262</v>
+      </c>
+      <c r="D5" s="4">
+        <v>316</v>
+      </c>
+      <c r="E5" s="6">
+        <v>0.2292213473315836</v>
+      </c>
+      <c r="F5" s="6">
         <v>0.252</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
-      <c r="A6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B6" s="4">
+    <row r="6" spans="1:6">
+      <c r="A6">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" s="4">
         <v>282</v>
       </c>
-      <c r="C6" s="6">
-        <v>0.2462882096069869</v>
-      </c>
-      <c r="D6" s="6">
+      <c r="D6" s="4">
+        <v>339</v>
+      </c>
+      <c r="E6" s="6">
+        <v>0.2467191601049869</v>
+      </c>
+      <c r="F6" s="6">
         <v>0.211</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
-      <c r="A7" t="s">
-        <v>40</v>
-      </c>
-      <c r="B7" s="4">
+    <row r="7" spans="1:6">
+      <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" s="4">
         <v>201</v>
       </c>
-      <c r="C7" s="6">
-        <v>0.1755458515283843</v>
-      </c>
-      <c r="D7" s="6">
+      <c r="D7" s="4">
+        <v>243</v>
+      </c>
+      <c r="E7" s="6">
+        <v>0.1758530183727034</v>
+      </c>
+      <c r="F7" s="6">
         <v>0.17</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
-      <c r="A8" t="s">
-        <v>41</v>
-      </c>
-      <c r="B8" s="4">
+    <row r="8" spans="1:6">
+      <c r="A8">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" s="4">
         <v>74</v>
       </c>
-      <c r="C8" s="6">
-        <v>0.06462882096069869</v>
-      </c>
-      <c r="D8" s="6">
+      <c r="D8" s="4">
+        <v>90</v>
+      </c>
+      <c r="E8" s="6">
+        <v>0.0647419072615923</v>
+      </c>
+      <c r="F8" s="6">
         <v>0.164</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
-      <c r="A9" t="s">
-        <v>42</v>
-      </c>
-      <c r="B9" s="4">
-        <v>325</v>
-      </c>
-      <c r="C9" s="6">
-        <v>0.2838427947598253</v>
-      </c>
-      <c r="D9" s="6">
+    <row r="9" spans="1:6">
+      <c r="A9">
+        <v>5</v>
+      </c>
+      <c r="B9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" s="4">
+        <v>324</v>
+      </c>
+      <c r="D9" s="4">
+        <v>391</v>
+      </c>
+      <c r="E9" s="6">
+        <v>0.2834645669291339</v>
+      </c>
+      <c r="F9" s="6">
         <v>0.06900000000000001</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:6">
       <c r="A10" s="5" t="s">
         <v>32</v>
       </c>
       <c r="B10" s="4">
-        <v>1145</v>
+        <v>1143</v>
       </c>
       <c r="C10" s="7">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:6">
       <c r="A12" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:6">
       <c r="A13" s="3" t="s">
         <v>34</v>
       </c>
@@ -1227,94 +1299,130 @@
       <c r="D13" s="3" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" t="s">
+      <c r="E13" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B14" s="4">
-        <v>339</v>
-      </c>
-      <c r="C14" s="6">
-        <v>0.2887563884156729</v>
-      </c>
-      <c r="D14" s="6">
+      <c r="F13" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14">
+        <v>1</v>
+      </c>
+      <c r="B14" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="4">
+        <v>346</v>
+      </c>
+      <c r="D14" s="4">
+        <v>416</v>
+      </c>
+      <c r="E14" s="6">
+        <v>0.295221843003413</v>
+      </c>
+      <c r="F14" s="6">
         <v>0.306</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
-      <c r="A15" t="s">
-        <v>39</v>
-      </c>
-      <c r="B15" s="4">
-        <v>298</v>
-      </c>
-      <c r="C15" s="6">
-        <v>0.2538330494037478</v>
-      </c>
-      <c r="D15" s="6">
+    <row r="15" spans="1:6">
+      <c r="A15">
+        <v>2</v>
+      </c>
+      <c r="B15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="4">
+        <v>303</v>
+      </c>
+      <c r="D15" s="4">
+        <v>366</v>
+      </c>
+      <c r="E15" s="6">
+        <v>0.2585324232081911</v>
+      </c>
+      <c r="F15" s="6">
         <v>0.209</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
-      <c r="A16" t="s">
-        <v>41</v>
-      </c>
-      <c r="B16" s="4">
-        <v>68</v>
-      </c>
-      <c r="C16" s="6">
-        <v>0.05792163543441227</v>
-      </c>
-      <c r="D16" s="6">
+    <row r="16" spans="1:6">
+      <c r="A16">
+        <v>3</v>
+      </c>
+      <c r="B16" t="s">
+        <v>43</v>
+      </c>
+      <c r="C16" s="4">
+        <v>72</v>
+      </c>
+      <c r="D16" s="4">
+        <v>89</v>
+      </c>
+      <c r="E16" s="6">
+        <v>0.06143344709897611</v>
+      </c>
+      <c r="F16" s="6">
         <v>0.142</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
-      <c r="A17" t="s">
-        <v>40</v>
-      </c>
-      <c r="B17" s="4">
-        <v>174</v>
-      </c>
-      <c r="C17" s="6">
-        <v>0.1482112436115843</v>
-      </c>
-      <c r="D17" s="6">
+    <row r="17" spans="1:6">
+      <c r="A17">
+        <v>4</v>
+      </c>
+      <c r="B17" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" s="4">
+        <v>176</v>
+      </c>
+      <c r="D17" s="4">
+        <v>214</v>
+      </c>
+      <c r="E17" s="6">
+        <v>0.1501706484641638</v>
+      </c>
+      <c r="F17" s="6">
         <v>0.139</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
-      <c r="A18" t="s">
-        <v>42</v>
-      </c>
-      <c r="B18" s="4">
-        <v>295</v>
-      </c>
-      <c r="C18" s="6">
-        <v>0.2512776831345826</v>
-      </c>
-      <c r="D18" s="6">
+    <row r="18" spans="1:6">
+      <c r="A18">
+        <v>5</v>
+      </c>
+      <c r="B18" t="s">
+        <v>44</v>
+      </c>
+      <c r="C18" s="4">
+        <v>275</v>
+      </c>
+      <c r="D18" s="4">
+        <v>333</v>
+      </c>
+      <c r="E18" s="6">
+        <v>0.234641638225256</v>
+      </c>
+      <c r="F18" s="6">
         <v>0.058</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
+    <row r="19" spans="1:6">
       <c r="A19" s="5" t="s">
         <v>32</v>
       </c>
       <c r="B19" s="4">
-        <v>1174</v>
+        <v>1172</v>
       </c>
       <c r="C19" s="7">
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
+    <row r="21" spans="1:6">
       <c r="A21" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
+    <row r="22" spans="1:6">
       <c r="A22" s="3" t="s">
         <v>34</v>
       </c>
@@ -1327,83 +1435,119 @@
       <c r="D22" s="3" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="23" spans="1:4">
-      <c r="A23" t="s">
+      <c r="E22" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23">
+        <v>1</v>
+      </c>
+      <c r="B23" t="s">
+        <v>42</v>
+      </c>
+      <c r="C23" s="4">
+        <v>252</v>
+      </c>
+      <c r="D23" s="4">
+        <v>306</v>
+      </c>
+      <c r="E23" s="6">
+        <v>0.4307692307692308</v>
+      </c>
+      <c r="F23" s="6">
+        <v>0.298</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24">
+        <v>2</v>
+      </c>
+      <c r="B24" t="s">
+        <v>43</v>
+      </c>
+      <c r="C24" s="4">
+        <v>84</v>
+      </c>
+      <c r="D24" s="4">
+        <v>104</v>
+      </c>
+      <c r="E24" s="6">
+        <v>0.1435897435897436</v>
+      </c>
+      <c r="F24" s="6">
+        <v>0.269</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25">
+        <v>3</v>
+      </c>
+      <c r="B25" t="s">
         <v>40</v>
       </c>
-      <c r="B23" s="4">
-        <v>255</v>
-      </c>
-      <c r="C23" s="6">
-        <v>0.4351535836177474</v>
-      </c>
-      <c r="D23" s="6">
-        <v>0.298</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4">
-      <c r="A24" t="s">
+      <c r="C25" s="4">
+        <v>161</v>
+      </c>
+      <c r="D25" s="4">
+        <v>195</v>
+      </c>
+      <c r="E25" s="6">
+        <v>0.2752136752136752</v>
+      </c>
+      <c r="F25" s="6">
+        <v>0.225</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26">
+        <v>4</v>
+      </c>
+      <c r="B26" t="s">
         <v>41</v>
       </c>
-      <c r="B24" s="4">
-        <v>89</v>
-      </c>
-      <c r="C24" s="6">
-        <v>0.1518771331058021</v>
-      </c>
-      <c r="D24" s="6">
-        <v>0.269</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4">
-      <c r="A25" t="s">
+      <c r="C26" s="4">
         <v>38</v>
       </c>
-      <c r="B25" s="4">
-        <v>170</v>
-      </c>
-      <c r="C25" s="6">
-        <v>0.2901023890784983</v>
-      </c>
-      <c r="D25" s="6">
-        <v>0.225</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4">
-      <c r="A26" t="s">
-        <v>39</v>
-      </c>
-      <c r="B26" s="4">
+      <c r="D26" s="4">
+        <v>47</v>
+      </c>
+      <c r="E26" s="6">
+        <v>0.06495726495726496</v>
+      </c>
+      <c r="F26" s="6">
+        <v>0.045</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27">
+        <v>5</v>
+      </c>
+      <c r="B27" t="s">
         <v>44</v>
       </c>
-      <c r="C26" s="6">
-        <v>0.07508532423208192</v>
-      </c>
-      <c r="D26" s="6">
-        <v>0.045</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4">
-      <c r="A27" t="s">
-        <v>42</v>
-      </c>
-      <c r="B27" s="4">
-        <v>28</v>
-      </c>
-      <c r="C27" s="6">
-        <v>0.04778156996587031</v>
-      </c>
-      <c r="D27" s="6">
+      <c r="C27" s="4">
+        <v>50</v>
+      </c>
+      <c r="D27" s="4">
+        <v>62</v>
+      </c>
+      <c r="E27" s="6">
+        <v>0.08547008547008547</v>
+      </c>
+      <c r="F27" s="6">
         <v>0.008</v>
       </c>
     </row>
-    <row r="28" spans="1:4">
+    <row r="28" spans="1:6">
       <c r="A28" s="5" t="s">
         <v>32</v>
       </c>
       <c r="B28" s="4">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="C28" s="7">
         <v>1</v>
@@ -1421,35 +1565,35 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B4" s="4">
-        <v>772</v>
+        <v>769</v>
       </c>
       <c r="C4" s="6">
-        <v>0.2657487091222031</v>
+        <v>0.2651724137931035</v>
       </c>
       <c r="D4" s="6">
         <v>0.3223210782341178</v>
@@ -1460,13 +1604,13 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B5" s="4">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="C5" s="6">
-        <v>0.2230636833046472</v>
+        <v>0.2237931034482759</v>
       </c>
       <c r="D5" s="6">
         <v>0.2844671001033621</v>
@@ -1477,13 +1621,13 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B6" s="4">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="C6" s="6">
-        <v>0.2148020654044751</v>
+        <v>0.2148275862068965</v>
       </c>
       <c r="D6" s="6">
         <v>0.1713177091328877</v>
@@ -1494,13 +1638,13 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B7" s="4">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="C7" s="6">
-        <v>0.2168674698795181</v>
+        <v>0.2168965517241379</v>
       </c>
       <c r="D7" s="6">
         <v>0.1622064538507951</v>
@@ -1511,13 +1655,13 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B8" s="4">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C8" s="6">
-        <v>0.07951807228915662</v>
+        <v>0.07931034482758621</v>
       </c>
       <c r="D8" s="6">
         <v>0.05968765867883735</v>
@@ -1531,7 +1675,7 @@
         <v>32</v>
       </c>
       <c r="B9" s="4">
-        <v>2905</v>
+        <v>2900</v>
       </c>
       <c r="C9" s="7">
         <v>1</v>
@@ -1550,115 +1694,112 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3" s="3" t="s">
         <v>26</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>29</v>
       </c>
       <c r="B4">
-        <v>1145</v>
+        <v>1143</v>
       </c>
       <c r="C4">
-        <v>1381</v>
+        <v>1379</v>
       </c>
       <c r="D4">
         <v>236</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>30</v>
       </c>
       <c r="B5">
-        <v>1174</v>
+        <v>1172</v>
       </c>
       <c r="C5">
-        <v>1420</v>
+        <v>1418</v>
       </c>
       <c r="D5">
         <v>246</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>31</v>
       </c>
       <c r="B6">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="C6">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="D6">
         <v>129</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:6">
       <c r="A7" s="5" t="s">
         <v>32</v>
       </c>
       <c r="B7" s="5">
-        <v>2905</v>
+        <v>2900</v>
       </c>
       <c r="C7" s="5">
-        <v>3516</v>
+        <v>3511</v>
       </c>
       <c r="D7" s="5">
         <v>611</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:6">
       <c r="A10" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
       <c r="A11" s="3" t="s">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="G11" s="3" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>38</v>
+        <v>60</v>
       </c>
       <c r="B12">
         <v>35</v>
@@ -1670,463 +1811,916 @@
         <v>95</v>
       </c>
       <c r="E12">
+        <v>41</v>
+      </c>
+      <c r="F12">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" t="s">
+        <v>61</v>
+      </c>
+      <c r="B13">
         <v>42</v>
       </c>
-      <c r="F12">
-        <v>263</v>
-      </c>
-      <c r="G12">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
-      <c r="A13" t="s">
+      <c r="C13">
+        <v>110</v>
+      </c>
+      <c r="D13">
+        <v>114</v>
+      </c>
+      <c r="E13">
+        <v>50</v>
+      </c>
+      <c r="F13">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" t="s">
+        <v>62</v>
+      </c>
+      <c r="B14">
+        <v>43</v>
+      </c>
+      <c r="C14">
+        <v>95</v>
+      </c>
+      <c r="D14">
+        <v>89</v>
+      </c>
+      <c r="E14">
+        <v>55</v>
+      </c>
+      <c r="F14">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" t="s">
+        <v>63</v>
+      </c>
+      <c r="B15">
+        <v>52</v>
+      </c>
+      <c r="C15">
+        <v>114</v>
+      </c>
+      <c r="D15">
+        <v>107</v>
+      </c>
+      <c r="E15">
+        <v>66</v>
+      </c>
+      <c r="F15">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" t="s">
+        <v>64</v>
+      </c>
+      <c r="B16">
+        <v>25</v>
+      </c>
+      <c r="C16">
+        <v>69</v>
+      </c>
+      <c r="D16">
+        <v>71</v>
+      </c>
+      <c r="E16">
+        <v>36</v>
+      </c>
+      <c r="F16">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
+        <v>65</v>
+      </c>
+      <c r="B17">
+        <v>30</v>
+      </c>
+      <c r="C17">
+        <v>83</v>
+      </c>
+      <c r="D17">
+        <v>86</v>
+      </c>
+      <c r="E17">
+        <v>44</v>
+      </c>
+      <c r="F17">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" t="s">
+        <v>66</v>
+      </c>
+      <c r="B18">
+        <v>9</v>
+      </c>
+      <c r="C18">
+        <v>26</v>
+      </c>
+      <c r="D18">
+        <v>25</v>
+      </c>
+      <c r="E18">
+        <v>14</v>
+      </c>
+      <c r="F18">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" t="s">
+        <v>67</v>
+      </c>
+      <c r="B19">
+        <v>11</v>
+      </c>
+      <c r="C19">
+        <v>32</v>
+      </c>
+      <c r="D19">
+        <v>30</v>
+      </c>
+      <c r="E19">
+        <v>17</v>
+      </c>
+      <c r="F19">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" t="s">
+        <v>68</v>
+      </c>
+      <c r="B20">
+        <v>31</v>
+      </c>
+      <c r="C20">
+        <v>112</v>
+      </c>
+      <c r="D20">
+        <v>123</v>
+      </c>
+      <c r="E20">
+        <v>58</v>
+      </c>
+      <c r="F20">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" t="s">
+        <v>69</v>
+      </c>
+      <c r="B21">
+        <v>38</v>
+      </c>
+      <c r="C21">
+        <v>135</v>
+      </c>
+      <c r="D21">
+        <v>148</v>
+      </c>
+      <c r="E21">
+        <v>70</v>
+      </c>
+      <c r="F21">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B22" s="5">
+        <v>143</v>
+      </c>
+      <c r="C22" s="5">
+        <v>393</v>
+      </c>
+      <c r="D22" s="5">
+        <v>403</v>
+      </c>
+      <c r="E22" s="5">
+        <v>204</v>
+      </c>
+      <c r="F22" s="5">
+        <v>1143</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B23" s="5">
+        <v>173</v>
+      </c>
+      <c r="C23" s="5">
+        <v>474</v>
+      </c>
+      <c r="D23" s="5">
+        <v>485</v>
+      </c>
+      <c r="E23" s="5">
+        <v>247</v>
+      </c>
+      <c r="F23" s="5">
+        <v>1379</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" t="s">
+        <v>60</v>
+      </c>
+      <c r="B27">
+        <v>50</v>
+      </c>
+      <c r="C27">
+        <v>84</v>
+      </c>
+      <c r="D27">
+        <v>100</v>
+      </c>
+      <c r="E27">
+        <v>54</v>
+      </c>
+      <c r="F27">
+        <v>58</v>
+      </c>
+      <c r="G27">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" t="s">
+        <v>61</v>
+      </c>
+      <c r="B28">
+        <v>60</v>
+      </c>
+      <c r="C28">
+        <v>101</v>
+      </c>
+      <c r="D28">
+        <v>120</v>
+      </c>
+      <c r="E28">
+        <v>65</v>
+      </c>
+      <c r="F28">
+        <v>70</v>
+      </c>
+      <c r="G28">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" t="s">
+        <v>62</v>
+      </c>
+      <c r="B29">
+        <v>29</v>
+      </c>
+      <c r="C29">
+        <v>76</v>
+      </c>
+      <c r="D29">
+        <v>99</v>
+      </c>
+      <c r="E29">
+        <v>57</v>
+      </c>
+      <c r="F29">
+        <v>42</v>
+      </c>
+      <c r="G29">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30" t="s">
+        <v>63</v>
+      </c>
+      <c r="B30">
+        <v>35</v>
+      </c>
+      <c r="C30">
+        <v>92</v>
+      </c>
+      <c r="D30">
+        <v>119</v>
+      </c>
+      <c r="E30">
+        <v>69</v>
+      </c>
+      <c r="F30">
+        <v>51</v>
+      </c>
+      <c r="G30">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31" t="s">
+        <v>66</v>
+      </c>
+      <c r="B31">
+        <v>7</v>
+      </c>
+      <c r="C31">
+        <v>17</v>
+      </c>
+      <c r="D31">
+        <v>21</v>
+      </c>
+      <c r="E31">
+        <v>15</v>
+      </c>
+      <c r="F31">
+        <v>12</v>
+      </c>
+      <c r="G31">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32" t="s">
+        <v>67</v>
+      </c>
+      <c r="B32">
+        <v>9</v>
+      </c>
+      <c r="C32">
+        <v>21</v>
+      </c>
+      <c r="D32">
+        <v>26</v>
+      </c>
+      <c r="E32">
+        <v>18</v>
+      </c>
+      <c r="F32">
+        <v>15</v>
+      </c>
+      <c r="G32">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9">
+      <c r="A33" t="s">
+        <v>64</v>
+      </c>
+      <c r="B33">
+        <v>15</v>
+      </c>
+      <c r="C33">
+        <v>32</v>
+      </c>
+      <c r="D33">
+        <v>62</v>
+      </c>
+      <c r="E33">
+        <v>31</v>
+      </c>
+      <c r="F33">
+        <v>36</v>
+      </c>
+      <c r="G33">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9">
+      <c r="A34" t="s">
+        <v>65</v>
+      </c>
+      <c r="B34">
+        <v>18</v>
+      </c>
+      <c r="C34">
         <v>39</v>
       </c>
-      <c r="B13">
-        <v>43</v>
-      </c>
-      <c r="C13">
-        <v>95</v>
-      </c>
-      <c r="D13">
-        <v>89</v>
-      </c>
-      <c r="E13">
-        <v>55</v>
-      </c>
-      <c r="F13">
-        <v>282</v>
-      </c>
-      <c r="G13">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
-      <c r="A14" t="s">
+      <c r="D34">
+        <v>75</v>
+      </c>
+      <c r="E34">
+        <v>38</v>
+      </c>
+      <c r="F34">
+        <v>44</v>
+      </c>
+      <c r="G34">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9">
+      <c r="A35" t="s">
+        <v>68</v>
+      </c>
+      <c r="B35">
+        <v>18</v>
+      </c>
+      <c r="C35">
+        <v>46</v>
+      </c>
+      <c r="D35">
+        <v>92</v>
+      </c>
+      <c r="E35">
+        <v>63</v>
+      </c>
+      <c r="F35">
+        <v>56</v>
+      </c>
+      <c r="G35">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9">
+      <c r="A36" t="s">
+        <v>69</v>
+      </c>
+      <c r="B36">
+        <v>22</v>
+      </c>
+      <c r="C36">
+        <v>56</v>
+      </c>
+      <c r="D36">
+        <v>111</v>
+      </c>
+      <c r="E36">
+        <v>76</v>
+      </c>
+      <c r="F36">
+        <v>68</v>
+      </c>
+      <c r="G36">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9">
+      <c r="A37" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B37" s="5">
+        <v>119</v>
+      </c>
+      <c r="C37" s="5">
+        <v>255</v>
+      </c>
+      <c r="D37" s="5">
+        <v>374</v>
+      </c>
+      <c r="E37" s="5">
+        <v>220</v>
+      </c>
+      <c r="F37" s="5">
+        <v>204</v>
+      </c>
+      <c r="G37" s="5">
+        <v>1172</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9">
+      <c r="A38" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B38" s="5">
+        <v>144</v>
+      </c>
+      <c r="C38" s="5">
+        <v>309</v>
+      </c>
+      <c r="D38" s="5">
+        <v>451</v>
+      </c>
+      <c r="E38" s="5">
+        <v>266</v>
+      </c>
+      <c r="F38" s="5">
+        <v>248</v>
+      </c>
+      <c r="G38" s="5">
+        <v>1418</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9">
+      <c r="A40" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9">
+      <c r="A41" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="F41" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="G41" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="H41" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="I41" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9">
+      <c r="A42" t="s">
+        <v>64</v>
+      </c>
+      <c r="B42">
+        <v>17</v>
+      </c>
+      <c r="C42">
+        <v>33</v>
+      </c>
+      <c r="D42">
+        <v>27</v>
+      </c>
+      <c r="E42">
+        <v>48</v>
+      </c>
+      <c r="F42">
+        <v>53</v>
+      </c>
+      <c r="G42">
+        <v>71</v>
+      </c>
+      <c r="H42">
+        <v>3</v>
+      </c>
+      <c r="I42">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9">
+      <c r="A43" t="s">
+        <v>65</v>
+      </c>
+      <c r="B43">
+        <v>21</v>
+      </c>
+      <c r="C43">
         <v>40</v>
       </c>
-      <c r="B14">
-        <v>25</v>
-      </c>
-      <c r="C14">
+      <c r="D43">
+        <v>33</v>
+      </c>
+      <c r="E43">
+        <v>58</v>
+      </c>
+      <c r="F43">
+        <v>64</v>
+      </c>
+      <c r="G43">
+        <v>86</v>
+      </c>
+      <c r="H43">
+        <v>4</v>
+      </c>
+      <c r="I43">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9">
+      <c r="A44" t="s">
+        <v>66</v>
+      </c>
+      <c r="B44">
+        <v>6</v>
+      </c>
+      <c r="C44">
+        <v>10</v>
+      </c>
+      <c r="D44">
+        <v>11</v>
+      </c>
+      <c r="E44">
+        <v>17</v>
+      </c>
+      <c r="F44">
+        <v>18</v>
+      </c>
+      <c r="G44">
+        <v>22</v>
+      </c>
+      <c r="H44">
+        <v>0</v>
+      </c>
+      <c r="I44">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9">
+      <c r="A45" t="s">
+        <v>67</v>
+      </c>
+      <c r="B45">
+        <v>8</v>
+      </c>
+      <c r="C45">
+        <v>12</v>
+      </c>
+      <c r="D45">
+        <v>14</v>
+      </c>
+      <c r="E45">
+        <v>21</v>
+      </c>
+      <c r="F45">
+        <v>22</v>
+      </c>
+      <c r="G45">
+        <v>27</v>
+      </c>
+      <c r="H45">
+        <v>0</v>
+      </c>
+      <c r="I45">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9">
+      <c r="A46" t="s">
+        <v>60</v>
+      </c>
+      <c r="B46">
+        <v>24</v>
+      </c>
+      <c r="C46">
+        <v>24</v>
+      </c>
+      <c r="D46">
+        <v>15</v>
+      </c>
+      <c r="E46">
+        <v>30</v>
+      </c>
+      <c r="F46">
+        <v>37</v>
+      </c>
+      <c r="G46">
+        <v>31</v>
+      </c>
+      <c r="H46">
+        <v>0</v>
+      </c>
+      <c r="I46">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9">
+      <c r="A47" t="s">
+        <v>61</v>
+      </c>
+      <c r="B47">
+        <v>29</v>
+      </c>
+      <c r="C47">
+        <v>29</v>
+      </c>
+      <c r="D47">
+        <v>18</v>
+      </c>
+      <c r="E47">
+        <v>36</v>
+      </c>
+      <c r="F47">
+        <v>45</v>
+      </c>
+      <c r="G47">
+        <v>38</v>
+      </c>
+      <c r="H47">
+        <v>0</v>
+      </c>
+      <c r="I47">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9">
+      <c r="A48" t="s">
+        <v>62</v>
+      </c>
+      <c r="B48">
+        <v>4</v>
+      </c>
+      <c r="C48">
+        <v>5</v>
+      </c>
+      <c r="D48">
+        <v>4</v>
+      </c>
+      <c r="E48">
+        <v>8</v>
+      </c>
+      <c r="F48">
+        <v>8</v>
+      </c>
+      <c r="G48">
+        <v>9</v>
+      </c>
+      <c r="H48">
+        <v>0</v>
+      </c>
+      <c r="I48">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9">
+      <c r="A49" t="s">
+        <v>63</v>
+      </c>
+      <c r="B49">
+        <v>5</v>
+      </c>
+      <c r="C49">
+        <v>6</v>
+      </c>
+      <c r="D49">
+        <v>5</v>
+      </c>
+      <c r="E49">
+        <v>10</v>
+      </c>
+      <c r="F49">
+        <v>10</v>
+      </c>
+      <c r="G49">
+        <v>11</v>
+      </c>
+      <c r="H49">
+        <v>0</v>
+      </c>
+      <c r="I49">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9">
+      <c r="A50" t="s">
+        <v>68</v>
+      </c>
+      <c r="B50">
+        <v>5</v>
+      </c>
+      <c r="C50">
+        <v>7</v>
+      </c>
+      <c r="D50">
+        <v>5</v>
+      </c>
+      <c r="E50">
+        <v>10</v>
+      </c>
+      <c r="F50">
+        <v>10</v>
+      </c>
+      <c r="G50">
+        <v>12</v>
+      </c>
+      <c r="H50">
+        <v>1</v>
+      </c>
+      <c r="I50">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9">
+      <c r="A51" t="s">
         <v>69</v>
       </c>
-      <c r="D14">
+      <c r="B51">
+        <v>6</v>
+      </c>
+      <c r="C51">
+        <v>9</v>
+      </c>
+      <c r="D51">
+        <v>6</v>
+      </c>
+      <c r="E51">
+        <v>12</v>
+      </c>
+      <c r="F51">
+        <v>12</v>
+      </c>
+      <c r="G51">
+        <v>15</v>
+      </c>
+      <c r="H51">
+        <v>2</v>
+      </c>
+      <c r="I51">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9">
+      <c r="A52" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B52" s="5">
+        <v>56</v>
+      </c>
+      <c r="C52" s="5">
+        <v>79</v>
+      </c>
+      <c r="D52" s="5">
+        <v>62</v>
+      </c>
+      <c r="E52" s="5">
+        <v>113</v>
+      </c>
+      <c r="F52" s="5">
+        <v>126</v>
+      </c>
+      <c r="G52" s="5">
+        <v>145</v>
+      </c>
+      <c r="H52" s="5">
+        <v>4</v>
+      </c>
+      <c r="I52" s="5">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9">
+      <c r="A53" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="E14">
-        <v>36</v>
-      </c>
-      <c r="F14">
-        <v>201</v>
-      </c>
-      <c r="G14">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7">
-      <c r="A15" t="s">
-        <v>41</v>
-      </c>
-      <c r="B15">
-        <v>9</v>
-      </c>
-      <c r="C15">
-        <v>26</v>
-      </c>
-      <c r="D15">
-        <v>25</v>
-      </c>
-      <c r="E15">
-        <v>14</v>
-      </c>
-      <c r="F15">
-        <v>74</v>
-      </c>
-      <c r="G15">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
-      <c r="A16" t="s">
-        <v>42</v>
-      </c>
-      <c r="B16">
-        <v>31</v>
-      </c>
-      <c r="C16">
-        <v>113</v>
-      </c>
-      <c r="D16">
-        <v>123</v>
-      </c>
-      <c r="E16">
-        <v>58</v>
-      </c>
-      <c r="F16">
-        <v>325</v>
-      </c>
-      <c r="G16">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10">
-      <c r="A19" s="2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10">
-      <c r="A20" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="H20" s="3" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10">
-      <c r="A21" t="s">
-        <v>38</v>
-      </c>
-      <c r="B21">
-        <v>49</v>
-      </c>
-      <c r="C21">
-        <v>83</v>
-      </c>
-      <c r="D21">
-        <v>98</v>
-      </c>
-      <c r="E21">
-        <v>53</v>
-      </c>
-      <c r="F21">
-        <v>56</v>
-      </c>
-      <c r="G21">
-        <v>339</v>
-      </c>
-      <c r="H21">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10">
-      <c r="A22" t="s">
-        <v>39</v>
-      </c>
-      <c r="B22">
-        <v>28</v>
-      </c>
-      <c r="C22">
-        <v>75</v>
-      </c>
-      <c r="D22">
-        <v>97</v>
-      </c>
-      <c r="E22">
-        <v>56</v>
-      </c>
-      <c r="F22">
-        <v>42</v>
-      </c>
-      <c r="G22">
-        <v>298</v>
-      </c>
-      <c r="H22">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10">
-      <c r="A23" t="s">
-        <v>41</v>
-      </c>
-      <c r="B23">
-        <v>7</v>
-      </c>
-      <c r="C23">
-        <v>16</v>
-      </c>
-      <c r="D23">
-        <v>20</v>
-      </c>
-      <c r="E23">
-        <v>14</v>
-      </c>
-      <c r="F23">
-        <v>11</v>
-      </c>
-      <c r="G23">
-        <v>68</v>
-      </c>
-      <c r="H23">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10">
-      <c r="A24" t="s">
-        <v>40</v>
-      </c>
-      <c r="B24">
-        <v>15</v>
-      </c>
-      <c r="C24">
-        <v>31</v>
-      </c>
-      <c r="D24">
-        <v>61</v>
-      </c>
-      <c r="E24">
-        <v>31</v>
-      </c>
-      <c r="F24">
-        <v>36</v>
-      </c>
-      <c r="G24">
-        <v>174</v>
-      </c>
-      <c r="H24">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10">
-      <c r="A25" t="s">
-        <v>42</v>
-      </c>
-      <c r="B25">
-        <v>19</v>
-      </c>
-      <c r="C25">
-        <v>49</v>
-      </c>
-      <c r="D25">
-        <v>99</v>
-      </c>
-      <c r="E25">
-        <v>68</v>
-      </c>
-      <c r="F25">
-        <v>60</v>
-      </c>
-      <c r="G25">
-        <v>295</v>
-      </c>
-      <c r="H25">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10">
-      <c r="A28" s="2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10">
-      <c r="A29" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="D29" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="E29" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="F29" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="G29" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="H29" s="3" t="s">
+      <c r="B53" s="5">
         <v>69</v>
       </c>
-      <c r="I29" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="J29" s="3" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10">
-      <c r="A30" t="s">
-        <v>40</v>
-      </c>
-      <c r="B30">
-        <v>17</v>
-      </c>
-      <c r="C30">
-        <v>34</v>
-      </c>
-      <c r="D30">
-        <v>27</v>
-      </c>
-      <c r="E30">
-        <v>49</v>
-      </c>
-      <c r="F30">
-        <v>53</v>
-      </c>
-      <c r="G30">
-        <v>72</v>
-      </c>
-      <c r="H30">
-        <v>3</v>
-      </c>
-      <c r="I30">
-        <v>255</v>
-      </c>
-      <c r="J30">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10">
-      <c r="A31" t="s">
-        <v>41</v>
-      </c>
-      <c r="B31">
+      <c r="C53" s="5">
+        <v>96</v>
+      </c>
+      <c r="D53" s="5">
+        <v>76</v>
+      </c>
+      <c r="E53" s="5">
+        <v>137</v>
+      </c>
+      <c r="F53" s="5">
+        <v>153</v>
+      </c>
+      <c r="G53" s="5">
+        <v>177</v>
+      </c>
+      <c r="H53" s="5">
         <v>6</v>
       </c>
-      <c r="C31">
-        <v>10</v>
-      </c>
-      <c r="D31">
-        <v>12</v>
-      </c>
-      <c r="E31">
-        <v>18</v>
-      </c>
-      <c r="F31">
-        <v>19</v>
-      </c>
-      <c r="G31">
-        <v>24</v>
-      </c>
-      <c r="H31">
-        <v>0</v>
-      </c>
-      <c r="I31">
-        <v>89</v>
-      </c>
-      <c r="J31">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10">
-      <c r="A32" t="s">
-        <v>38</v>
-      </c>
-      <c r="B32">
-        <v>25</v>
-      </c>
-      <c r="C32">
-        <v>25</v>
-      </c>
-      <c r="D32">
-        <v>17</v>
-      </c>
-      <c r="E32">
-        <v>31</v>
-      </c>
-      <c r="F32">
-        <v>39</v>
-      </c>
-      <c r="G32">
-        <v>33</v>
-      </c>
-      <c r="H32">
-        <v>0</v>
-      </c>
-      <c r="I32">
-        <v>170</v>
-      </c>
-      <c r="J32">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10">
-      <c r="A33" t="s">
-        <v>39</v>
-      </c>
-      <c r="B33">
-        <v>2</v>
-      </c>
-      <c r="C33">
-        <v>13</v>
-      </c>
-      <c r="D33">
-        <v>0</v>
-      </c>
-      <c r="E33">
-        <v>4</v>
-      </c>
-      <c r="F33">
-        <v>13</v>
-      </c>
-      <c r="G33">
-        <v>12</v>
-      </c>
-      <c r="H33">
-        <v>0</v>
-      </c>
-      <c r="I33">
-        <v>44</v>
-      </c>
-      <c r="J33">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10">
-      <c r="A34" t="s">
-        <v>42</v>
-      </c>
-      <c r="B34">
-        <v>4</v>
-      </c>
-      <c r="C34">
-        <v>4</v>
-      </c>
-      <c r="D34">
-        <v>4</v>
-      </c>
-      <c r="E34">
-        <v>4</v>
-      </c>
-      <c r="F34">
-        <v>3</v>
-      </c>
-      <c r="G34">
-        <v>6</v>
-      </c>
-      <c r="H34">
-        <v>3</v>
-      </c>
-      <c r="I34">
-        <v>28</v>
-      </c>
-      <c r="J34">
-        <v>36</v>
+      <c r="I53" s="5">
+        <v>714</v>
       </c>
     </row>
   </sheetData>
@@ -2141,37 +2735,37 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
-        <v>71</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="3" t="s">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B5" s="6">
-        <v>0.1248908296943231</v>
+        <v>0.1251093613298338</v>
       </c>
       <c r="C5" s="6">
         <v>0.136</v>
@@ -2185,27 +2779,27 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B6" s="6">
-        <v>0.3441048034934498</v>
+        <v>0.3438320209973753</v>
       </c>
       <c r="C6" s="6">
         <v>0.339</v>
       </c>
       <c r="D6" s="4">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="E6" s="4">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B7" s="6">
-        <v>0.3519650655021834</v>
+        <v>0.352580927384077</v>
       </c>
       <c r="C7" s="6">
         <v>0.346</v>
@@ -2219,19 +2813,19 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B8" s="6">
-        <v>0.1790393013100437</v>
+        <v>0.1784776902887139</v>
       </c>
       <c r="C8" s="6">
         <v>0.179</v>
       </c>
       <c r="D8" s="4">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E8" s="4">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -2245,114 +2839,114 @@
         <v>1</v>
       </c>
       <c r="D9" s="4">
-        <v>1145</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="2" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="3" t="s">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="B13" s="6">
-        <v>0.100511073253833</v>
+        <v>0.1015358361774744</v>
       </c>
       <c r="C13" s="6">
         <v>0.112</v>
       </c>
       <c r="D13" s="4">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E13" s="4">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B14" s="6">
-        <v>0.2163543441226576</v>
+        <v>0.2175767918088737</v>
       </c>
       <c r="C14" s="6">
         <v>0.237</v>
       </c>
       <c r="D14" s="4">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E14" s="4">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B15" s="6">
-        <v>0.3194207836456559</v>
+        <v>0.3191126279863481</v>
       </c>
       <c r="C15" s="6">
         <v>0.305</v>
       </c>
       <c r="D15" s="4">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E15" s="4">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B16" s="6">
-        <v>0.1890971039182283</v>
+        <v>0.1877133105802048</v>
       </c>
       <c r="C16" s="6">
         <v>0.181</v>
       </c>
       <c r="D16" s="4">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="E16" s="4">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B17" s="6">
-        <v>0.1746166950596252</v>
+        <v>0.174061433447099</v>
       </c>
       <c r="C17" s="6">
         <v>0.165</v>
       </c>
       <c r="D17" s="4">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E17" s="4">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -2366,148 +2960,148 @@
         <v>1</v>
       </c>
       <c r="D18" s="4">
-        <v>1174</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="2" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="3" t="s">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="B22" s="6">
-        <v>0.09215017064846416</v>
+        <v>0.09572649572649573</v>
       </c>
       <c r="C22" s="6">
         <v>0.095</v>
       </c>
       <c r="D22" s="4">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E22" s="4">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="B23" s="6">
-        <v>0.1467576791808874</v>
+        <v>0.135042735042735</v>
       </c>
       <c r="C23" s="6">
         <v>0.139</v>
       </c>
       <c r="D23" s="4">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="E23" s="4">
-        <v>104</v>
+        <v>96</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="B24" s="6">
-        <v>0.1023890784982935</v>
+        <v>0.105982905982906</v>
       </c>
       <c r="C24" s="6">
         <v>0.101</v>
       </c>
       <c r="D24" s="4">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E24" s="4">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="B25" s="6">
-        <v>0.1808873720136519</v>
+        <v>0.1931623931623932</v>
       </c>
       <c r="C25" s="6">
         <v>0.202</v>
       </c>
       <c r="D25" s="4">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="E25" s="4">
-        <v>129</v>
+        <v>137</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="B26" s="6">
-        <v>0.2167235494880546</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="C26" s="6">
         <v>0.22</v>
       </c>
       <c r="D26" s="4">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E26" s="4">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="B27" s="6">
-        <v>0.2508532423208191</v>
+        <v>0.2478632478632479</v>
       </c>
       <c r="C27" s="6">
         <v>0.244</v>
       </c>
       <c r="D27" s="4">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="E27" s="4">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="B28" s="6">
-        <v>0.01023890784982935</v>
+        <v>0.006837606837606838</v>
       </c>
       <c r="C28" s="6">
         <v>0</v>
       </c>
       <c r="D28" s="4">
+        <v>4</v>
+      </c>
+      <c r="E28" s="4">
         <v>6</v>
-      </c>
-      <c r="E28" s="4">
-        <v>8</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -2521,7 +3115,7 @@
         <v>1</v>
       </c>
       <c r="D29" s="4">
-        <v>586</v>
+        <v>585</v>
       </c>
     </row>
   </sheetData>
@@ -2536,150 +3130,150 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>77</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B6" s="4">
-        <v>772</v>
+        <v>769</v>
       </c>
       <c r="C6" s="8">
-        <v>201.05</v>
+        <v>200.52</v>
       </c>
       <c r="D6" s="8">
-        <v>116.52</v>
+        <v>117.07</v>
       </c>
       <c r="E6" s="8">
-        <v>317.57</v>
+        <v>317.59</v>
       </c>
       <c r="F6" s="8">
         <v>317.76</v>
       </c>
       <c r="G6" s="8">
-        <v>0.19</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B7" s="4">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="C7" s="8">
-        <v>177.41</v>
+        <v>176.95</v>
       </c>
       <c r="D7" s="8">
-        <v>102.84</v>
+        <v>103.32</v>
       </c>
       <c r="E7" s="8">
-        <v>280.25</v>
+        <v>280.27</v>
       </c>
       <c r="F7" s="8">
         <v>280.44</v>
       </c>
       <c r="G7" s="8">
-        <v>0.19</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B8" s="4">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="C8" s="8">
-        <v>168.78</v>
+        <v>168.71</v>
       </c>
       <c r="D8" s="8">
         <v>0</v>
       </c>
       <c r="E8" s="8">
-        <v>168.78</v>
+        <v>168.71</v>
       </c>
       <c r="F8" s="8">
         <v>168.89</v>
       </c>
       <c r="G8" s="8">
-        <v>0.11</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B9" s="4">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="C9" s="8">
-        <v>159.9</v>
+        <v>159.74</v>
       </c>
       <c r="D9" s="8">
         <v>0</v>
       </c>
       <c r="E9" s="8">
-        <v>159.9</v>
+        <v>159.74</v>
       </c>
       <c r="F9" s="8">
         <v>159.91</v>
       </c>
       <c r="G9" s="8">
-        <v>0.01</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B10" s="4">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C10" s="8">
-        <v>58.78</v>
+        <v>58.68</v>
       </c>
       <c r="D10" s="8">
         <v>0</v>
       </c>
       <c r="E10" s="8">
-        <v>58.78</v>
+        <v>58.68</v>
       </c>
       <c r="F10" s="8">
         <v>58.84</v>
       </c>
       <c r="G10" s="8">
-        <v>0.06</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -2687,26 +3281,26 @@
         <v>32</v>
       </c>
       <c r="B11" s="4">
-        <v>2905</v>
+        <v>2900</v>
       </c>
       <c r="E11" s="8">
-        <v>985.28</v>
+        <v>984.99</v>
       </c>
       <c r="F11" s="8">
         <v>985.84</v>
       </c>
       <c r="G11" s="8">
-        <v>0.5600000000000001</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="2" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" s="2" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -2714,7 +3308,7 @@
         <v>26</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -2753,58 +3347,58 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="3" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>30</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B4">
-        <v>897</v>
+        <v>901</v>
       </c>
       <c r="C4">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="D4">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="E4">
-        <v>116.52</v>
+        <v>117.07</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B5">
-        <v>792</v>
+        <v>796</v>
       </c>
       <c r="C5">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="D5">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="E5">
-        <v>102.84</v>
+        <v>103.32</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -2812,10 +3406,10 @@
         <v>32</v>
       </c>
       <c r="B6" s="4">
-        <v>1689</v>
+        <v>1697</v>
       </c>
       <c r="E6" s="8">
-        <v>219.36</v>
+        <v>220.4</v>
       </c>
     </row>
   </sheetData>
@@ -2830,72 +3424,72 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>93</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="2" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="3" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="B5" s="8">
         <v>361.2</v>
       </c>
       <c r="C5" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="B6" s="8">
         <v>125.1</v>
       </c>
       <c r="C6" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="B7" s="8">
         <v>157</v>
       </c>
       <c r="C7" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="B8" s="8">
         <v>62.8</v>
       </c>
       <c r="C8" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="5" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="B9" s="8">
         <v>706.1</v>
@@ -2903,67 +3497,67 @@
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="2" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="3" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="B13" s="8">
         <v>157</v>
       </c>
       <c r="C13" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
       <c r="B14" s="8">
         <v>94.2</v>
       </c>
       <c r="C14" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="B15" s="8">
         <v>65.59999999999999</v>
       </c>
       <c r="C15" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="B16" s="8">
         <v>65.5</v>
       </c>
       <c r="C16" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="5" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="B17" s="8">
         <v>382.3</v>
@@ -2971,7 +3565,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="5" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="B19" s="8">
         <v>1088.4</v>
@@ -2989,7 +3583,7 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -2999,27 +3593,27 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="3" t="s">
-        <v>53</v>
+        <v>128</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>116</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B5">
         <v>35</v>
@@ -3031,15 +3625,15 @@
         <v>95</v>
       </c>
       <c r="E5">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F5">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B6">
         <v>43</v>
@@ -3059,7 +3653,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B7">
         <v>25</v>
@@ -3079,7 +3673,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B8">
         <v>9</v>
@@ -3099,13 +3693,13 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B9">
         <v>31</v>
       </c>
       <c r="C9">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D9">
         <v>123</v>
@@ -3114,7 +3708,7 @@
         <v>58</v>
       </c>
       <c r="F9">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -3124,108 +3718,108 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="3" t="s">
-        <v>53</v>
+        <v>128</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>116</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B13">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C13">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D13">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E13">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F13">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G13">
-        <v>339</v>
+        <v>346</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B14">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C14">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D14">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E14">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F14">
         <v>42</v>
       </c>
       <c r="G14">
-        <v>298</v>
+        <v>303</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B15">
         <v>7</v>
       </c>
       <c r="C15">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D15">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E15">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F15">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G15">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B16">
         <v>15</v>
       </c>
       <c r="C16">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D16">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E16">
         <v>31</v>
@@ -3234,30 +3828,30 @@
         <v>36</v>
       </c>
       <c r="G16">
-        <v>174</v>
+        <v>176</v>
       </c>
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B17">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C17">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D17">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="E17">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="F17">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G17">
-        <v>295</v>
+        <v>275</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -3267,65 +3861,65 @@
     </row>
     <row r="20" spans="1:9">
       <c r="A20" s="3" t="s">
-        <v>53</v>
+        <v>128</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>116</v>
+        <v>59</v>
       </c>
     </row>
     <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B21">
         <v>17</v>
       </c>
       <c r="C21">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D21">
         <v>27</v>
       </c>
       <c r="E21">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F21">
         <v>53</v>
       </c>
       <c r="G21">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H21">
         <v>3</v>
       </c>
       <c r="I21">
-        <v>255</v>
+        <v>252</v>
       </c>
     </row>
     <row r="22" spans="1:9">
       <c r="A22" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B22">
         <v>6</v>
@@ -3334,109 +3928,109 @@
         <v>10</v>
       </c>
       <c r="D22">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E22">
+        <v>17</v>
+      </c>
+      <c r="F22">
         <v>18</v>
       </c>
-      <c r="F22">
-        <v>19</v>
-      </c>
       <c r="G22">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="H22">
         <v>0</v>
       </c>
       <c r="I22">
-        <v>89</v>
+        <v>84</v>
       </c>
     </row>
     <row r="23" spans="1:9">
       <c r="A23" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B23">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C23">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D23">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E23">
+        <v>30</v>
+      </c>
+      <c r="F23">
+        <v>37</v>
+      </c>
+      <c r="G23">
         <v>31</v>
-      </c>
-      <c r="F23">
-        <v>39</v>
-      </c>
-      <c r="G23">
-        <v>33</v>
       </c>
       <c r="H23">
         <v>0</v>
       </c>
       <c r="I23">
-        <v>170</v>
+        <v>161</v>
       </c>
     </row>
     <row r="24" spans="1:9">
       <c r="A24" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B24">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C24">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D24">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E24">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F24">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="G24">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="H24">
         <v>0</v>
       </c>
       <c r="I24">
-        <v>44</v>
+        <v>38</v>
       </c>
     </row>
     <row r="25" spans="1:9">
       <c r="A25" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B25">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C25">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D25">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E25">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F25">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G25">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H25">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I25">
-        <v>28</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Explore Pants: shorts 1550, dashboard tallas, CAB 2XL y Negro CAB
Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/EXPLORE_PANTS_Proyeccion_Produccion.xlsx
+++ b/EXPLORE_PANTS_Proyeccion_Produccion.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="140">
   <si>
     <t>EXPLORE PANTS — PROYECCIÓN ANCLADA A JUSTIFICACIÓN NOVAKTEX</t>
   </si>
@@ -31,7 +31,7 @@
     <t>Fuente: DATA_JUSTIFICACI_N_COMPRA_TELA_NOVAKTEX_REPEl_c4ef.xlsx</t>
   </si>
   <si>
-    <t>Meta Explore Pants: 2,900 und · Shorts R1 ≥ 1,500 und</t>
+    <t>Meta Explore Pants: tela completa · Shorts R1 = 1,550 und</t>
   </si>
   <si>
     <t>Demanda proyectada Jul–Dic: 2,228 und</t>
@@ -40,7 +40,7 @@
     <t>Stock referencia justificación: 2,988 und (1,636 tiendas + 1,352 taller)</t>
   </si>
   <si>
-    <t>Stock actual dashboard: 2,988 und</t>
+    <t>Stock actual dashboard: 3,249 und</t>
   </si>
   <si>
     <t>Tela en almacén (existencias): 985.8 kg · uso total Explore + Shorts</t>
@@ -151,15 +151,15 @@
     <t>Kaki</t>
   </si>
   <si>
+    <t>Gris Oscuro</t>
+  </si>
+  <si>
+    <t>Verde Militar</t>
+  </si>
+  <si>
     <t>Azul Marino</t>
   </si>
   <si>
-    <t>Verde Militar</t>
-  </si>
-  <si>
-    <t>Gris Oscuro</t>
-  </si>
-  <si>
     <t>EXPLORE PANTS — UNIDADES A PRODUCIR POR COLOR (TOTAL)</t>
   </si>
   <si>
@@ -202,6 +202,9 @@
     <t>XL</t>
   </si>
   <si>
+    <t>2XL</t>
+  </si>
+  <si>
     <t>Total</t>
   </si>
   <si>
@@ -217,24 +220,24 @@
     <t>Kaki — MÁX</t>
   </si>
   <si>
+    <t>Gris Oscuro — MÍN</t>
+  </si>
+  <si>
+    <t>Gris Oscuro — MÁX</t>
+  </si>
+  <si>
+    <t>Verde Militar — MÍN</t>
+  </si>
+  <si>
+    <t>Verde Militar — MÁX</t>
+  </si>
+  <si>
     <t>Azul Marino — MÍN</t>
   </si>
   <si>
     <t>Azul Marino — MÁX</t>
   </si>
   <si>
-    <t>Verde Militar — MÍN</t>
-  </si>
-  <si>
-    <t>Verde Militar — MÁX</t>
-  </si>
-  <si>
-    <t>Gris Oscuro — MÍN</t>
-  </si>
-  <si>
-    <t>Gris Oscuro — MÁX</t>
-  </si>
-  <si>
     <t>TOTAL — MÍN</t>
   </si>
   <si>
@@ -316,7 +319,7 @@
     <t>Delta</t>
   </si>
   <si>
-    <t>Shorts R1 total: 1,697 und · 220.4 kg</t>
+    <t>Shorts R1 total: 1,550 und · 201.81 kg</t>
   </si>
   <si>
     <t>Consumo referencial por género (kg/und)</t>
@@ -418,7 +421,7 @@
     <t>1. Tela en almacén: 985.8 kg — se usa completa (Explore + Shorts R1).</t>
   </si>
   <si>
-    <t>2. Explore Pants meta ~2,900 und · Shorts R1 ≥ 1,500 und (Negro/Gris, CAB/DAMA).</t>
+    <t>2. Explore Pants: und según tela restante · Shorts R1 = 1,550 und (Negro/Gris, CAB/DAMA).</t>
   </si>
   <si>
     <t>3. Rango MÍN/MÁX Explore: factor temporada alta ×1.2.</t>
@@ -995,7 +998,7 @@
         <v>760</v>
       </c>
       <c r="C27" s="4">
-        <v>760</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -1006,7 +1009,7 @@
         <v>3668</v>
       </c>
       <c r="C28" s="4">
-        <v>3660</v>
+        <v>3921</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -1025,10 +1028,10 @@
         <v>29</v>
       </c>
       <c r="B31">
-        <v>1143</v>
+        <v>1189</v>
       </c>
       <c r="C31">
-        <v>1379</v>
+        <v>1437</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -1036,10 +1039,10 @@
         <v>30</v>
       </c>
       <c r="B32">
-        <v>1172</v>
+        <v>1192</v>
       </c>
       <c r="C32">
-        <v>1418</v>
+        <v>1442</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -1058,10 +1061,10 @@
         <v>32</v>
       </c>
       <c r="B34" s="5">
-        <v>2900</v>
+        <v>2966</v>
       </c>
       <c r="C34" s="5">
-        <v>3511</v>
+        <v>3593</v>
       </c>
     </row>
   </sheetData>
@@ -1082,52 +1085,52 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -1178,16 +1181,16 @@
         <v>40</v>
       </c>
       <c r="C5" s="4">
-        <v>262</v>
+        <v>322</v>
       </c>
       <c r="D5" s="4">
-        <v>316</v>
+        <v>389</v>
       </c>
       <c r="E5" s="6">
-        <v>0.2292213473315836</v>
+        <v>0.2708158116063919</v>
       </c>
       <c r="F5" s="6">
-        <v>0.252</v>
+        <v>0.272</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1198,16 +1201,16 @@
         <v>41</v>
       </c>
       <c r="C6" s="4">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D6" s="4">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="E6" s="6">
-        <v>0.2467191601049869</v>
+        <v>0.2380151387720774</v>
       </c>
       <c r="F6" s="6">
-        <v>0.211</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1218,16 +1221,16 @@
         <v>42</v>
       </c>
       <c r="C7" s="4">
-        <v>201</v>
+        <v>275</v>
       </c>
       <c r="D7" s="4">
-        <v>243</v>
+        <v>332</v>
       </c>
       <c r="E7" s="6">
-        <v>0.1758530183727034</v>
+        <v>0.2312867956265769</v>
       </c>
       <c r="F7" s="6">
-        <v>0.17</v>
+        <v>0.196</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1238,16 +1241,16 @@
         <v>43</v>
       </c>
       <c r="C8" s="4">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="D8" s="4">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="E8" s="6">
-        <v>0.0647419072615923</v>
+        <v>0.07232968881412952</v>
       </c>
       <c r="F8" s="6">
-        <v>0.164</v>
+        <v>0.162</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1258,16 +1261,16 @@
         <v>44</v>
       </c>
       <c r="C9" s="4">
-        <v>324</v>
+        <v>223</v>
       </c>
       <c r="D9" s="4">
-        <v>391</v>
+        <v>269</v>
       </c>
       <c r="E9" s="6">
-        <v>0.2834645669291339</v>
+        <v>0.1875525651808242</v>
       </c>
       <c r="F9" s="6">
-        <v>0.06900000000000001</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1275,7 +1278,7 @@
         <v>32</v>
       </c>
       <c r="B10" s="4">
-        <v>1143</v>
+        <v>1189</v>
       </c>
       <c r="C10" s="7">
         <v>1</v>
@@ -1314,16 +1317,16 @@
         <v>40</v>
       </c>
       <c r="C14" s="4">
-        <v>346</v>
+        <v>334</v>
       </c>
       <c r="D14" s="4">
-        <v>416</v>
+        <v>402</v>
       </c>
       <c r="E14" s="6">
-        <v>0.295221843003413</v>
+        <v>0.2802013422818792</v>
       </c>
       <c r="F14" s="6">
-        <v>0.306</v>
+        <v>0.298</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -1334,16 +1337,16 @@
         <v>41</v>
       </c>
       <c r="C15" s="4">
-        <v>303</v>
+        <v>334</v>
       </c>
       <c r="D15" s="4">
-        <v>366</v>
+        <v>403</v>
       </c>
       <c r="E15" s="6">
-        <v>0.2585324232081911</v>
+        <v>0.2802013422818792</v>
       </c>
       <c r="F15" s="6">
-        <v>0.209</v>
+        <v>0.223</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -1351,19 +1354,19 @@
         <v>3</v>
       </c>
       <c r="B16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C16" s="4">
-        <v>72</v>
+        <v>264</v>
       </c>
       <c r="D16" s="4">
-        <v>89</v>
+        <v>320</v>
       </c>
       <c r="E16" s="6">
-        <v>0.06143344709897611</v>
+        <v>0.2214765100671141</v>
       </c>
       <c r="F16" s="6">
-        <v>0.142</v>
+        <v>0.198</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -1371,19 +1374,19 @@
         <v>4</v>
       </c>
       <c r="B17" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C17" s="4">
-        <v>176</v>
+        <v>191</v>
       </c>
       <c r="D17" s="4">
-        <v>214</v>
+        <v>232</v>
       </c>
       <c r="E17" s="6">
-        <v>0.1501706484641638</v>
+        <v>0.1602348993288591</v>
       </c>
       <c r="F17" s="6">
-        <v>0.139</v>
+        <v>0.145</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -1391,19 +1394,19 @@
         <v>5</v>
       </c>
       <c r="B18" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C18" s="4">
-        <v>275</v>
+        <v>69</v>
       </c>
       <c r="D18" s="4">
-        <v>333</v>
+        <v>85</v>
       </c>
       <c r="E18" s="6">
-        <v>0.234641638225256</v>
+        <v>0.05788590604026846</v>
       </c>
       <c r="F18" s="6">
-        <v>0.058</v>
+        <v>0.136</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -1411,7 +1414,7 @@
         <v>32</v>
       </c>
       <c r="B19" s="4">
-        <v>1172</v>
+        <v>1192</v>
       </c>
       <c r="C19" s="7">
         <v>1</v>
@@ -1447,19 +1450,19 @@
         <v>1</v>
       </c>
       <c r="B23" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C23" s="4">
-        <v>252</v>
+        <v>205</v>
       </c>
       <c r="D23" s="4">
-        <v>306</v>
+        <v>249</v>
       </c>
       <c r="E23" s="6">
-        <v>0.4307692307692308</v>
+        <v>0.3504273504273504</v>
       </c>
       <c r="F23" s="6">
-        <v>0.298</v>
+        <v>0.284</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -1470,16 +1473,16 @@
         <v>43</v>
       </c>
       <c r="C24" s="4">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="D24" s="4">
-        <v>104</v>
+        <v>87</v>
       </c>
       <c r="E24" s="6">
-        <v>0.1435897435897436</v>
+        <v>0.1213675213675214</v>
       </c>
       <c r="F24" s="6">
-        <v>0.269</v>
+        <v>0.253</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -1490,13 +1493,13 @@
         <v>40</v>
       </c>
       <c r="C25" s="4">
-        <v>161</v>
+        <v>138</v>
       </c>
       <c r="D25" s="4">
-        <v>195</v>
+        <v>168</v>
       </c>
       <c r="E25" s="6">
-        <v>0.2752136752136752</v>
+        <v>0.2358974358974359</v>
       </c>
       <c r="F25" s="6">
         <v>0.225</v>
@@ -1507,19 +1510,19 @@
         <v>4</v>
       </c>
       <c r="B26" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C26" s="4">
-        <v>38</v>
+        <v>169</v>
       </c>
       <c r="D26" s="4">
-        <v>47</v>
+        <v>206</v>
       </c>
       <c r="E26" s="6">
-        <v>0.06495726495726496</v>
+        <v>0.2888888888888889</v>
       </c>
       <c r="F26" s="6">
-        <v>0.045</v>
+        <v>0.154</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -1527,19 +1530,19 @@
         <v>5</v>
       </c>
       <c r="B27" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C27" s="4">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="D27" s="4">
-        <v>62</v>
+        <v>4</v>
       </c>
       <c r="E27" s="6">
-        <v>0.08547008547008547</v>
+        <v>0.003418803418803419</v>
       </c>
       <c r="F27" s="6">
-        <v>0.008</v>
+        <v>0.08400000000000001</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -1590,10 +1593,10 @@
         <v>40</v>
       </c>
       <c r="B4" s="4">
-        <v>769</v>
+        <v>794</v>
       </c>
       <c r="C4" s="6">
-        <v>0.2651724137931035</v>
+        <v>0.2677006068779501</v>
       </c>
       <c r="D4" s="6">
         <v>0.3223210782341178</v>
@@ -1604,13 +1607,13 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B5" s="4">
-        <v>649</v>
+        <v>708</v>
       </c>
       <c r="C5" s="6">
-        <v>0.2237931034482759</v>
+        <v>0.2387053270397842</v>
       </c>
       <c r="D5" s="6">
         <v>0.2844671001033621</v>
@@ -1624,10 +1627,10 @@
         <v>41</v>
       </c>
       <c r="B6" s="4">
-        <v>623</v>
+        <v>619</v>
       </c>
       <c r="C6" s="6">
-        <v>0.2148275862068965</v>
+        <v>0.2086985839514498</v>
       </c>
       <c r="D6" s="6">
         <v>0.1713177091328877</v>
@@ -1638,13 +1641,13 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B7" s="4">
-        <v>629</v>
+        <v>619</v>
       </c>
       <c r="C7" s="6">
-        <v>0.2168965517241379</v>
+        <v>0.2086985839514498</v>
       </c>
       <c r="D7" s="6">
         <v>0.1622064538507951</v>
@@ -1658,10 +1661,10 @@
         <v>43</v>
       </c>
       <c r="B8" s="4">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="C8" s="6">
-        <v>0.07931034482758621</v>
+        <v>0.07619689817936615</v>
       </c>
       <c r="D8" s="6">
         <v>0.05968765867883735</v>
@@ -1675,7 +1678,7 @@
         <v>32</v>
       </c>
       <c r="B9" s="4">
-        <v>2900</v>
+        <v>2966</v>
       </c>
       <c r="C9" s="7">
         <v>1</v>
@@ -1697,12 +1700,12 @@
   <dimension ref="A1:I53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:7">
       <c r="A3" s="3" t="s">
         <v>26</v>
       </c>
@@ -1716,35 +1719,35 @@
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:7">
       <c r="A4" t="s">
         <v>29</v>
       </c>
       <c r="B4">
-        <v>1143</v>
+        <v>1189</v>
       </c>
       <c r="C4">
-        <v>1379</v>
+        <v>1437</v>
       </c>
       <c r="D4">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
       <c r="A5" t="s">
         <v>30</v>
       </c>
       <c r="B5">
-        <v>1172</v>
+        <v>1192</v>
       </c>
       <c r="C5">
-        <v>1418</v>
+        <v>1442</v>
       </c>
       <c r="D5">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
       <c r="A6" t="s">
         <v>31</v>
       </c>
@@ -1758,26 +1761,26 @@
         <v>129</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:7">
       <c r="A7" s="5" t="s">
         <v>32</v>
       </c>
       <c r="B7" s="5">
-        <v>2900</v>
+        <v>2966</v>
       </c>
       <c r="C7" s="5">
-        <v>3511</v>
+        <v>3593</v>
       </c>
       <c r="D7" s="5">
-        <v>611</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
       <c r="A10" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:7">
       <c r="A11" s="3" t="s">
         <v>35</v>
       </c>
@@ -1796,250 +1799,289 @@
       <c r="F11" s="3" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="12" spans="1:6">
+      <c r="G11" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B12">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C12">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="D12">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="E12">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="F12">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6">
+        <v>21</v>
+      </c>
+      <c r="G12">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B13">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="C13">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="D13">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="E13">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="F13">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6">
+        <v>26</v>
+      </c>
+      <c r="G13">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
       <c r="A14" t="s">
+        <v>63</v>
+      </c>
+      <c r="B14">
+        <v>44</v>
+      </c>
+      <c r="C14">
+        <v>92</v>
+      </c>
+      <c r="D14">
+        <v>85</v>
+      </c>
+      <c r="E14">
+        <v>51</v>
+      </c>
+      <c r="F14">
+        <v>11</v>
+      </c>
+      <c r="G14">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" t="s">
+        <v>64</v>
+      </c>
+      <c r="B15">
+        <v>53</v>
+      </c>
+      <c r="C15">
+        <v>111</v>
+      </c>
+      <c r="D15">
+        <v>102</v>
+      </c>
+      <c r="E15">
         <v>62</v>
       </c>
-      <c r="B14">
-        <v>43</v>
-      </c>
-      <c r="C14">
-        <v>95</v>
-      </c>
-      <c r="D14">
-        <v>89</v>
-      </c>
-      <c r="E14">
-        <v>55</v>
-      </c>
-      <c r="F14">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6">
-      <c r="A15" t="s">
-        <v>63</v>
-      </c>
-      <c r="B15">
-        <v>52</v>
-      </c>
-      <c r="C15">
-        <v>114</v>
-      </c>
-      <c r="D15">
-        <v>107</v>
-      </c>
-      <c r="E15">
-        <v>66</v>
-      </c>
       <c r="F15">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6">
+        <v>14</v>
+      </c>
+      <c r="G15">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B16">
-        <v>25</v>
+        <v>46</v>
       </c>
       <c r="C16">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="D16">
-        <v>71</v>
+        <v>94</v>
       </c>
       <c r="E16">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="F16">
-        <v>201</v>
+        <v>4</v>
+      </c>
+      <c r="G16">
+        <v>275</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B17">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C17">
-        <v>83</v>
+        <v>105</v>
       </c>
       <c r="D17">
-        <v>86</v>
+        <v>113</v>
       </c>
       <c r="E17">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="F17">
-        <v>243</v>
+        <v>5</v>
+      </c>
+      <c r="G17">
+        <v>332</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B18">
         <v>9</v>
       </c>
       <c r="C18">
+        <v>25</v>
+      </c>
+      <c r="D18">
         <v>26</v>
       </c>
-      <c r="D18">
-        <v>25</v>
-      </c>
       <c r="E18">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F18">
-        <v>74</v>
+        <v>13</v>
+      </c>
+      <c r="G18">
+        <v>86</v>
       </c>
     </row>
     <row r="19" spans="1:7">
       <c r="A19" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B19">
         <v>11</v>
       </c>
       <c r="C19">
+        <v>30</v>
+      </c>
+      <c r="D19">
         <v>32</v>
       </c>
-      <c r="D19">
-        <v>30</v>
-      </c>
       <c r="E19">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F19">
-        <v>90</v>
+        <v>16</v>
+      </c>
+      <c r="G19">
+        <v>105</v>
       </c>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B20">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="C20">
-        <v>112</v>
+        <v>66</v>
       </c>
       <c r="D20">
-        <v>123</v>
+        <v>64</v>
       </c>
       <c r="E20">
-        <v>58</v>
+        <v>35</v>
       </c>
       <c r="F20">
-        <v>324</v>
+        <v>35</v>
+      </c>
+      <c r="G20">
+        <v>223</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B21">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="C21">
-        <v>135</v>
+        <v>80</v>
       </c>
       <c r="D21">
-        <v>148</v>
+        <v>77</v>
       </c>
       <c r="E21">
-        <v>70</v>
+        <v>42</v>
       </c>
       <c r="F21">
-        <v>391</v>
+        <v>42</v>
+      </c>
+      <c r="G21">
+        <v>269</v>
       </c>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B22" s="5">
-        <v>143</v>
+        <v>163</v>
       </c>
       <c r="C22" s="5">
-        <v>393</v>
+        <v>372</v>
       </c>
       <c r="D22" s="5">
-        <v>403</v>
+        <v>372</v>
       </c>
       <c r="E22" s="5">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="F22" s="5">
-        <v>1143</v>
+        <v>84</v>
+      </c>
+      <c r="G22" s="5">
+        <v>1189</v>
       </c>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B23" s="5">
-        <v>173</v>
+        <v>198</v>
       </c>
       <c r="C23" s="5">
-        <v>474</v>
+        <v>449</v>
       </c>
       <c r="D23" s="5">
-        <v>485</v>
+        <v>448</v>
       </c>
       <c r="E23" s="5">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="F23" s="5">
-        <v>1379</v>
+        <v>103</v>
+      </c>
+      <c r="G23" s="5">
+        <v>1437</v>
       </c>
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -2047,7 +2089,7 @@
         <v>35</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>55</v>
@@ -2062,288 +2104,288 @@
         <v>58</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="27" spans="1:7">
       <c r="A27" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B27">
+        <v>53</v>
+      </c>
+      <c r="C27">
+        <v>83</v>
+      </c>
+      <c r="D27">
+        <v>99</v>
+      </c>
+      <c r="E27">
         <v>50</v>
       </c>
-      <c r="C27">
-        <v>84</v>
-      </c>
-      <c r="D27">
-        <v>100</v>
-      </c>
-      <c r="E27">
-        <v>54</v>
-      </c>
       <c r="F27">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="G27">
-        <v>346</v>
+        <v>334</v>
       </c>
     </row>
     <row r="28" spans="1:7">
       <c r="A28" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B28">
+        <v>64</v>
+      </c>
+      <c r="C28">
+        <v>100</v>
+      </c>
+      <c r="D28">
+        <v>119</v>
+      </c>
+      <c r="E28">
         <v>60</v>
       </c>
-      <c r="C28">
-        <v>101</v>
-      </c>
-      <c r="D28">
-        <v>120</v>
-      </c>
-      <c r="E28">
-        <v>65</v>
-      </c>
       <c r="F28">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="G28">
-        <v>416</v>
+        <v>402</v>
       </c>
     </row>
     <row r="29" spans="1:7">
       <c r="A29" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B29">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="C29">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="D29">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="E29">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="F29">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G29">
-        <v>303</v>
+        <v>334</v>
       </c>
     </row>
     <row r="30" spans="1:7">
       <c r="A30" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B30">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C30">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="D30">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="E30">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="F30">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G30">
-        <v>366</v>
+        <v>403</v>
       </c>
     </row>
     <row r="31" spans="1:7">
       <c r="A31" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B31">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="C31">
-        <v>17</v>
+        <v>67</v>
       </c>
       <c r="D31">
-        <v>21</v>
+        <v>77</v>
       </c>
       <c r="E31">
-        <v>15</v>
+        <v>48</v>
       </c>
       <c r="F31">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="G31">
-        <v>72</v>
+        <v>264</v>
       </c>
     </row>
     <row r="32" spans="1:7">
       <c r="A32" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B32">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="C32">
-        <v>21</v>
+        <v>81</v>
       </c>
       <c r="D32">
-        <v>26</v>
+        <v>93</v>
       </c>
       <c r="E32">
-        <v>18</v>
+        <v>58</v>
       </c>
       <c r="F32">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="G32">
-        <v>89</v>
+        <v>320</v>
       </c>
     </row>
     <row r="33" spans="1:9">
       <c r="A33" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="B33">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C33">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="D33">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E33">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="F33">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G33">
-        <v>176</v>
+        <v>191</v>
       </c>
     </row>
     <row r="34" spans="1:9">
       <c r="A34" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="B34">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C34">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="D34">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="E34">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F34">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G34">
-        <v>214</v>
+        <v>232</v>
       </c>
     </row>
     <row r="35" spans="1:9">
       <c r="A35" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B35">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="C35">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="D35">
-        <v>92</v>
+        <v>20</v>
       </c>
       <c r="E35">
-        <v>63</v>
+        <v>14</v>
       </c>
       <c r="F35">
-        <v>56</v>
+        <v>11</v>
       </c>
       <c r="G35">
-        <v>275</v>
+        <v>69</v>
       </c>
     </row>
     <row r="36" spans="1:9">
       <c r="A36" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B36">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="C36">
-        <v>56</v>
+        <v>21</v>
       </c>
       <c r="D36">
-        <v>111</v>
+        <v>24</v>
       </c>
       <c r="E36">
-        <v>76</v>
+        <v>17</v>
       </c>
       <c r="F36">
-        <v>68</v>
+        <v>14</v>
       </c>
       <c r="G36">
-        <v>333</v>
+        <v>85</v>
       </c>
     </row>
     <row r="37" spans="1:9">
       <c r="A37" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B37" s="5">
-        <v>119</v>
+        <v>145</v>
       </c>
       <c r="C37" s="5">
-        <v>255</v>
+        <v>291</v>
       </c>
       <c r="D37" s="5">
-        <v>374</v>
+        <v>366</v>
       </c>
       <c r="E37" s="5">
-        <v>220</v>
+        <v>209</v>
       </c>
       <c r="F37" s="5">
-        <v>204</v>
+        <v>181</v>
       </c>
       <c r="G37" s="5">
-        <v>1172</v>
+        <v>1192</v>
       </c>
     </row>
     <row r="38" spans="1:9">
       <c r="A38" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B38" s="5">
-        <v>144</v>
+        <v>177</v>
       </c>
       <c r="C38" s="5">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="D38" s="5">
-        <v>451</v>
+        <v>441</v>
       </c>
       <c r="E38" s="5">
-        <v>266</v>
+        <v>252</v>
       </c>
       <c r="F38" s="5">
-        <v>248</v>
+        <v>220</v>
       </c>
       <c r="G38" s="5">
-        <v>1418</v>
+        <v>1442</v>
       </c>
     </row>
     <row r="40" spans="1:9">
       <c r="A40" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="41" spans="1:9">
@@ -2351,344 +2393,344 @@
         <v>35</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H41" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="I41" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="42" spans="1:9">
       <c r="A42" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="B42">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C42">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="D42">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="E42">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="F42">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="G42">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="H42">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I42">
-        <v>252</v>
+        <v>205</v>
       </c>
     </row>
     <row r="43" spans="1:9">
       <c r="A43" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="B43">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C43">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="D43">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="E43">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="F43">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="G43">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="H43">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I43">
-        <v>306</v>
+        <v>249</v>
       </c>
     </row>
     <row r="44" spans="1:9">
       <c r="A44" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B44">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C44">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D44">
         <v>11</v>
       </c>
       <c r="E44">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F44">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="G44">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="H44">
         <v>0</v>
       </c>
       <c r="I44">
-        <v>84</v>
+        <v>71</v>
       </c>
     </row>
     <row r="45" spans="1:9">
       <c r="A45" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B45">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C45">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D45">
         <v>14</v>
       </c>
       <c r="E45">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F45">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="G45">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="H45">
         <v>0</v>
       </c>
       <c r="I45">
-        <v>104</v>
+        <v>87</v>
       </c>
     </row>
     <row r="46" spans="1:9">
       <c r="A46" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B46">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="C46">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="D46">
         <v>15</v>
       </c>
       <c r="E46">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F46">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="G46">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H46">
         <v>0</v>
       </c>
       <c r="I46">
-        <v>161</v>
+        <v>138</v>
       </c>
     </row>
     <row r="47" spans="1:9">
       <c r="A47" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B47">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="C47">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D47">
         <v>18</v>
       </c>
       <c r="E47">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="F47">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="G47">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="H47">
         <v>0</v>
       </c>
       <c r="I47">
-        <v>195</v>
+        <v>168</v>
       </c>
     </row>
     <row r="48" spans="1:9">
       <c r="A48" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B48">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="C48">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="D48">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="E48">
-        <v>8</v>
+        <v>45</v>
       </c>
       <c r="F48">
-        <v>8</v>
+        <v>36</v>
       </c>
       <c r="G48">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="H48">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I48">
-        <v>38</v>
+        <v>169</v>
       </c>
     </row>
     <row r="49" spans="1:9">
       <c r="A49" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B49">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="C49">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="D49">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="E49">
-        <v>10</v>
+        <v>54</v>
       </c>
       <c r="F49">
-        <v>10</v>
+        <v>44</v>
       </c>
       <c r="G49">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="H49">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I49">
-        <v>47</v>
+        <v>206</v>
       </c>
     </row>
     <row r="50" spans="1:9">
       <c r="A50" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="B50">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C50">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D50">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E50">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F50">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G50">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="H50">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I50">
-        <v>50</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51" spans="1:9">
       <c r="A51" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="B51">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="C51">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="D51">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E51">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="F51">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="G51">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="H51">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I51">
-        <v>62</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52" spans="1:9">
       <c r="A52" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B52" s="5">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C52" s="5">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="D52" s="5">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E52" s="5">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="F52" s="5">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G52" s="5">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="H52" s="5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I52" s="5">
         <v>585</v>
@@ -2696,28 +2738,28 @@
     </row>
     <row r="53" spans="1:9">
       <c r="A53" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B53" s="5">
         <v>71</v>
       </c>
-      <c r="B53" s="5">
-        <v>69</v>
-      </c>
       <c r="C53" s="5">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D53" s="5">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E53" s="5">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="F53" s="5">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="G53" s="5">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="H53" s="5">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I53" s="5">
         <v>714</v>
@@ -2730,22 +2772,22 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>38</v>
@@ -2754,10 +2796,10 @@
         <v>39</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -2765,16 +2807,16 @@
         <v>55</v>
       </c>
       <c r="B5" s="6">
-        <v>0.1251093613298338</v>
+        <v>0.1370899915895711</v>
       </c>
       <c r="C5" s="6">
-        <v>0.136</v>
+        <v>0.141</v>
       </c>
       <c r="D5" s="4">
-        <v>143</v>
+        <v>163</v>
       </c>
       <c r="E5" s="4">
-        <v>173</v>
+        <v>198</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -2782,16 +2824,16 @@
         <v>56</v>
       </c>
       <c r="B6" s="6">
-        <v>0.3438320209973753</v>
+        <v>0.3128679562657696</v>
       </c>
       <c r="C6" s="6">
-        <v>0.339</v>
+        <v>0.334</v>
       </c>
       <c r="D6" s="4">
-        <v>393</v>
+        <v>372</v>
       </c>
       <c r="E6" s="4">
-        <v>474</v>
+        <v>449</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -2799,16 +2841,16 @@
         <v>57</v>
       </c>
       <c r="B7" s="6">
-        <v>0.352580927384077</v>
+        <v>0.3128679562657696</v>
       </c>
       <c r="C7" s="6">
-        <v>0.346</v>
+        <v>0.336</v>
       </c>
       <c r="D7" s="4">
-        <v>403</v>
+        <v>372</v>
       </c>
       <c r="E7" s="4">
-        <v>485</v>
+        <v>448</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -2816,190 +2858,190 @@
         <v>58</v>
       </c>
       <c r="B8" s="6">
-        <v>0.1784776902887139</v>
+        <v>0.1665264928511354</v>
       </c>
       <c r="C8" s="6">
-        <v>0.179</v>
+        <v>0.178</v>
       </c>
       <c r="D8" s="4">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="E8" s="4">
-        <v>247</v>
+        <v>239</v>
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="5" t="s">
+      <c r="A9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B9" s="6">
+        <v>0.07064760302775441</v>
+      </c>
+      <c r="C9" s="6">
+        <v>0.011</v>
+      </c>
+      <c r="D9" s="4">
+        <v>84</v>
+      </c>
+      <c r="E9" s="4">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="7">
+      <c r="B10" s="7">
         <v>1</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C10" s="7">
         <v>1</v>
       </c>
-      <c r="D9" s="4">
-        <v>1143</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5">
-      <c r="A11" s="2" t="s">
+      <c r="D10" s="4">
+        <v>1189</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="E13" s="3" t="s">
         <v>87</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5">
-      <c r="A13" t="s">
-        <v>73</v>
-      </c>
-      <c r="B13" s="6">
-        <v>0.1015358361774744</v>
-      </c>
-      <c r="C13" s="6">
-        <v>0.112</v>
-      </c>
-      <c r="D13" s="4">
-        <v>119</v>
-      </c>
-      <c r="E13" s="4">
-        <v>144</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>55</v>
+        <v>74</v>
       </c>
       <c r="B14" s="6">
-        <v>0.2175767918088737</v>
+        <v>0.1216442953020134</v>
       </c>
       <c r="C14" s="6">
-        <v>0.237</v>
+        <v>0.122</v>
       </c>
       <c r="D14" s="4">
-        <v>255</v>
+        <v>145</v>
       </c>
       <c r="E14" s="4">
-        <v>309</v>
+        <v>177</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B15" s="6">
-        <v>0.3191126279863481</v>
+        <v>0.2441275167785235</v>
       </c>
       <c r="C15" s="6">
-        <v>0.305</v>
+        <v>0.244</v>
       </c>
       <c r="D15" s="4">
-        <v>374</v>
+        <v>291</v>
       </c>
       <c r="E15" s="4">
-        <v>451</v>
+        <v>352</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B16" s="6">
-        <v>0.1877133105802048</v>
+        <v>0.3070469798657718</v>
       </c>
       <c r="C16" s="6">
-        <v>0.181</v>
+        <v>0.305</v>
       </c>
       <c r="D16" s="4">
-        <v>220</v>
+        <v>366</v>
       </c>
       <c r="E16" s="4">
-        <v>266</v>
+        <v>441</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
+        <v>57</v>
+      </c>
+      <c r="B17" s="6">
+        <v>0.1753355704697987</v>
+      </c>
+      <c r="C17" s="6">
+        <v>0.176</v>
+      </c>
+      <c r="D17" s="4">
+        <v>209</v>
+      </c>
+      <c r="E17" s="4">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" t="s">
         <v>58</v>
       </c>
-      <c r="B17" s="6">
-        <v>0.174061433447099</v>
-      </c>
-      <c r="C17" s="6">
-        <v>0.165</v>
-      </c>
-      <c r="D17" s="4">
-        <v>204</v>
-      </c>
-      <c r="E17" s="4">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5">
-      <c r="A18" s="5" t="s">
+      <c r="B18" s="6">
+        <v>0.1518456375838926</v>
+      </c>
+      <c r="C18" s="6">
+        <v>0.153</v>
+      </c>
+      <c r="D18" s="4">
+        <v>181</v>
+      </c>
+      <c r="E18" s="4">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="7">
+      <c r="B19" s="7">
         <v>1</v>
       </c>
-      <c r="C18" s="7">
+      <c r="C19" s="7">
         <v>1</v>
       </c>
-      <c r="D18" s="4">
-        <v>1172</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5">
-      <c r="A20" s="2" t="s">
-        <v>88</v>
+      <c r="D19" s="4">
+        <v>1192</v>
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="B21" s="3" t="s">
+      <c r="A21" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B22" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C22" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D21" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="E21" s="3" t="s">
+      <c r="D22" s="3" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="22" spans="1:5">
-      <c r="A22" t="s">
-        <v>75</v>
-      </c>
-      <c r="B22" s="6">
-        <v>0.09572649572649573</v>
-      </c>
-      <c r="C22" s="6">
-        <v>0.095</v>
-      </c>
-      <c r="D22" s="4">
-        <v>56</v>
-      </c>
-      <c r="E22" s="4">
-        <v>69</v>
+      <c r="E22" s="3" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -3007,16 +3049,16 @@
         <v>76</v>
       </c>
       <c r="B23" s="6">
-        <v>0.135042735042735</v>
+        <v>0.09914529914529914</v>
       </c>
       <c r="C23" s="6">
-        <v>0.139</v>
+        <v>0.09300000000000001</v>
       </c>
       <c r="D23" s="4">
-        <v>79</v>
+        <v>58</v>
       </c>
       <c r="E23" s="4">
-        <v>96</v>
+        <v>71</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -3024,16 +3066,16 @@
         <v>77</v>
       </c>
       <c r="B24" s="6">
-        <v>0.105982905982906</v>
+        <v>0.1282051282051282</v>
       </c>
       <c r="C24" s="6">
-        <v>0.101</v>
+        <v>0.131</v>
       </c>
       <c r="D24" s="4">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="E24" s="4">
-        <v>76</v>
+        <v>92</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -3041,16 +3083,16 @@
         <v>78</v>
       </c>
       <c r="B25" s="6">
-        <v>0.1931623931623932</v>
+        <v>0.1025641025641026</v>
       </c>
       <c r="C25" s="6">
-        <v>0.202</v>
+        <v>0.115</v>
       </c>
       <c r="D25" s="4">
-        <v>113</v>
+        <v>60</v>
       </c>
       <c r="E25" s="4">
-        <v>137</v>
+        <v>73</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -3058,16 +3100,16 @@
         <v>79</v>
       </c>
       <c r="B26" s="6">
-        <v>0.2153846153846154</v>
+        <v>0.2102564102564103</v>
       </c>
       <c r="C26" s="6">
-        <v>0.22</v>
+        <v>0.198</v>
       </c>
       <c r="D26" s="4">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="E26" s="4">
-        <v>153</v>
+        <v>149</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -3075,16 +3117,16 @@
         <v>80</v>
       </c>
       <c r="B27" s="6">
-        <v>0.2478632478632479</v>
+        <v>0.2170940170940171</v>
       </c>
       <c r="C27" s="6">
-        <v>0.244</v>
+        <v>0.215</v>
       </c>
       <c r="D27" s="4">
-        <v>145</v>
+        <v>127</v>
       </c>
       <c r="E27" s="4">
-        <v>177</v>
+        <v>155</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -3092,29 +3134,46 @@
         <v>81</v>
       </c>
       <c r="B28" s="6">
-        <v>0.006837606837606838</v>
+        <v>0.2393162393162393</v>
       </c>
       <c r="C28" s="6">
+        <v>0.248</v>
+      </c>
+      <c r="D28" s="4">
+        <v>140</v>
+      </c>
+      <c r="E28" s="4">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" t="s">
+        <v>82</v>
+      </c>
+      <c r="B29" s="6">
+        <v>0.003418803418803419</v>
+      </c>
+      <c r="C29" s="6">
         <v>0</v>
       </c>
-      <c r="D28" s="4">
+      <c r="D29" s="4">
+        <v>2</v>
+      </c>
+      <c r="E29" s="4">
         <v>4</v>
       </c>
-      <c r="E28" s="4">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5">
-      <c r="A29" s="5" t="s">
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B29" s="7">
+      <c r="B30" s="7">
         <v>1</v>
       </c>
-      <c r="C29" s="7">
+      <c r="C30" s="7">
         <v>1</v>
       </c>
-      <c r="D29" s="4">
+      <c r="D30" s="4">
         <v>585</v>
       </c>
     </row>
@@ -3130,12 +3189,12 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -3143,22 +3202,22 @@
         <v>35</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -3166,45 +3225,45 @@
         <v>40</v>
       </c>
       <c r="B6" s="4">
-        <v>769</v>
+        <v>794</v>
       </c>
       <c r="C6" s="8">
-        <v>200.52</v>
+        <v>210.46</v>
       </c>
       <c r="D6" s="8">
-        <v>117.07</v>
+        <v>107.2</v>
       </c>
       <c r="E6" s="8">
-        <v>317.59</v>
+        <v>317.66</v>
       </c>
       <c r="F6" s="8">
         <v>317.76</v>
       </c>
       <c r="G6" s="8">
-        <v>0.17</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B7" s="4">
-        <v>649</v>
+        <v>708</v>
       </c>
       <c r="C7" s="8">
-        <v>176.95</v>
+        <v>185.68</v>
       </c>
       <c r="D7" s="8">
-        <v>103.32</v>
+        <v>94.61</v>
       </c>
       <c r="E7" s="8">
-        <v>280.27</v>
+        <v>280.29</v>
       </c>
       <c r="F7" s="8">
         <v>280.44</v>
       </c>
       <c r="G7" s="8">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -3212,45 +3271,45 @@
         <v>41</v>
       </c>
       <c r="B8" s="4">
-        <v>623</v>
+        <v>619</v>
       </c>
       <c r="C8" s="8">
-        <v>168.71</v>
+        <v>168.84</v>
       </c>
       <c r="D8" s="8">
         <v>0</v>
       </c>
       <c r="E8" s="8">
-        <v>168.71</v>
+        <v>168.84</v>
       </c>
       <c r="F8" s="8">
         <v>168.89</v>
       </c>
       <c r="G8" s="8">
-        <v>0.18</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B9" s="4">
-        <v>629</v>
+        <v>619</v>
       </c>
       <c r="C9" s="8">
-        <v>159.74</v>
+        <v>159.75</v>
       </c>
       <c r="D9" s="8">
         <v>0</v>
       </c>
       <c r="E9" s="8">
-        <v>159.74</v>
+        <v>159.75</v>
       </c>
       <c r="F9" s="8">
         <v>159.91</v>
       </c>
       <c r="G9" s="8">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -3258,22 +3317,22 @@
         <v>43</v>
       </c>
       <c r="B10" s="4">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="C10" s="8">
-        <v>58.68</v>
+        <v>58.67</v>
       </c>
       <c r="D10" s="8">
         <v>0</v>
       </c>
       <c r="E10" s="8">
-        <v>58.68</v>
+        <v>58.67</v>
       </c>
       <c r="F10" s="8">
         <v>58.84</v>
       </c>
       <c r="G10" s="8">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -3281,26 +3340,26 @@
         <v>32</v>
       </c>
       <c r="B11" s="4">
-        <v>2900</v>
+        <v>2966</v>
       </c>
       <c r="E11" s="8">
-        <v>984.99</v>
+        <v>985.21</v>
       </c>
       <c r="F11" s="8">
         <v>985.84</v>
       </c>
       <c r="G11" s="8">
-        <v>0.85</v>
+        <v>0.63</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -3308,7 +3367,7 @@
         <v>26</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -3347,24 +3406,24 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>30</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -3372,33 +3431,33 @@
         <v>40</v>
       </c>
       <c r="B4">
-        <v>901</v>
+        <v>823</v>
       </c>
       <c r="C4">
-        <v>445</v>
+        <v>420</v>
       </c>
       <c r="D4">
-        <v>456</v>
+        <v>403</v>
       </c>
       <c r="E4">
-        <v>117.07</v>
+        <v>107.2</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B5">
-        <v>796</v>
+        <v>727</v>
       </c>
       <c r="C5">
-        <v>393</v>
+        <v>371</v>
       </c>
       <c r="D5">
-        <v>403</v>
+        <v>356</v>
       </c>
       <c r="E5">
-        <v>103.32</v>
+        <v>94.61</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -3406,10 +3465,10 @@
         <v>32</v>
       </c>
       <c r="B6" s="4">
-        <v>1697</v>
+        <v>1550</v>
       </c>
       <c r="E6" s="8">
-        <v>220.4</v>
+        <v>201.81</v>
       </c>
     </row>
   </sheetData>
@@ -3424,72 +3483,72 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B5" s="8">
         <v>361.2</v>
       </c>
       <c r="C5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B6" s="8">
         <v>125.1</v>
       </c>
       <c r="C6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B7" s="8">
         <v>157</v>
       </c>
       <c r="C7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B8" s="8">
         <v>62.8</v>
       </c>
       <c r="C8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B9" s="8">
         <v>706.1</v>
@@ -3497,67 +3556,67 @@
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B13" s="8">
         <v>157</v>
       </c>
       <c r="C13" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B14" s="8">
         <v>94.2</v>
       </c>
       <c r="C14" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B15" s="8">
         <v>65.59999999999999</v>
       </c>
       <c r="C15" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B16" s="8">
         <v>65.5</v>
       </c>
       <c r="C16" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B17" s="8">
         <v>382.3</v>
@@ -3565,7 +3624,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B19" s="8">
         <v>1088.4</v>
@@ -3583,7 +3642,7 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -3593,7 +3652,7 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>55</v>
@@ -3609,6 +3668,9 @@
       </c>
       <c r="F4" s="3" t="s">
         <v>59</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -3616,19 +3678,22 @@
         <v>40</v>
       </c>
       <c r="B5">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C5">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="D5">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="E5">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="F5">
-        <v>262</v>
+        <v>21</v>
+      </c>
+      <c r="G5">
+        <v>322</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -3636,19 +3701,22 @@
         <v>41</v>
       </c>
       <c r="B6">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C6">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D6">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E6">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="F6">
-        <v>282</v>
+        <v>11</v>
+      </c>
+      <c r="G6">
+        <v>283</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -3656,19 +3724,22 @@
         <v>42</v>
       </c>
       <c r="B7">
-        <v>25</v>
+        <v>46</v>
       </c>
       <c r="C7">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="D7">
-        <v>71</v>
+        <v>94</v>
       </c>
       <c r="E7">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="F7">
-        <v>201</v>
+        <v>4</v>
+      </c>
+      <c r="G7">
+        <v>275</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -3679,16 +3750,19 @@
         <v>9</v>
       </c>
       <c r="C8">
+        <v>25</v>
+      </c>
+      <c r="D8">
         <v>26</v>
       </c>
-      <c r="D8">
-        <v>25</v>
-      </c>
       <c r="E8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F8">
-        <v>74</v>
+        <v>13</v>
+      </c>
+      <c r="G8">
+        <v>86</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -3696,19 +3770,22 @@
         <v>44</v>
       </c>
       <c r="B9">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="C9">
-        <v>112</v>
+        <v>66</v>
       </c>
       <c r="D9">
-        <v>123</v>
+        <v>64</v>
       </c>
       <c r="E9">
-        <v>58</v>
+        <v>35</v>
       </c>
       <c r="F9">
-        <v>324</v>
+        <v>35</v>
+      </c>
+      <c r="G9">
+        <v>223</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -3718,10 +3795,10 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>55</v>
@@ -3736,7 +3813,7 @@
         <v>58</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -3744,22 +3821,22 @@
         <v>40</v>
       </c>
       <c r="B13">
+        <v>53</v>
+      </c>
+      <c r="C13">
+        <v>83</v>
+      </c>
+      <c r="D13">
+        <v>99</v>
+      </c>
+      <c r="E13">
         <v>50</v>
       </c>
-      <c r="C13">
-        <v>84</v>
-      </c>
-      <c r="D13">
-        <v>100</v>
-      </c>
-      <c r="E13">
-        <v>54</v>
-      </c>
       <c r="F13">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="G13">
-        <v>346</v>
+        <v>334</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -3767,91 +3844,91 @@
         <v>41</v>
       </c>
       <c r="B14">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="C14">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="D14">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="E14">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="F14">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G14">
-        <v>303</v>
+        <v>334</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B15">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="C15">
-        <v>17</v>
+        <v>67</v>
       </c>
       <c r="D15">
-        <v>21</v>
+        <v>77</v>
       </c>
       <c r="E15">
-        <v>15</v>
+        <v>48</v>
       </c>
       <c r="F15">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="G15">
-        <v>72</v>
+        <v>264</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B16">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C16">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="D16">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E16">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="F16">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G16">
-        <v>176</v>
+        <v>191</v>
       </c>
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B17">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="C17">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="D17">
-        <v>92</v>
+        <v>20</v>
       </c>
       <c r="E17">
-        <v>63</v>
+        <v>14</v>
       </c>
       <c r="F17">
-        <v>56</v>
+        <v>11</v>
       </c>
       <c r="G17">
-        <v>275</v>
+        <v>69</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -3861,60 +3938,60 @@
     </row>
     <row r="20" spans="1:9">
       <c r="A20" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B21">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C21">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="D21">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="E21">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="F21">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="G21">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="H21">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I21">
-        <v>252</v>
+        <v>205</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -3922,28 +3999,28 @@
         <v>43</v>
       </c>
       <c r="B22">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C22">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D22">
         <v>11</v>
       </c>
       <c r="E22">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F22">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="G22">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="H22">
         <v>0</v>
       </c>
       <c r="I22">
-        <v>84</v>
+        <v>71</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -3951,86 +4028,86 @@
         <v>40</v>
       </c>
       <c r="B23">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="C23">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="D23">
         <v>15</v>
       </c>
       <c r="E23">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F23">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="G23">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H23">
         <v>0</v>
       </c>
       <c r="I23">
-        <v>161</v>
+        <v>138</v>
       </c>
     </row>
     <row r="24" spans="1:9">
       <c r="A24" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B24">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="C24">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="D24">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="E24">
-        <v>8</v>
+        <v>45</v>
       </c>
       <c r="F24">
-        <v>8</v>
+        <v>36</v>
       </c>
       <c r="G24">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="H24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I24">
-        <v>38</v>
+        <v>169</v>
       </c>
     </row>
     <row r="25" spans="1:9">
       <c r="A25" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B25">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C25">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D25">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E25">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F25">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="G25">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="H25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I25">
-        <v>50</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Explore Pants: CAB/DAMA manual, KIDS con Kaki sin talla 14, hoja Tela Explore
Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/EXPLORE_PANTS_Proyeccion_Produccion.xlsx
+++ b/EXPLORE_PANTS_Proyeccion_Produccion.xlsx
@@ -14,16 +14,17 @@
     <sheet name="Producción por Talla" sheetId="5" r:id="rId5"/>
     <sheet name="Verificación Tela" sheetId="6" r:id="rId6"/>
     <sheet name="Shorts R1" sheetId="7" r:id="rId7"/>
-    <sheet name="Compra en 2 Órdenes" sheetId="8" r:id="rId8"/>
-    <sheet name="Producción Color × Talla" sheetId="9" r:id="rId9"/>
-    <sheet name="Metodología" sheetId="10" r:id="rId10"/>
+    <sheet name="Tela Explore Pants" sheetId="8" r:id="rId8"/>
+    <sheet name="Compra en 2 Órdenes" sheetId="9" r:id="rId9"/>
+    <sheet name="Producción Color × Talla" sheetId="10" r:id="rId10"/>
+    <sheet name="Metodología" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="151">
   <si>
     <t>EXPLORE PANTS — PROYECCIÓN ANCLADA A JUSTIFICACIÓN NOVAKTEX</t>
   </si>
@@ -55,7 +56,7 @@
     <t>KIDS 550–620 und · CAB sin 3XL · DAMA sin 2XL</t>
   </si>
   <si>
-    <t>KIDS Gris/Azul: presencia en todas las tallas (curva dashboard)</t>
+    <t>KIDS: tallas 2–12 (sin 14) · incluye Kaki · CAB/DAMA manual</t>
   </si>
   <si>
     <t>Consumo referencial: CAB 0.3 · DAMA 0.25 · KIDS 0.22 kg/und</t>
@@ -271,9 +272,6 @@
     <t>12</t>
   </si>
   <si>
-    <t>14</t>
-  </si>
-  <si>
     <t>EXPLORE PANTS — CURVA DE TALLA POR GÉNERO (vs dashboard)</t>
   </si>
   <si>
@@ -343,6 +341,39 @@
     <t>Kg tela</t>
   </si>
   <si>
+    <t>USO DE TELA — SOLO EXPLORE PANTS (sin Shorts R1)</t>
+  </si>
+  <si>
+    <t>Consumo ref.: CAB 0.3 · DAMA 0.25 · KIDS 0.22 kg/und · presupuesto = existencia − shorts</t>
+  </si>
+  <si>
+    <t>Und CAB</t>
+  </si>
+  <si>
+    <t>Und DAMA</t>
+  </si>
+  <si>
+    <t>Und KIDS</t>
+  </si>
+  <si>
+    <t>Und total</t>
+  </si>
+  <si>
+    <t>Kg CAB</t>
+  </si>
+  <si>
+    <t>Kg DAMA</t>
+  </si>
+  <si>
+    <t>Kg KIDS</t>
+  </si>
+  <si>
+    <t>Kg presup.</t>
+  </si>
+  <si>
+    <t>Delta kg</t>
+  </si>
+  <si>
     <t>PROPUESTA COMPRA 65% AHORA / 35% SEPTIEMBRE (archivo justificación)</t>
   </si>
   <si>
@@ -430,7 +461,10 @@
     <t>4. COLOR: ranking ventas por género; si CAB Negro queda bajo vs Gris es por kg Negro/Gris en Shorts R1 + consumo de existencia Gris (no por mezcla de compra).</t>
   </si>
   <si>
-    <t>5. KIDS Gris/Azul: presencia 2–14 con curva talla dashboard; Gris piso ~48 und. CAB sin 3XL · DAMA sin 2XL.</t>
+    <t>5. KIDS: tallas 2–12 (sin 14), incluye Kaki; Gris/Azul curva dashboard. CAB/DAMA: matriz manual (Kaki recortable para cuadrar tela).</t>
+  </si>
+  <si>
+    <t>CAB sin 3XL · DAMA sin 2XL.</t>
   </si>
   <si>
     <t>6. Shorts R1: CAB 0.14 · DAMA 0.12 kg/und.</t>
@@ -1039,10 +1073,10 @@
         <v>30</v>
       </c>
       <c r="B32">
-        <v>1192</v>
+        <v>1186</v>
       </c>
       <c r="C32">
-        <v>1442</v>
+        <v>1433</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -1053,7 +1087,7 @@
         <v>585</v>
       </c>
       <c r="C33">
-        <v>714</v>
+        <v>710</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -1061,10 +1095,10 @@
         <v>32</v>
       </c>
       <c r="B34" s="5">
-        <v>2966</v>
+        <v>2960</v>
       </c>
       <c r="C34" s="5">
-        <v>3593</v>
+        <v>3580</v>
       </c>
     </row>
   </sheetData>
@@ -1077,7 +1111,443 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:H24"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5">
+        <v>41</v>
+      </c>
+      <c r="C5">
+        <v>102</v>
+      </c>
+      <c r="D5">
+        <v>103</v>
+      </c>
+      <c r="E5">
+        <v>60</v>
+      </c>
+      <c r="F5">
+        <v>16</v>
+      </c>
+      <c r="G5">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B6">
+        <v>44</v>
+      </c>
+      <c r="C6">
+        <v>92</v>
+      </c>
+      <c r="D6">
+        <v>85</v>
+      </c>
+      <c r="E6">
+        <v>51</v>
+      </c>
+      <c r="F6">
+        <v>11</v>
+      </c>
+      <c r="G6">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7">
+        <v>46</v>
+      </c>
+      <c r="C7">
+        <v>87</v>
+      </c>
+      <c r="D7">
+        <v>94</v>
+      </c>
+      <c r="E7">
+        <v>44</v>
+      </c>
+      <c r="F7">
+        <v>4</v>
+      </c>
+      <c r="G7">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8">
+        <v>9</v>
+      </c>
+      <c r="C8">
+        <v>25</v>
+      </c>
+      <c r="D8">
+        <v>26</v>
+      </c>
+      <c r="E8">
+        <v>13</v>
+      </c>
+      <c r="F8">
+        <v>13</v>
+      </c>
+      <c r="G8">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9">
+        <v>23</v>
+      </c>
+      <c r="C9">
+        <v>66</v>
+      </c>
+      <c r="D9">
+        <v>64</v>
+      </c>
+      <c r="E9">
+        <v>35</v>
+      </c>
+      <c r="F9">
+        <v>35</v>
+      </c>
+      <c r="G9">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13">
+        <v>45</v>
+      </c>
+      <c r="C13">
+        <v>83</v>
+      </c>
+      <c r="D13">
+        <v>94</v>
+      </c>
+      <c r="E13">
+        <v>55</v>
+      </c>
+      <c r="F13">
+        <v>51</v>
+      </c>
+      <c r="G13">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
+        <v>41</v>
+      </c>
+      <c r="B14">
+        <v>38</v>
+      </c>
+      <c r="C14">
+        <v>86</v>
+      </c>
+      <c r="D14">
+        <v>104</v>
+      </c>
+      <c r="E14">
+        <v>63</v>
+      </c>
+      <c r="F14">
+        <v>43</v>
+      </c>
+      <c r="G14">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15">
+        <v>31</v>
+      </c>
+      <c r="C15">
+        <v>67</v>
+      </c>
+      <c r="D15">
+        <v>77</v>
+      </c>
+      <c r="E15">
+        <v>48</v>
+      </c>
+      <c r="F15">
+        <v>41</v>
+      </c>
+      <c r="G15">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16">
+        <v>23</v>
+      </c>
+      <c r="C16">
+        <v>38</v>
+      </c>
+      <c r="D16">
+        <v>66</v>
+      </c>
+      <c r="E16">
+        <v>30</v>
+      </c>
+      <c r="F16">
+        <v>34</v>
+      </c>
+      <c r="G16">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="A17" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17">
+        <v>10</v>
+      </c>
+      <c r="C17">
+        <v>16</v>
+      </c>
+      <c r="D17">
+        <v>19</v>
+      </c>
+      <c r="E17">
+        <v>14</v>
+      </c>
+      <c r="F17">
+        <v>10</v>
+      </c>
+      <c r="G17">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
+      <c r="A19" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
+      <c r="A21" t="s">
+        <v>44</v>
+      </c>
+      <c r="B21">
+        <v>16</v>
+      </c>
+      <c r="C21">
+        <v>28</v>
+      </c>
+      <c r="D21">
+        <v>20</v>
+      </c>
+      <c r="E21">
+        <v>38</v>
+      </c>
+      <c r="F21">
+        <v>44</v>
+      </c>
+      <c r="G21">
+        <v>59</v>
+      </c>
+      <c r="H21">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22" t="s">
+        <v>43</v>
+      </c>
+      <c r="B22">
+        <v>5</v>
+      </c>
+      <c r="C22">
+        <v>8</v>
+      </c>
+      <c r="D22">
+        <v>11</v>
+      </c>
+      <c r="E22">
+        <v>14</v>
+      </c>
+      <c r="F22">
+        <v>14</v>
+      </c>
+      <c r="G22">
+        <v>19</v>
+      </c>
+      <c r="H22">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" t="s">
+        <v>40</v>
+      </c>
+      <c r="B23">
+        <v>20</v>
+      </c>
+      <c r="C23">
+        <v>19</v>
+      </c>
+      <c r="D23">
+        <v>16</v>
+      </c>
+      <c r="E23">
+        <v>27</v>
+      </c>
+      <c r="F23">
+        <v>34</v>
+      </c>
+      <c r="G23">
+        <v>29</v>
+      </c>
+      <c r="H23">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
+      <c r="A24" t="s">
+        <v>42</v>
+      </c>
+      <c r="B24">
+        <v>17</v>
+      </c>
+      <c r="C24">
+        <v>21</v>
+      </c>
+      <c r="D24">
+        <v>14</v>
+      </c>
+      <c r="E24">
+        <v>44</v>
+      </c>
+      <c r="F24">
+        <v>35</v>
+      </c>
+      <c r="G24">
+        <v>33</v>
+      </c>
+      <c r="H24">
+        <v>164</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:A12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="100.7109375" customWidth="1"/>
@@ -1085,52 +1555,57 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>132</v>
+        <v>142</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" t="s">
-        <v>139</v>
+        <v>149</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1">
+      <c r="A12" t="s">
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -1140,7 +1615,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1317,13 +1792,13 @@
         <v>40</v>
       </c>
       <c r="C14" s="4">
-        <v>334</v>
+        <v>328</v>
       </c>
       <c r="D14" s="4">
-        <v>402</v>
+        <v>395</v>
       </c>
       <c r="E14" s="6">
-        <v>0.2802013422818792</v>
+        <v>0.2765598650927487</v>
       </c>
       <c r="F14" s="6">
         <v>0.298</v>
@@ -1343,7 +1818,7 @@
         <v>403</v>
       </c>
       <c r="E15" s="6">
-        <v>0.2802013422818792</v>
+        <v>0.2816188870151771</v>
       </c>
       <c r="F15" s="6">
         <v>0.223</v>
@@ -1363,7 +1838,7 @@
         <v>320</v>
       </c>
       <c r="E16" s="6">
-        <v>0.2214765100671141</v>
+        <v>0.2225969645868466</v>
       </c>
       <c r="F16" s="6">
         <v>0.198</v>
@@ -1380,10 +1855,10 @@
         <v>191</v>
       </c>
       <c r="D17" s="4">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E17" s="6">
-        <v>0.1602348993288591</v>
+        <v>0.1610455311973019</v>
       </c>
       <c r="F17" s="6">
         <v>0.145</v>
@@ -1400,10 +1875,10 @@
         <v>69</v>
       </c>
       <c r="D18" s="4">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E18" s="6">
-        <v>0.05788590604026846</v>
+        <v>0.0581787521079258</v>
       </c>
       <c r="F18" s="6">
         <v>0.136</v>
@@ -1414,7 +1889,7 @@
         <v>32</v>
       </c>
       <c r="B19" s="4">
-        <v>1192</v>
+        <v>1186</v>
       </c>
       <c r="C19" s="7">
         <v>1</v>
@@ -1456,7 +1931,7 @@
         <v>205</v>
       </c>
       <c r="D23" s="4">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E23" s="6">
         <v>0.3504273504273504</v>
@@ -1493,13 +1968,13 @@
         <v>40</v>
       </c>
       <c r="C25" s="4">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="D25" s="4">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="E25" s="6">
-        <v>0.2358974358974359</v>
+        <v>0.2478632478632479</v>
       </c>
       <c r="F25" s="6">
         <v>0.225</v>
@@ -1513,46 +1988,26 @@
         <v>42</v>
       </c>
       <c r="C26" s="4">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="D26" s="4">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="E26" s="6">
-        <v>0.2888888888888889</v>
+        <v>0.2803418803418803</v>
       </c>
       <c r="F26" s="6">
         <v>0.154</v>
       </c>
     </row>
     <row r="27" spans="1:6">
-      <c r="A27">
-        <v>5</v>
-      </c>
-      <c r="B27" t="s">
-        <v>41</v>
-      </c>
-      <c r="C27" s="4">
-        <v>2</v>
-      </c>
-      <c r="D27" s="4">
-        <v>4</v>
-      </c>
-      <c r="E27" s="6">
-        <v>0.003418803418803419</v>
-      </c>
-      <c r="F27" s="6">
-        <v>0.08400000000000001</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6">
-      <c r="A28" s="5" t="s">
+      <c r="A27" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B28" s="4">
+      <c r="B27" s="4">
         <v>585</v>
       </c>
-      <c r="C28" s="7">
+      <c r="C27" s="7">
         <v>1</v>
       </c>
     </row>
@@ -1593,10 +2048,10 @@
         <v>40</v>
       </c>
       <c r="B4" s="4">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="C4" s="6">
-        <v>0.2677006068779501</v>
+        <v>0.2685810810810811</v>
       </c>
       <c r="D4" s="6">
         <v>0.3223210782341178</v>
@@ -1610,10 +2065,10 @@
         <v>42</v>
       </c>
       <c r="B5" s="4">
-        <v>708</v>
+        <v>703</v>
       </c>
       <c r="C5" s="6">
-        <v>0.2387053270397842</v>
+        <v>0.2375</v>
       </c>
       <c r="D5" s="6">
         <v>0.2844671001033621</v>
@@ -1627,10 +2082,10 @@
         <v>41</v>
       </c>
       <c r="B6" s="4">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="C6" s="6">
-        <v>0.2086985839514498</v>
+        <v>0.208445945945946</v>
       </c>
       <c r="D6" s="6">
         <v>0.1713177091328877</v>
@@ -1647,7 +2102,7 @@
         <v>619</v>
       </c>
       <c r="C7" s="6">
-        <v>0.2086985839514498</v>
+        <v>0.2091216216216216</v>
       </c>
       <c r="D7" s="6">
         <v>0.1622064538507951</v>
@@ -1664,7 +2119,7 @@
         <v>226</v>
       </c>
       <c r="C8" s="6">
-        <v>0.07619689817936615</v>
+        <v>0.07635135135135135</v>
       </c>
       <c r="D8" s="6">
         <v>0.05968765867883735</v>
@@ -1678,7 +2133,7 @@
         <v>32</v>
       </c>
       <c r="B9" s="4">
-        <v>2966</v>
+        <v>2960</v>
       </c>
       <c r="C9" s="7">
         <v>1</v>
@@ -1697,7 +2152,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -1738,13 +2193,13 @@
         <v>30</v>
       </c>
       <c r="B5">
-        <v>1192</v>
+        <v>1186</v>
       </c>
       <c r="C5">
-        <v>1442</v>
+        <v>1433</v>
       </c>
       <c r="D5">
-        <v>250</v>
+        <v>247</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -1755,10 +2210,10 @@
         <v>585</v>
       </c>
       <c r="C6">
-        <v>714</v>
+        <v>710</v>
       </c>
       <c r="D6">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -1766,13 +2221,13 @@
         <v>32</v>
       </c>
       <c r="B7" s="5">
-        <v>2966</v>
+        <v>2960</v>
       </c>
       <c r="C7" s="5">
-        <v>3593</v>
+        <v>3580</v>
       </c>
       <c r="D7" s="5">
-        <v>627</v>
+        <v>620</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -1817,10 +2272,10 @@
         <v>103</v>
       </c>
       <c r="E12">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="F12">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="G12">
         <v>322</v>
@@ -1840,10 +2295,10 @@
         <v>124</v>
       </c>
       <c r="E13">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F13">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="G13">
         <v>389</v>
@@ -2047,10 +2502,10 @@
         <v>372</v>
       </c>
       <c r="E22" s="5">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="F22" s="5">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="G22" s="5">
         <v>1189</v>
@@ -2070,10 +2525,10 @@
         <v>448</v>
       </c>
       <c r="E23" s="5">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="F23" s="5">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="G23" s="5">
         <v>1437</v>
@@ -2112,22 +2567,22 @@
         <v>61</v>
       </c>
       <c r="B27">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="C27">
         <v>83</v>
       </c>
       <c r="D27">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="E27">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F27">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G27">
-        <v>334</v>
+        <v>328</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -2135,22 +2590,22 @@
         <v>62</v>
       </c>
       <c r="B28">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="C28">
         <v>100</v>
       </c>
       <c r="D28">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="E28">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="F28">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G28">
-        <v>402</v>
+        <v>395</v>
       </c>
     </row>
     <row r="29" spans="1:7">
@@ -2245,12 +2700,12 @@
         <v>320</v>
       </c>
     </row>
-    <row r="33" spans="1:9">
+    <row r="33" spans="1:8">
       <c r="A33" t="s">
         <v>69</v>
       </c>
       <c r="B33">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C33">
         <v>38</v>
@@ -2259,21 +2714,21 @@
         <v>66</v>
       </c>
       <c r="E33">
+        <v>30</v>
+      </c>
+      <c r="F33">
         <v>34</v>
-      </c>
-      <c r="F33">
-        <v>37</v>
       </c>
       <c r="G33">
         <v>191</v>
       </c>
     </row>
-    <row r="34" spans="1:9">
+    <row r="34" spans="1:8">
       <c r="A34" t="s">
         <v>70</v>
       </c>
       <c r="B34">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C34">
         <v>46</v>
@@ -2282,113 +2737,113 @@
         <v>80</v>
       </c>
       <c r="E34">
+        <v>36</v>
+      </c>
+      <c r="F34">
         <v>41</v>
       </c>
-      <c r="F34">
-        <v>45</v>
-      </c>
       <c r="G34">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8">
       <c r="A35" t="s">
         <v>67</v>
       </c>
       <c r="B35">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C35">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D35">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E35">
         <v>14</v>
       </c>
       <c r="F35">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G35">
         <v>69</v>
       </c>
     </row>
-    <row r="36" spans="1:9">
+    <row r="36" spans="1:8">
       <c r="A36" t="s">
         <v>68</v>
       </c>
       <c r="B36">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C36">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D36">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E36">
         <v>17</v>
       </c>
       <c r="F36">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G36">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
       <c r="A37" s="5" t="s">
         <v>71</v>
       </c>
       <c r="B37" s="5">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C37" s="5">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D37" s="5">
-        <v>366</v>
+        <v>360</v>
       </c>
       <c r="E37" s="5">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F37" s="5">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G37" s="5">
-        <v>1192</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9">
+        <v>1186</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
       <c r="A38" s="5" t="s">
         <v>72</v>
       </c>
       <c r="B38" s="5">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C38" s="5">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="D38" s="5">
-        <v>441</v>
+        <v>434</v>
       </c>
       <c r="E38" s="5">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F38" s="5">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="G38" s="5">
-        <v>1442</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9">
+        <v>1433</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
       <c r="A40" s="2" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="41" spans="1:9">
+    <row r="41" spans="1:8">
       <c r="A41" s="3" t="s">
         <v>35</v>
       </c>
@@ -2411,13 +2866,10 @@
         <v>81</v>
       </c>
       <c r="H41" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="I41" s="3" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="42" spans="1:9">
+    <row r="42" spans="1:8">
       <c r="A42" t="s">
         <v>69</v>
       </c>
@@ -2437,16 +2889,13 @@
         <v>44</v>
       </c>
       <c r="G42">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H42">
-        <v>1</v>
-      </c>
-      <c r="I42">
         <v>205</v>
       </c>
     </row>
-    <row r="43" spans="1:9">
+    <row r="43" spans="1:8">
       <c r="A43" t="s">
         <v>70</v>
       </c>
@@ -2466,16 +2915,13 @@
         <v>53</v>
       </c>
       <c r="G43">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H43">
-        <v>2</v>
-      </c>
-      <c r="I43">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8">
       <c r="A44" t="s">
         <v>67</v>
       </c>
@@ -2498,13 +2944,10 @@
         <v>19</v>
       </c>
       <c r="H44">
-        <v>0</v>
-      </c>
-      <c r="I44">
         <v>71</v>
       </c>
     </row>
-    <row r="45" spans="1:9">
+    <row r="45" spans="1:8">
       <c r="A45" t="s">
         <v>68</v>
       </c>
@@ -2527,76 +2970,67 @@
         <v>23</v>
       </c>
       <c r="H45">
-        <v>0</v>
-      </c>
-      <c r="I45">
         <v>87</v>
       </c>
     </row>
-    <row r="46" spans="1:9">
+    <row r="46" spans="1:8">
       <c r="A46" t="s">
         <v>61</v>
       </c>
       <c r="B46">
+        <v>20</v>
+      </c>
+      <c r="C46">
         <v>19</v>
       </c>
-      <c r="C46">
-        <v>18</v>
-      </c>
       <c r="D46">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E46">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F46">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G46">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H46">
-        <v>0</v>
-      </c>
-      <c r="I46">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8">
       <c r="A47" t="s">
         <v>62</v>
       </c>
       <c r="B47">
+        <v>24</v>
+      </c>
+      <c r="C47">
         <v>23</v>
       </c>
-      <c r="C47">
-        <v>22</v>
-      </c>
       <c r="D47">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E47">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F47">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G47">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H47">
-        <v>0</v>
-      </c>
-      <c r="I47">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8">
       <c r="A48" t="s">
         <v>65</v>
       </c>
       <c r="B48">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C48">
         <v>21</v>
@@ -2605,27 +3039,24 @@
         <v>14</v>
       </c>
       <c r="E48">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F48">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G48">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H48">
-        <v>1</v>
-      </c>
-      <c r="I48">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8">
       <c r="A49" t="s">
         <v>66</v>
       </c>
       <c r="B49">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C49">
         <v>26</v>
@@ -2634,135 +3065,68 @@
         <v>17</v>
       </c>
       <c r="E49">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F49">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="G49">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H49">
-        <v>2</v>
-      </c>
-      <c r="I49">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9">
-      <c r="A50" t="s">
-        <v>63</v>
-      </c>
-      <c r="B50">
-        <v>0</v>
-      </c>
-      <c r="C50">
-        <v>0</v>
-      </c>
-      <c r="D50">
-        <v>0</v>
-      </c>
-      <c r="E50">
-        <v>0</v>
-      </c>
-      <c r="F50">
-        <v>1</v>
-      </c>
-      <c r="G50">
-        <v>1</v>
-      </c>
-      <c r="H50">
-        <v>0</v>
-      </c>
-      <c r="I50">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9">
-      <c r="A51" t="s">
-        <v>64</v>
-      </c>
-      <c r="B51">
-        <v>0</v>
-      </c>
-      <c r="C51">
-        <v>0</v>
-      </c>
-      <c r="D51">
-        <v>0</v>
-      </c>
-      <c r="E51">
-        <v>0</v>
-      </c>
-      <c r="F51">
-        <v>2</v>
-      </c>
-      <c r="G51">
-        <v>2</v>
-      </c>
-      <c r="H51">
-        <v>0</v>
-      </c>
-      <c r="I51">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9">
-      <c r="A52" s="5" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8">
+      <c r="A50" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B52" s="5">
+      <c r="B50" s="5">
         <v>58</v>
       </c>
-      <c r="C52" s="5">
+      <c r="C50" s="5">
+        <v>76</v>
+      </c>
+      <c r="D50" s="5">
+        <v>61</v>
+      </c>
+      <c r="E50" s="5">
+        <v>123</v>
+      </c>
+      <c r="F50" s="5">
+        <v>127</v>
+      </c>
+      <c r="G50" s="5">
+        <v>140</v>
+      </c>
+      <c r="H50" s="5">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
+      <c r="A51" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B51" s="5">
+        <v>71</v>
+      </c>
+      <c r="C51" s="5">
+        <v>93</v>
+      </c>
+      <c r="D51" s="5">
         <v>75</v>
       </c>
-      <c r="D52" s="5">
-        <v>60</v>
-      </c>
-      <c r="E52" s="5">
-        <v>123</v>
-      </c>
-      <c r="F52" s="5">
-        <v>127</v>
-      </c>
-      <c r="G52" s="5">
-        <v>140</v>
-      </c>
-      <c r="H52" s="5">
-        <v>2</v>
-      </c>
-      <c r="I52" s="5">
-        <v>585</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9">
-      <c r="A53" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="B53" s="5">
-        <v>71</v>
-      </c>
-      <c r="C53" s="5">
-        <v>92</v>
-      </c>
-      <c r="D53" s="5">
-        <v>73</v>
-      </c>
-      <c r="E53" s="5">
+      <c r="E51" s="5">
         <v>149</v>
       </c>
-      <c r="F53" s="5">
-        <v>155</v>
-      </c>
-      <c r="G53" s="5">
-        <v>170</v>
-      </c>
-      <c r="H53" s="5">
-        <v>4</v>
-      </c>
-      <c r="I53" s="5">
-        <v>714</v>
+      <c r="F51" s="5">
+        <v>153</v>
+      </c>
+      <c r="G51" s="5">
+        <v>169</v>
+      </c>
+      <c r="H51" s="5">
+        <v>710</v>
       </c>
     </row>
   </sheetData>
@@ -2772,22 +3136,22 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>38</v>
@@ -2796,10 +3160,10 @@
         <v>39</v>
       </c>
       <c r="D4" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>86</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -2858,16 +3222,16 @@
         <v>58</v>
       </c>
       <c r="B8" s="6">
-        <v>0.1665264928511354</v>
+        <v>0.1707317073170732</v>
       </c>
       <c r="C8" s="6">
         <v>0.178</v>
       </c>
       <c r="D8" s="4">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="E8" s="4">
-        <v>239</v>
+        <v>245</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -2875,16 +3239,16 @@
         <v>59</v>
       </c>
       <c r="B9" s="6">
-        <v>0.07064760302775441</v>
+        <v>0.06644238856181665</v>
       </c>
       <c r="C9" s="6">
         <v>0.011</v>
       </c>
       <c r="D9" s="4">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="E9" s="4">
-        <v>103</v>
+        <v>97</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -2903,12 +3267,12 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>38</v>
@@ -2917,10 +3281,10 @@
         <v>39</v>
       </c>
       <c r="D13" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="E13" s="3" t="s">
         <v>86</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -2928,16 +3292,16 @@
         <v>74</v>
       </c>
       <c r="B14" s="6">
-        <v>0.1216442953020134</v>
+        <v>0.1239460370994941</v>
       </c>
       <c r="C14" s="6">
         <v>0.122</v>
       </c>
       <c r="D14" s="4">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="E14" s="4">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -2945,16 +3309,16 @@
         <v>55</v>
       </c>
       <c r="B15" s="6">
-        <v>0.2441275167785235</v>
+        <v>0.2445193929173693</v>
       </c>
       <c r="C15" s="6">
         <v>0.244</v>
       </c>
       <c r="D15" s="4">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E15" s="4">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -2962,16 +3326,16 @@
         <v>56</v>
       </c>
       <c r="B16" s="6">
-        <v>0.3070469798657718</v>
+        <v>0.3035413153456998</v>
       </c>
       <c r="C16" s="6">
         <v>0.305</v>
       </c>
       <c r="D16" s="4">
-        <v>366</v>
+        <v>360</v>
       </c>
       <c r="E16" s="4">
-        <v>441</v>
+        <v>434</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -2979,16 +3343,16 @@
         <v>57</v>
       </c>
       <c r="B17" s="6">
-        <v>0.1753355704697987</v>
+        <v>0.1770657672849916</v>
       </c>
       <c r="C17" s="6">
         <v>0.176</v>
       </c>
       <c r="D17" s="4">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E17" s="4">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -2996,16 +3360,16 @@
         <v>58</v>
       </c>
       <c r="B18" s="6">
-        <v>0.1518456375838926</v>
+        <v>0.1509274873524452</v>
       </c>
       <c r="C18" s="6">
         <v>0.153</v>
       </c>
       <c r="D18" s="4">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="E18" s="4">
-        <v>220</v>
+        <v>217</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -3019,17 +3383,17 @@
         <v>1</v>
       </c>
       <c r="D19" s="4">
-        <v>1192</v>
+        <v>1186</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>38</v>
@@ -3038,10 +3402,10 @@
         <v>39</v>
       </c>
       <c r="D22" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="E22" s="3" t="s">
         <v>86</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -3066,16 +3430,16 @@
         <v>77</v>
       </c>
       <c r="B24" s="6">
-        <v>0.1282051282051282</v>
+        <v>0.1299145299145299</v>
       </c>
       <c r="C24" s="6">
         <v>0.131</v>
       </c>
       <c r="D24" s="4">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E24" s="4">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -3083,16 +3447,16 @@
         <v>78</v>
       </c>
       <c r="B25" s="6">
-        <v>0.1025641025641026</v>
+        <v>0.1042735042735043</v>
       </c>
       <c r="C25" s="6">
         <v>0.115</v>
       </c>
       <c r="D25" s="4">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E25" s="4">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -3126,7 +3490,7 @@
         <v>127</v>
       </c>
       <c r="E27" s="4">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -3143,37 +3507,20 @@
         <v>140</v>
       </c>
       <c r="E28" s="4">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" t="s">
-        <v>82</v>
-      </c>
-      <c r="B29" s="6">
-        <v>0.003418803418803419</v>
-      </c>
-      <c r="C29" s="6">
-        <v>0</v>
+      <c r="A29" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B29" s="7">
+        <v>1</v>
+      </c>
+      <c r="C29" s="7">
+        <v>1</v>
       </c>
       <c r="D29" s="4">
-        <v>2</v>
-      </c>
-      <c r="E29" s="4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5">
-      <c r="A30" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B30" s="7">
-        <v>1</v>
-      </c>
-      <c r="C30" s="7">
-        <v>1</v>
-      </c>
-      <c r="D30" s="4">
         <v>585</v>
       </c>
     </row>
@@ -3189,12 +3536,12 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -3202,22 +3549,22 @@
         <v>35</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>96</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -3225,22 +3572,22 @@
         <v>40</v>
       </c>
       <c r="B6" s="4">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="C6" s="8">
-        <v>210.46</v>
+        <v>210.5</v>
       </c>
       <c r="D6" s="8">
         <v>107.2</v>
       </c>
       <c r="E6" s="8">
-        <v>317.66</v>
+        <v>317.7</v>
       </c>
       <c r="F6" s="8">
         <v>317.76</v>
       </c>
       <c r="G6" s="8">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -3248,22 +3595,22 @@
         <v>42</v>
       </c>
       <c r="B7" s="4">
-        <v>708</v>
+        <v>703</v>
       </c>
       <c r="C7" s="8">
-        <v>185.68</v>
+        <v>184.58</v>
       </c>
       <c r="D7" s="8">
         <v>94.61</v>
       </c>
       <c r="E7" s="8">
-        <v>280.29</v>
+        <v>279.19</v>
       </c>
       <c r="F7" s="8">
         <v>280.44</v>
       </c>
       <c r="G7" s="8">
-        <v>0.15</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -3271,22 +3618,22 @@
         <v>41</v>
       </c>
       <c r="B8" s="4">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="C8" s="8">
-        <v>168.84</v>
+        <v>168.4</v>
       </c>
       <c r="D8" s="8">
         <v>0</v>
       </c>
       <c r="E8" s="8">
-        <v>168.84</v>
+        <v>168.4</v>
       </c>
       <c r="F8" s="8">
         <v>168.89</v>
       </c>
       <c r="G8" s="8">
-        <v>0.05</v>
+        <v>0.49</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -3340,26 +3687,26 @@
         <v>32</v>
       </c>
       <c r="B11" s="4">
-        <v>2966</v>
+        <v>2960</v>
       </c>
       <c r="E11" s="8">
-        <v>985.21</v>
+        <v>983.71</v>
       </c>
       <c r="F11" s="8">
         <v>985.84</v>
       </c>
       <c r="G11" s="8">
-        <v>0.63</v>
+        <v>2.13</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -3367,7 +3714,7 @@
         <v>26</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -3406,24 +3753,24 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>103</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>104</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>30</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -3478,156 +3825,244 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:11">
       <c r="A1" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="2" t="s">
+    <row r="5" spans="1:11">
+      <c r="A5" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
+      <c r="F5" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="B5" s="8">
-        <v>361.2</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="G5" s="3" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="6" spans="1:3">
+      <c r="H5" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>113</v>
-      </c>
-      <c r="B6" s="8">
-        <v>125.1</v>
-      </c>
-      <c r="C6" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
+        <v>40</v>
+      </c>
+      <c r="B6">
+        <v>322</v>
+      </c>
+      <c r="C6">
+        <v>328</v>
+      </c>
+      <c r="D6">
+        <v>145</v>
+      </c>
+      <c r="E6">
+        <v>795</v>
+      </c>
+      <c r="F6">
+        <v>96.59999999999999</v>
+      </c>
+      <c r="G6">
+        <v>82</v>
+      </c>
+      <c r="H6">
+        <v>31.9</v>
+      </c>
+      <c r="I6">
+        <v>210.5</v>
+      </c>
+      <c r="J6">
+        <v>210.56</v>
+      </c>
+      <c r="K6">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>114</v>
-      </c>
-      <c r="B7" s="8">
-        <v>157</v>
-      </c>
-      <c r="C7" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
+        <v>42</v>
+      </c>
+      <c r="B7">
+        <v>275</v>
+      </c>
+      <c r="C7">
+        <v>264</v>
+      </c>
+      <c r="D7">
+        <v>164</v>
+      </c>
+      <c r="E7">
+        <v>703</v>
+      </c>
+      <c r="F7">
+        <v>82.5</v>
+      </c>
+      <c r="G7">
+        <v>66</v>
+      </c>
+      <c r="H7">
+        <v>36.08</v>
+      </c>
+      <c r="I7">
+        <v>184.58</v>
+      </c>
+      <c r="J7">
+        <v>185.83</v>
+      </c>
+      <c r="K7">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
       <c r="A8" t="s">
-        <v>116</v>
-      </c>
-      <c r="B8" s="8">
-        <v>62.8</v>
-      </c>
-      <c r="C8" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="B9" s="8">
-        <v>706.1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11" s="2" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3">
-      <c r="A12" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3">
-      <c r="A13" t="s">
-        <v>121</v>
-      </c>
-      <c r="B13" s="8">
-        <v>157</v>
-      </c>
-      <c r="C13" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3">
-      <c r="A14" t="s">
-        <v>123</v>
-      </c>
-      <c r="B14" s="8">
-        <v>94.2</v>
-      </c>
-      <c r="C14" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3">
-      <c r="A15" t="s">
-        <v>124</v>
-      </c>
-      <c r="B15" s="8">
-        <v>65.59999999999999</v>
-      </c>
-      <c r="C15" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3">
-      <c r="A16" t="s">
-        <v>125</v>
-      </c>
-      <c r="B16" s="8">
-        <v>65.5</v>
-      </c>
-      <c r="C16" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2">
-      <c r="A17" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="B17" s="8">
-        <v>382.3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2">
-      <c r="A19" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="B19" s="8">
-        <v>1088.4</v>
+        <v>41</v>
+      </c>
+      <c r="B8">
+        <v>283</v>
+      </c>
+      <c r="C8">
+        <v>334</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>617</v>
+      </c>
+      <c r="F8">
+        <v>84.90000000000001</v>
+      </c>
+      <c r="G8">
+        <v>83.5</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>168.4</v>
+      </c>
+      <c r="J8">
+        <v>168.89</v>
+      </c>
+      <c r="K8">
+        <v>0.49</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9">
+        <v>223</v>
+      </c>
+      <c r="C9">
+        <v>191</v>
+      </c>
+      <c r="D9">
+        <v>205</v>
+      </c>
+      <c r="E9">
+        <v>619</v>
+      </c>
+      <c r="F9">
+        <v>66.90000000000001</v>
+      </c>
+      <c r="G9">
+        <v>47.75</v>
+      </c>
+      <c r="H9">
+        <v>45.1</v>
+      </c>
+      <c r="I9">
+        <v>159.75</v>
+      </c>
+      <c r="J9">
+        <v>159.91</v>
+      </c>
+      <c r="K9">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10">
+        <v>86</v>
+      </c>
+      <c r="C10">
+        <v>69</v>
+      </c>
+      <c r="D10">
+        <v>71</v>
+      </c>
+      <c r="E10">
+        <v>226</v>
+      </c>
+      <c r="F10">
+        <v>25.8</v>
+      </c>
+      <c r="G10">
+        <v>17.25</v>
+      </c>
+      <c r="H10">
+        <v>15.62</v>
+      </c>
+      <c r="I10">
+        <v>58.67</v>
+      </c>
+      <c r="J10">
+        <v>58.84</v>
+      </c>
+      <c r="K10">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E11" s="4">
+        <v>2960</v>
+      </c>
+      <c r="I11" s="8">
+        <v>781.9</v>
+      </c>
+      <c r="J11" s="8">
+        <v>784.03</v>
+      </c>
+      <c r="K11" s="8">
+        <v>2.13</v>
       </c>
     </row>
   </sheetData>
@@ -3637,477 +4072,156 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B5" s="8">
+        <v>361.2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>123</v>
+      </c>
+      <c r="B6" s="8">
+        <v>125.1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>124</v>
+      </c>
+      <c r="B7" s="8">
+        <v>157</v>
+      </c>
+      <c r="C7" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>126</v>
+      </c>
+      <c r="B8" s="8">
+        <v>62.8</v>
+      </c>
+      <c r="C8" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="3" t="s">
+      <c r="B9" s="8">
+        <v>706.1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" t="s">
-        <v>40</v>
-      </c>
-      <c r="B5">
-        <v>41</v>
-      </c>
-      <c r="C5">
-        <v>102</v>
-      </c>
-      <c r="D5">
-        <v>103</v>
-      </c>
-      <c r="E5">
-        <v>55</v>
-      </c>
-      <c r="F5">
-        <v>21</v>
-      </c>
-      <c r="G5">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" t="s">
-        <v>41</v>
-      </c>
-      <c r="B6">
-        <v>44</v>
-      </c>
-      <c r="C6">
-        <v>92</v>
-      </c>
-      <c r="D6">
-        <v>85</v>
-      </c>
-      <c r="E6">
-        <v>51</v>
-      </c>
-      <c r="F6">
-        <v>11</v>
-      </c>
-      <c r="G6">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" t="s">
-        <v>42</v>
-      </c>
-      <c r="B7">
-        <v>46</v>
-      </c>
-      <c r="C7">
-        <v>87</v>
-      </c>
-      <c r="D7">
-        <v>94</v>
-      </c>
-      <c r="E7">
-        <v>44</v>
-      </c>
-      <c r="F7">
-        <v>4</v>
-      </c>
-      <c r="G7">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="A8" t="s">
-        <v>43</v>
-      </c>
-      <c r="B8">
-        <v>9</v>
-      </c>
-      <c r="C8">
-        <v>25</v>
-      </c>
-      <c r="D8">
-        <v>26</v>
-      </c>
-      <c r="E8">
-        <v>13</v>
-      </c>
-      <c r="F8">
-        <v>13</v>
-      </c>
-      <c r="G8">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="A9" t="s">
-        <v>44</v>
-      </c>
-      <c r="B9">
-        <v>23</v>
-      </c>
-      <c r="C9">
-        <v>66</v>
-      </c>
-      <c r="D9">
-        <v>64</v>
-      </c>
-      <c r="E9">
-        <v>35</v>
-      </c>
-      <c r="F9">
-        <v>35</v>
-      </c>
-      <c r="G9">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
-      <c r="A11" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
+    </row>
+    <row r="12" spans="1:3">
       <c r="A12" s="3" t="s">
-        <v>129</v>
+        <v>118</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>74</v>
+        <v>119</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>40</v>
-      </c>
-      <c r="B13">
-        <v>53</v>
-      </c>
-      <c r="C13">
-        <v>83</v>
-      </c>
-      <c r="D13">
-        <v>99</v>
-      </c>
-      <c r="E13">
-        <v>50</v>
-      </c>
-      <c r="F13">
-        <v>49</v>
-      </c>
-      <c r="G13">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
+        <v>131</v>
+      </c>
+      <c r="B13" s="8">
+        <v>157</v>
+      </c>
+      <c r="C13" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>41</v>
-      </c>
-      <c r="B14">
-        <v>38</v>
-      </c>
-      <c r="C14">
-        <v>86</v>
-      </c>
-      <c r="D14">
-        <v>104</v>
-      </c>
-      <c r="E14">
-        <v>63</v>
-      </c>
-      <c r="F14">
-        <v>43</v>
-      </c>
-      <c r="G14">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7">
+        <v>133</v>
+      </c>
+      <c r="B14" s="8">
+        <v>94.2</v>
+      </c>
+      <c r="C14" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>42</v>
-      </c>
-      <c r="B15">
-        <v>31</v>
-      </c>
-      <c r="C15">
-        <v>67</v>
-      </c>
-      <c r="D15">
-        <v>77</v>
-      </c>
-      <c r="E15">
-        <v>48</v>
-      </c>
-      <c r="F15">
-        <v>41</v>
-      </c>
-      <c r="G15">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
+        <v>134</v>
+      </c>
+      <c r="B15" s="8">
+        <v>65.59999999999999</v>
+      </c>
+      <c r="C15" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>44</v>
-      </c>
-      <c r="B16">
-        <v>16</v>
-      </c>
-      <c r="C16">
-        <v>38</v>
-      </c>
-      <c r="D16">
-        <v>66</v>
-      </c>
-      <c r="E16">
-        <v>34</v>
-      </c>
-      <c r="F16">
-        <v>37</v>
-      </c>
-      <c r="G16">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9">
-      <c r="A17" t="s">
-        <v>43</v>
-      </c>
-      <c r="B17">
-        <v>7</v>
-      </c>
-      <c r="C17">
-        <v>17</v>
-      </c>
-      <c r="D17">
-        <v>20</v>
-      </c>
-      <c r="E17">
-        <v>14</v>
-      </c>
-      <c r="F17">
-        <v>11</v>
-      </c>
-      <c r="G17">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9">
-      <c r="A19" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9">
-      <c r="A20" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="H20" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="I20" s="3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9">
-      <c r="A21" t="s">
-        <v>44</v>
-      </c>
-      <c r="B21">
-        <v>16</v>
-      </c>
-      <c r="C21">
-        <v>28</v>
-      </c>
-      <c r="D21">
-        <v>20</v>
-      </c>
-      <c r="E21">
-        <v>38</v>
-      </c>
-      <c r="F21">
-        <v>44</v>
-      </c>
-      <c r="G21">
-        <v>58</v>
-      </c>
-      <c r="H21">
-        <v>1</v>
-      </c>
-      <c r="I21">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9">
-      <c r="A22" t="s">
-        <v>43</v>
-      </c>
-      <c r="B22">
-        <v>5</v>
-      </c>
-      <c r="C22">
-        <v>8</v>
-      </c>
-      <c r="D22">
-        <v>11</v>
-      </c>
-      <c r="E22">
-        <v>14</v>
-      </c>
-      <c r="F22">
-        <v>14</v>
-      </c>
-      <c r="G22">
-        <v>19</v>
-      </c>
-      <c r="H22">
-        <v>0</v>
-      </c>
-      <c r="I22">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9">
-      <c r="A23" t="s">
-        <v>40</v>
-      </c>
-      <c r="B23">
-        <v>19</v>
-      </c>
-      <c r="C23">
-        <v>18</v>
-      </c>
-      <c r="D23">
-        <v>15</v>
-      </c>
-      <c r="E23">
-        <v>26</v>
-      </c>
-      <c r="F23">
-        <v>32</v>
-      </c>
-      <c r="G23">
-        <v>28</v>
-      </c>
-      <c r="H23">
-        <v>0</v>
-      </c>
-      <c r="I23">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9">
-      <c r="A24" t="s">
-        <v>42</v>
-      </c>
-      <c r="B24">
-        <v>18</v>
-      </c>
-      <c r="C24">
-        <v>21</v>
-      </c>
-      <c r="D24">
-        <v>14</v>
-      </c>
-      <c r="E24">
-        <v>45</v>
-      </c>
-      <c r="F24">
-        <v>36</v>
-      </c>
-      <c r="G24">
-        <v>34</v>
-      </c>
-      <c r="H24">
-        <v>1</v>
-      </c>
-      <c r="I24">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9">
-      <c r="A25" t="s">
-        <v>41</v>
-      </c>
-      <c r="B25">
-        <v>0</v>
-      </c>
-      <c r="C25">
-        <v>0</v>
-      </c>
-      <c r="D25">
-        <v>0</v>
-      </c>
-      <c r="E25">
-        <v>0</v>
-      </c>
-      <c r="F25">
-        <v>1</v>
-      </c>
-      <c r="G25">
-        <v>1</v>
-      </c>
-      <c r="H25">
-        <v>0</v>
-      </c>
-      <c r="I25">
-        <v>2</v>
+        <v>135</v>
+      </c>
+      <c r="B16" s="8">
+        <v>65.5</v>
+      </c>
+      <c r="C16" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="B17" s="8">
+        <v>382.3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="B19" s="8">
+        <v>1088.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix KIDS Kaki: reservar tela y evitar que Gris lo absorba
Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/EXPLORE_PANTS_Proyeccion_Produccion.xlsx
+++ b/EXPLORE_PANTS_Proyeccion_Produccion.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="151">
   <si>
     <t>EXPLORE PANTS — PROYECCIÓN ANCLADA A JUSTIFICACIÓN NOVAKTEX</t>
   </si>
@@ -1062,10 +1062,10 @@
         <v>29</v>
       </c>
       <c r="B31">
-        <v>1189</v>
+        <v>1170</v>
       </c>
       <c r="C31">
-        <v>1437</v>
+        <v>1414</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -1073,10 +1073,10 @@
         <v>30</v>
       </c>
       <c r="B32">
-        <v>1186</v>
+        <v>1167</v>
       </c>
       <c r="C32">
-        <v>1433</v>
+        <v>1410</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -1087,7 +1087,7 @@
         <v>585</v>
       </c>
       <c r="C33">
-        <v>710</v>
+        <v>712</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -1095,10 +1095,10 @@
         <v>32</v>
       </c>
       <c r="B34" s="5">
-        <v>2960</v>
+        <v>2922</v>
       </c>
       <c r="C34" s="5">
-        <v>3580</v>
+        <v>3536</v>
       </c>
     </row>
   </sheetData>
@@ -1111,7 +1111,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -1178,10 +1178,10 @@
         <v>44</v>
       </c>
       <c r="C6">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="D6">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="E6">
         <v>51</v>
@@ -1190,7 +1190,7 @@
         <v>11</v>
       </c>
       <c r="G6">
-        <v>283</v>
+        <v>264</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -1324,7 +1324,7 @@
         <v>86</v>
       </c>
       <c r="D14">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="E14">
         <v>63</v>
@@ -1333,7 +1333,7 @@
         <v>43</v>
       </c>
       <c r="G14">
-        <v>334</v>
+        <v>315</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -1519,25 +1519,51 @@
         <v>42</v>
       </c>
       <c r="B24">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C24">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D24">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E24">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="F24">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="G24">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="H24">
-        <v>164</v>
+        <v>115</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
+      <c r="A25" t="s">
+        <v>41</v>
+      </c>
+      <c r="B25">
+        <v>5</v>
+      </c>
+      <c r="C25">
+        <v>9</v>
+      </c>
+      <c r="D25">
+        <v>7</v>
+      </c>
+      <c r="E25">
+        <v>6</v>
+      </c>
+      <c r="F25">
+        <v>10</v>
+      </c>
+      <c r="G25">
+        <v>12</v>
+      </c>
+      <c r="H25">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1615,7 +1641,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1662,7 +1688,7 @@
         <v>389</v>
       </c>
       <c r="E5" s="6">
-        <v>0.2708158116063919</v>
+        <v>0.2752136752136752</v>
       </c>
       <c r="F5" s="6">
         <v>0.272</v>
@@ -1676,13 +1702,13 @@
         <v>41</v>
       </c>
       <c r="C6" s="4">
-        <v>283</v>
+        <v>264</v>
       </c>
       <c r="D6" s="4">
-        <v>342</v>
+        <v>319</v>
       </c>
       <c r="E6" s="6">
-        <v>0.2380151387720774</v>
+        <v>0.2256410256410256</v>
       </c>
       <c r="F6" s="6">
         <v>0.21</v>
@@ -1702,7 +1728,7 @@
         <v>332</v>
       </c>
       <c r="E7" s="6">
-        <v>0.2312867956265769</v>
+        <v>0.235042735042735</v>
       </c>
       <c r="F7" s="6">
         <v>0.196</v>
@@ -1722,7 +1748,7 @@
         <v>105</v>
       </c>
       <c r="E8" s="6">
-        <v>0.07232968881412952</v>
+        <v>0.07350427350427351</v>
       </c>
       <c r="F8" s="6">
         <v>0.162</v>
@@ -1742,7 +1768,7 @@
         <v>269</v>
       </c>
       <c r="E9" s="6">
-        <v>0.1875525651808242</v>
+        <v>0.1905982905982906</v>
       </c>
       <c r="F9" s="6">
         <v>0.16</v>
@@ -1753,7 +1779,7 @@
         <v>32</v>
       </c>
       <c r="B10" s="4">
-        <v>1189</v>
+        <v>1170</v>
       </c>
       <c r="C10" s="7">
         <v>1</v>
@@ -1798,7 +1824,7 @@
         <v>395</v>
       </c>
       <c r="E14" s="6">
-        <v>0.2765598650927487</v>
+        <v>0.2810625535561268</v>
       </c>
       <c r="F14" s="6">
         <v>0.298</v>
@@ -1812,13 +1838,13 @@
         <v>41</v>
       </c>
       <c r="C15" s="4">
-        <v>334</v>
+        <v>315</v>
       </c>
       <c r="D15" s="4">
-        <v>403</v>
+        <v>380</v>
       </c>
       <c r="E15" s="6">
-        <v>0.2816188870151771</v>
+        <v>0.2699228791773779</v>
       </c>
       <c r="F15" s="6">
         <v>0.223</v>
@@ -1838,7 +1864,7 @@
         <v>320</v>
       </c>
       <c r="E16" s="6">
-        <v>0.2225969645868466</v>
+        <v>0.2262210796915167</v>
       </c>
       <c r="F16" s="6">
         <v>0.198</v>
@@ -1858,7 +1884,7 @@
         <v>231</v>
       </c>
       <c r="E17" s="6">
-        <v>0.1610455311973019</v>
+        <v>0.1636675235646958</v>
       </c>
       <c r="F17" s="6">
         <v>0.145</v>
@@ -1878,7 +1904,7 @@
         <v>84</v>
       </c>
       <c r="E18" s="6">
-        <v>0.0581787521079258</v>
+        <v>0.05912596401028278</v>
       </c>
       <c r="F18" s="6">
         <v>0.136</v>
@@ -1889,7 +1915,7 @@
         <v>32</v>
       </c>
       <c r="B19" s="4">
-        <v>1186</v>
+        <v>1167</v>
       </c>
       <c r="C19" s="7">
         <v>1</v>
@@ -1988,26 +2014,46 @@
         <v>42</v>
       </c>
       <c r="C26" s="4">
-        <v>164</v>
+        <v>115</v>
       </c>
       <c r="D26" s="4">
-        <v>199</v>
+        <v>140</v>
       </c>
       <c r="E26" s="6">
-        <v>0.2803418803418803</v>
+        <v>0.1965811965811966</v>
       </c>
       <c r="F26" s="6">
         <v>0.154</v>
       </c>
     </row>
     <row r="27" spans="1:6">
-      <c r="A27" s="5" t="s">
+      <c r="A27">
+        <v>5</v>
+      </c>
+      <c r="B27" t="s">
+        <v>41</v>
+      </c>
+      <c r="C27" s="4">
+        <v>49</v>
+      </c>
+      <c r="D27" s="4">
+        <v>61</v>
+      </c>
+      <c r="E27" s="6">
+        <v>0.08376068376068375</v>
+      </c>
+      <c r="F27" s="6">
+        <v>0.08400000000000001</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B27" s="4">
+      <c r="B28" s="4">
         <v>585</v>
       </c>
-      <c r="C27" s="7">
+      <c r="C28" s="7">
         <v>1</v>
       </c>
     </row>
@@ -2051,7 +2097,7 @@
         <v>795</v>
       </c>
       <c r="C4" s="6">
-        <v>0.2685810810810811</v>
+        <v>0.2720739219712526</v>
       </c>
       <c r="D4" s="6">
         <v>0.3223210782341178</v>
@@ -2065,10 +2111,10 @@
         <v>42</v>
       </c>
       <c r="B5" s="4">
-        <v>703</v>
+        <v>654</v>
       </c>
       <c r="C5" s="6">
-        <v>0.2375</v>
+        <v>0.2238193018480493</v>
       </c>
       <c r="D5" s="6">
         <v>0.2844671001033621</v>
@@ -2082,10 +2128,10 @@
         <v>41</v>
       </c>
       <c r="B6" s="4">
-        <v>617</v>
+        <v>628</v>
       </c>
       <c r="C6" s="6">
-        <v>0.208445945945946</v>
+        <v>0.21492128678987</v>
       </c>
       <c r="D6" s="6">
         <v>0.1713177091328877</v>
@@ -2102,7 +2148,7 @@
         <v>619</v>
       </c>
       <c r="C7" s="6">
-        <v>0.2091216216216216</v>
+        <v>0.2118412046543463</v>
       </c>
       <c r="D7" s="6">
         <v>0.1622064538507951</v>
@@ -2119,7 +2165,7 @@
         <v>226</v>
       </c>
       <c r="C8" s="6">
-        <v>0.07635135135135135</v>
+        <v>0.07734428473648186</v>
       </c>
       <c r="D8" s="6">
         <v>0.05968765867883735</v>
@@ -2133,7 +2179,7 @@
         <v>32</v>
       </c>
       <c r="B9" s="4">
-        <v>2960</v>
+        <v>2922</v>
       </c>
       <c r="C9" s="7">
         <v>1</v>
@@ -2152,7 +2198,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -2179,13 +2225,13 @@
         <v>29</v>
       </c>
       <c r="B4">
-        <v>1189</v>
+        <v>1170</v>
       </c>
       <c r="C4">
-        <v>1437</v>
+        <v>1414</v>
       </c>
       <c r="D4">
-        <v>248</v>
+        <v>244</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -2193,13 +2239,13 @@
         <v>30</v>
       </c>
       <c r="B5">
-        <v>1186</v>
+        <v>1167</v>
       </c>
       <c r="C5">
-        <v>1433</v>
+        <v>1410</v>
       </c>
       <c r="D5">
-        <v>247</v>
+        <v>243</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -2210,10 +2256,10 @@
         <v>585</v>
       </c>
       <c r="C6">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="D6">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -2221,13 +2267,13 @@
         <v>32</v>
       </c>
       <c r="B7" s="5">
-        <v>2960</v>
+        <v>2922</v>
       </c>
       <c r="C7" s="5">
-        <v>3580</v>
+        <v>3536</v>
       </c>
       <c r="D7" s="5">
-        <v>620</v>
+        <v>614</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -2312,10 +2358,10 @@
         <v>44</v>
       </c>
       <c r="C14">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="D14">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="E14">
         <v>51</v>
@@ -2324,7 +2370,7 @@
         <v>11</v>
       </c>
       <c r="G14">
-        <v>283</v>
+        <v>264</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -2335,10 +2381,10 @@
         <v>53</v>
       </c>
       <c r="C15">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="D15">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="E15">
         <v>62</v>
@@ -2347,7 +2393,7 @@
         <v>14</v>
       </c>
       <c r="G15">
-        <v>342</v>
+        <v>319</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -2496,10 +2542,10 @@
         <v>163</v>
       </c>
       <c r="C22" s="5">
-        <v>372</v>
+        <v>359</v>
       </c>
       <c r="D22" s="5">
-        <v>372</v>
+        <v>366</v>
       </c>
       <c r="E22" s="5">
         <v>203</v>
@@ -2508,7 +2554,7 @@
         <v>79</v>
       </c>
       <c r="G22" s="5">
-        <v>1189</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -2519,10 +2565,10 @@
         <v>198</v>
       </c>
       <c r="C23" s="5">
-        <v>449</v>
+        <v>433</v>
       </c>
       <c r="D23" s="5">
-        <v>448</v>
+        <v>441</v>
       </c>
       <c r="E23" s="5">
         <v>245</v>
@@ -2531,7 +2577,7 @@
         <v>97</v>
       </c>
       <c r="G23" s="5">
-        <v>1437</v>
+        <v>1414</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -2619,7 +2665,7 @@
         <v>86</v>
       </c>
       <c r="D29">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="E29">
         <v>63</v>
@@ -2628,7 +2674,7 @@
         <v>43</v>
       </c>
       <c r="G29">
-        <v>334</v>
+        <v>315</v>
       </c>
     </row>
     <row r="30" spans="1:7">
@@ -2642,7 +2688,7 @@
         <v>104</v>
       </c>
       <c r="D30">
-        <v>125</v>
+        <v>102</v>
       </c>
       <c r="E30">
         <v>76</v>
@@ -2651,7 +2697,7 @@
         <v>52</v>
       </c>
       <c r="G30">
-        <v>403</v>
+        <v>380</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -2803,7 +2849,7 @@
         <v>290</v>
       </c>
       <c r="D37" s="5">
-        <v>360</v>
+        <v>341</v>
       </c>
       <c r="E37" s="5">
         <v>210</v>
@@ -2812,7 +2858,7 @@
         <v>179</v>
       </c>
       <c r="G37" s="5">
-        <v>1186</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -2826,7 +2872,7 @@
         <v>351</v>
       </c>
       <c r="D38" s="5">
-        <v>434</v>
+        <v>411</v>
       </c>
       <c r="E38" s="5">
         <v>253</v>
@@ -2835,7 +2881,7 @@
         <v>217</v>
       </c>
       <c r="G38" s="5">
-        <v>1433</v>
+        <v>1410</v>
       </c>
     </row>
     <row r="40" spans="1:8">
@@ -3030,25 +3076,25 @@
         <v>65</v>
       </c>
       <c r="B48">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C48">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D48">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E48">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="F48">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="G48">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="H48">
-        <v>164</v>
+        <v>115</v>
       </c>
     </row>
     <row r="49" spans="1:8">
@@ -3056,77 +3102,129 @@
         <v>66</v>
       </c>
       <c r="B49">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="C49">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="D49">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E49">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="F49">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="G49">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="H49">
-        <v>199</v>
+        <v>140</v>
       </c>
     </row>
     <row r="50" spans="1:8">
-      <c r="A50" s="5" t="s">
+      <c r="A50" t="s">
+        <v>63</v>
+      </c>
+      <c r="B50">
+        <v>5</v>
+      </c>
+      <c r="C50">
+        <v>9</v>
+      </c>
+      <c r="D50">
+        <v>7</v>
+      </c>
+      <c r="E50">
+        <v>6</v>
+      </c>
+      <c r="F50">
+        <v>10</v>
+      </c>
+      <c r="G50">
+        <v>12</v>
+      </c>
+      <c r="H50">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
+      <c r="A51" t="s">
+        <v>64</v>
+      </c>
+      <c r="B51">
+        <v>6</v>
+      </c>
+      <c r="C51">
+        <v>11</v>
+      </c>
+      <c r="D51">
+        <v>9</v>
+      </c>
+      <c r="E51">
+        <v>8</v>
+      </c>
+      <c r="F51">
+        <v>12</v>
+      </c>
+      <c r="G51">
+        <v>15</v>
+      </c>
+      <c r="H51">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8">
+      <c r="A52" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B50" s="5">
+      <c r="B52" s="5">
         <v>58</v>
       </c>
-      <c r="C50" s="5">
-        <v>76</v>
-      </c>
-      <c r="D50" s="5">
-        <v>61</v>
-      </c>
-      <c r="E50" s="5">
-        <v>123</v>
-      </c>
-      <c r="F50" s="5">
-        <v>127</v>
-      </c>
-      <c r="G50" s="5">
-        <v>140</v>
-      </c>
-      <c r="H50" s="5">
+      <c r="C52" s="5">
+        <v>79</v>
+      </c>
+      <c r="D52" s="5">
+        <v>64</v>
+      </c>
+      <c r="E52" s="5">
+        <v>116</v>
+      </c>
+      <c r="F52" s="5">
+        <v>126</v>
+      </c>
+      <c r="G52" s="5">
+        <v>142</v>
+      </c>
+      <c r="H52" s="5">
         <v>585</v>
       </c>
     </row>
-    <row r="51" spans="1:8">
-      <c r="A51" s="5" t="s">
+    <row r="53" spans="1:8">
+      <c r="A53" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="B51" s="5">
+      <c r="B53" s="5">
         <v>71</v>
       </c>
-      <c r="C51" s="5">
-        <v>93</v>
-      </c>
-      <c r="D51" s="5">
-        <v>75</v>
-      </c>
-      <c r="E51" s="5">
-        <v>149</v>
-      </c>
-      <c r="F51" s="5">
-        <v>153</v>
-      </c>
-      <c r="G51" s="5">
-        <v>169</v>
-      </c>
-      <c r="H51" s="5">
-        <v>710</v>
+      <c r="C53" s="5">
+        <v>96</v>
+      </c>
+      <c r="D53" s="5">
+        <v>79</v>
+      </c>
+      <c r="E53" s="5">
+        <v>142</v>
+      </c>
+      <c r="F53" s="5">
+        <v>152</v>
+      </c>
+      <c r="G53" s="5">
+        <v>172</v>
+      </c>
+      <c r="H53" s="5">
+        <v>712</v>
       </c>
     </row>
   </sheetData>
@@ -3171,7 +3269,7 @@
         <v>55</v>
       </c>
       <c r="B5" s="6">
-        <v>0.1370899915895711</v>
+        <v>0.1393162393162393</v>
       </c>
       <c r="C5" s="6">
         <v>0.141</v>
@@ -3188,16 +3286,16 @@
         <v>56</v>
       </c>
       <c r="B6" s="6">
-        <v>0.3128679562657696</v>
+        <v>0.3068376068376069</v>
       </c>
       <c r="C6" s="6">
         <v>0.334</v>
       </c>
       <c r="D6" s="4">
-        <v>372</v>
+        <v>359</v>
       </c>
       <c r="E6" s="4">
-        <v>449</v>
+        <v>433</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -3205,16 +3303,16 @@
         <v>57</v>
       </c>
       <c r="B7" s="6">
-        <v>0.3128679562657696</v>
+        <v>0.3128205128205128</v>
       </c>
       <c r="C7" s="6">
         <v>0.336</v>
       </c>
       <c r="D7" s="4">
-        <v>372</v>
+        <v>366</v>
       </c>
       <c r="E7" s="4">
-        <v>448</v>
+        <v>441</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -3222,7 +3320,7 @@
         <v>58</v>
       </c>
       <c r="B8" s="6">
-        <v>0.1707317073170732</v>
+        <v>0.1735042735042735</v>
       </c>
       <c r="C8" s="6">
         <v>0.178</v>
@@ -3239,7 +3337,7 @@
         <v>59</v>
       </c>
       <c r="B9" s="6">
-        <v>0.06644238856181665</v>
+        <v>0.06752136752136752</v>
       </c>
       <c r="C9" s="6">
         <v>0.011</v>
@@ -3262,7 +3360,7 @@
         <v>1</v>
       </c>
       <c r="D10" s="4">
-        <v>1189</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -3292,7 +3390,7 @@
         <v>74</v>
       </c>
       <c r="B14" s="6">
-        <v>0.1239460370994941</v>
+        <v>0.1259640102827763</v>
       </c>
       <c r="C14" s="6">
         <v>0.122</v>
@@ -3309,7 +3407,7 @@
         <v>55</v>
       </c>
       <c r="B15" s="6">
-        <v>0.2445193929173693</v>
+        <v>0.2485004284490146</v>
       </c>
       <c r="C15" s="6">
         <v>0.244</v>
@@ -3326,16 +3424,16 @@
         <v>56</v>
       </c>
       <c r="B16" s="6">
-        <v>0.3035413153456998</v>
+        <v>0.2922022279348758</v>
       </c>
       <c r="C16" s="6">
         <v>0.305</v>
       </c>
       <c r="D16" s="4">
-        <v>360</v>
+        <v>341</v>
       </c>
       <c r="E16" s="4">
-        <v>434</v>
+        <v>411</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -3343,7 +3441,7 @@
         <v>57</v>
       </c>
       <c r="B17" s="6">
-        <v>0.1770657672849916</v>
+        <v>0.1799485861182519</v>
       </c>
       <c r="C17" s="6">
         <v>0.176</v>
@@ -3360,7 +3458,7 @@
         <v>58</v>
       </c>
       <c r="B18" s="6">
-        <v>0.1509274873524452</v>
+        <v>0.1533847472150814</v>
       </c>
       <c r="C18" s="6">
         <v>0.153</v>
@@ -3383,7 +3481,7 @@
         <v>1</v>
       </c>
       <c r="D19" s="4">
-        <v>1186</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -3430,16 +3528,16 @@
         <v>77</v>
       </c>
       <c r="B24" s="6">
-        <v>0.1299145299145299</v>
+        <v>0.135042735042735</v>
       </c>
       <c r="C24" s="6">
         <v>0.131</v>
       </c>
       <c r="D24" s="4">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="E24" s="4">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -3447,16 +3545,16 @@
         <v>78</v>
       </c>
       <c r="B25" s="6">
-        <v>0.1042735042735043</v>
+        <v>0.1094017094017094</v>
       </c>
       <c r="C25" s="6">
         <v>0.115</v>
       </c>
       <c r="D25" s="4">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="E25" s="4">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -3464,16 +3562,16 @@
         <v>79</v>
       </c>
       <c r="B26" s="6">
-        <v>0.2102564102564103</v>
+        <v>0.1982905982905983</v>
       </c>
       <c r="C26" s="6">
         <v>0.198</v>
       </c>
       <c r="D26" s="4">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="E26" s="4">
-        <v>149</v>
+        <v>142</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -3481,16 +3579,16 @@
         <v>80</v>
       </c>
       <c r="B27" s="6">
-        <v>0.2170940170940171</v>
+        <v>0.2153846153846154</v>
       </c>
       <c r="C27" s="6">
         <v>0.215</v>
       </c>
       <c r="D27" s="4">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E27" s="4">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -3498,16 +3596,16 @@
         <v>81</v>
       </c>
       <c r="B28" s="6">
-        <v>0.2393162393162393</v>
+        <v>0.2427350427350427</v>
       </c>
       <c r="C28" s="6">
         <v>0.248</v>
       </c>
       <c r="D28" s="4">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="E28" s="4">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -3595,22 +3693,22 @@
         <v>42</v>
       </c>
       <c r="B7" s="4">
-        <v>703</v>
+        <v>654</v>
       </c>
       <c r="C7" s="8">
-        <v>184.58</v>
+        <v>173.8</v>
       </c>
       <c r="D7" s="8">
         <v>94.61</v>
       </c>
       <c r="E7" s="8">
-        <v>279.19</v>
+        <v>268.41</v>
       </c>
       <c r="F7" s="8">
         <v>280.44</v>
       </c>
       <c r="G7" s="8">
-        <v>1.25</v>
+        <v>12.03</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -3618,22 +3716,22 @@
         <v>41</v>
       </c>
       <c r="B8" s="4">
-        <v>617</v>
+        <v>628</v>
       </c>
       <c r="C8" s="8">
-        <v>168.4</v>
+        <v>168.73</v>
       </c>
       <c r="D8" s="8">
         <v>0</v>
       </c>
       <c r="E8" s="8">
-        <v>168.4</v>
+        <v>168.73</v>
       </c>
       <c r="F8" s="8">
         <v>168.89</v>
       </c>
       <c r="G8" s="8">
-        <v>0.49</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -3687,16 +3785,16 @@
         <v>32</v>
       </c>
       <c r="B11" s="4">
-        <v>2960</v>
+        <v>2922</v>
       </c>
       <c r="E11" s="8">
-        <v>983.71</v>
+        <v>973.26</v>
       </c>
       <c r="F11" s="8">
         <v>985.84</v>
       </c>
       <c r="G11" s="8">
-        <v>2.13</v>
+        <v>12.58</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -3919,10 +4017,10 @@
         <v>264</v>
       </c>
       <c r="D7">
-        <v>164</v>
+        <v>115</v>
       </c>
       <c r="E7">
-        <v>703</v>
+        <v>654</v>
       </c>
       <c r="F7">
         <v>82.5</v>
@@ -3931,16 +4029,16 @@
         <v>66</v>
       </c>
       <c r="H7">
-        <v>36.08</v>
+        <v>25.3</v>
       </c>
       <c r="I7">
-        <v>184.58</v>
+        <v>173.8</v>
       </c>
       <c r="J7">
         <v>185.83</v>
       </c>
       <c r="K7">
-        <v>1.25</v>
+        <v>12.03</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -3948,34 +4046,34 @@
         <v>41</v>
       </c>
       <c r="B8">
-        <v>283</v>
+        <v>264</v>
       </c>
       <c r="C8">
-        <v>334</v>
+        <v>315</v>
       </c>
       <c r="D8">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E8">
-        <v>617</v>
+        <v>628</v>
       </c>
       <c r="F8">
-        <v>84.90000000000001</v>
+        <v>79.2</v>
       </c>
       <c r="G8">
-        <v>83.5</v>
+        <v>78.75</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>10.78</v>
       </c>
       <c r="I8">
-        <v>168.4</v>
+        <v>168.73</v>
       </c>
       <c r="J8">
         <v>168.89</v>
       </c>
       <c r="K8">
-        <v>0.49</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -4053,16 +4151,16 @@
         <v>32</v>
       </c>
       <c r="E11" s="4">
-        <v>2960</v>
+        <v>2922</v>
       </c>
       <c r="I11" s="8">
-        <v>781.9</v>
+        <v>771.45</v>
       </c>
       <c r="J11" s="8">
         <v>784.03</v>
       </c>
       <c r="K11" s="8">
-        <v>2.13</v>
+        <v>12.58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Aplicar matrices manuales CAB/DAMA/KIDS al Excel (dashboard)
Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/EXPLORE_PANTS_Proyeccion_Produccion.xlsx
+++ b/EXPLORE_PANTS_Proyeccion_Produccion.xlsx
@@ -165,7 +165,7 @@
     <t>EXPLORE PANTS — UNIDADES A PRODUCIR POR COLOR (TOTAL)</t>
   </si>
   <si>
-    <t>Generado: 2026-09-23 15:21 UTC</t>
+    <t>Generado: 2026-09-23 15:37 UTC</t>
   </si>
   <si>
     <t>Und CAB</t>
@@ -1103,7 +1103,7 @@
         <v>585</v>
       </c>
       <c r="C33">
-        <v>712</v>
+        <v>711</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -1114,7 +1114,7 @@
         <v>2905</v>
       </c>
       <c r="C34" s="5">
-        <v>3516</v>
+        <v>3515</v>
       </c>
     </row>
   </sheetData>
@@ -1419,19 +1419,19 @@
         <v>44</v>
       </c>
       <c r="B9">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C9">
         <v>66</v>
       </c>
       <c r="D9">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="E9">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="F9">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="G9">
         <v>223</v>
@@ -1496,10 +1496,10 @@
         <v>38</v>
       </c>
       <c r="C14">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="D14">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="E14">
         <v>63</v>
@@ -1542,10 +1542,10 @@
         <v>23</v>
       </c>
       <c r="C16">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="D16">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="E16">
         <v>30</v>
@@ -1565,13 +1565,13 @@
         <v>10</v>
       </c>
       <c r="C17">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D17">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E17">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F17">
         <v>10</v>
@@ -1668,22 +1668,22 @@
         <v>40</v>
       </c>
       <c r="B23">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C23">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D23">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E23">
         <v>27</v>
       </c>
       <c r="F23">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="G23">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="H23">
         <v>145</v>
@@ -1694,22 +1694,22 @@
         <v>42</v>
       </c>
       <c r="B24">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C24">
         <v>12</v>
       </c>
       <c r="D24">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E24">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F24">
         <v>20</v>
       </c>
       <c r="G24">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="H24">
         <v>94</v>
@@ -1723,13 +1723,13 @@
         <v>6</v>
       </c>
       <c r="C25">
+        <v>10</v>
+      </c>
+      <c r="D25">
+        <v>10</v>
+      </c>
+      <c r="E25">
         <v>13</v>
-      </c>
-      <c r="D25">
-        <v>11</v>
-      </c>
-      <c r="E25">
-        <v>9</v>
       </c>
       <c r="F25">
         <v>14</v>
@@ -2212,7 +2212,7 @@
         <v>70</v>
       </c>
       <c r="D27" s="4">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E27" s="6">
         <v>0.1196581196581197</v>
@@ -2548,22 +2548,22 @@
         <v>40</v>
       </c>
       <c r="B6">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C6">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D6">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E6">
         <v>27</v>
       </c>
       <c r="F6">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="G6">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="H6">
         <v>145</v>
@@ -2574,22 +2574,22 @@
         <v>42</v>
       </c>
       <c r="B7">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C7">
         <v>12</v>
       </c>
       <c r="D7">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E7">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F7">
         <v>20</v>
       </c>
       <c r="G7">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="H7">
         <v>94</v>
@@ -2603,13 +2603,13 @@
         <v>6</v>
       </c>
       <c r="C8">
+        <v>10</v>
+      </c>
+      <c r="D8">
+        <v>10</v>
+      </c>
+      <c r="E8">
         <v>13</v>
-      </c>
-      <c r="D8">
-        <v>11</v>
-      </c>
-      <c r="E8">
-        <v>9</v>
       </c>
       <c r="F8">
         <v>14</v>
@@ -2694,10 +2694,10 @@
         <v>585</v>
       </c>
       <c r="C6">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="D6">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -2708,10 +2708,10 @@
         <v>2905</v>
       </c>
       <c r="C7" s="5">
-        <v>3516</v>
+        <v>3515</v>
       </c>
       <c r="D7" s="5">
-        <v>611</v>
+        <v>610</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -2931,19 +2931,19 @@
         <v>85</v>
       </c>
       <c r="B20">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C20">
         <v>66</v>
       </c>
       <c r="D20">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="E20">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="F20">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="G20">
         <v>223</v>
@@ -2954,19 +2954,19 @@
         <v>86</v>
       </c>
       <c r="B21">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="C21">
         <v>80</v>
       </c>
       <c r="D21">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="E21">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="F21">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="G21">
         <v>269</v>
@@ -2977,19 +2977,19 @@
         <v>87</v>
       </c>
       <c r="B22" s="5">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="C22" s="5">
         <v>354</v>
       </c>
       <c r="D22" s="5">
-        <v>362</v>
+        <v>368</v>
       </c>
       <c r="E22" s="5">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="F22" s="5">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="G22" s="5">
         <v>1161</v>
@@ -3000,19 +3000,19 @@
         <v>88</v>
       </c>
       <c r="B23" s="5">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="C23" s="5">
         <v>427</v>
       </c>
       <c r="D23" s="5">
-        <v>436</v>
+        <v>443</v>
       </c>
       <c r="E23" s="5">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="F23" s="5">
-        <v>97</v>
+        <v>76</v>
       </c>
       <c r="G23" s="5">
         <v>1403</v>
@@ -3100,10 +3100,10 @@
         <v>38</v>
       </c>
       <c r="C29">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="D29">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="E29">
         <v>63</v>
@@ -3123,10 +3123,10 @@
         <v>46</v>
       </c>
       <c r="C30">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="D30">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="E30">
         <v>76</v>
@@ -3192,10 +3192,10 @@
         <v>23</v>
       </c>
       <c r="C33">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="D33">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="E33">
         <v>30</v>
@@ -3215,10 +3215,10 @@
         <v>28</v>
       </c>
       <c r="C34">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="D34">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="E34">
         <v>36</v>
@@ -3238,13 +3238,13 @@
         <v>10</v>
       </c>
       <c r="C35">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D35">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E35">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F35">
         <v>10</v>
@@ -3261,13 +3261,13 @@
         <v>12</v>
       </c>
       <c r="C36">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D36">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E36">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F36">
         <v>12</v>
@@ -3284,13 +3284,13 @@
         <v>147</v>
       </c>
       <c r="C37" s="5">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="D37" s="5">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="E37" s="5">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F37" s="5">
         <v>179</v>
@@ -3307,13 +3307,13 @@
         <v>178</v>
       </c>
       <c r="C38" s="5">
-        <v>346</v>
+        <v>352</v>
       </c>
       <c r="D38" s="5">
-        <v>407</v>
+        <v>403</v>
       </c>
       <c r="E38" s="5">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="F38" s="5">
         <v>217</v>
@@ -3462,22 +3462,22 @@
         <v>77</v>
       </c>
       <c r="B46">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C46">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D46">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E46">
         <v>27</v>
       </c>
       <c r="F46">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="G46">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="H46">
         <v>145</v>
@@ -3488,22 +3488,22 @@
         <v>78</v>
       </c>
       <c r="B47">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C47">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D47">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E47">
         <v>33</v>
       </c>
       <c r="F47">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="G47">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="H47">
         <v>176</v>
@@ -3514,22 +3514,22 @@
         <v>81</v>
       </c>
       <c r="B48">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C48">
         <v>12</v>
       </c>
       <c r="D48">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E48">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F48">
         <v>20</v>
       </c>
       <c r="G48">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="H48">
         <v>94</v>
@@ -3540,22 +3540,22 @@
         <v>82</v>
       </c>
       <c r="B49">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C49">
         <v>15</v>
       </c>
       <c r="D49">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E49">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F49">
         <v>24</v>
       </c>
       <c r="G49">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="H49">
         <v>114</v>
@@ -3569,13 +3569,13 @@
         <v>6</v>
       </c>
       <c r="C50">
+        <v>10</v>
+      </c>
+      <c r="D50">
+        <v>10</v>
+      </c>
+      <c r="E50">
         <v>13</v>
-      </c>
-      <c r="D50">
-        <v>11</v>
-      </c>
-      <c r="E50">
-        <v>9</v>
       </c>
       <c r="F50">
         <v>14</v>
@@ -3595,13 +3595,13 @@
         <v>8</v>
       </c>
       <c r="C51">
+        <v>12</v>
+      </c>
+      <c r="D51">
+        <v>12</v>
+      </c>
+      <c r="E51">
         <v>16</v>
-      </c>
-      <c r="D51">
-        <v>14</v>
-      </c>
-      <c r="E51">
-        <v>11</v>
       </c>
       <c r="F51">
         <v>17</v>
@@ -3610,7 +3610,7 @@
         <v>21</v>
       </c>
       <c r="H51">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="52" spans="1:8">
@@ -3618,22 +3618,22 @@
         <v>87</v>
       </c>
       <c r="B52" s="5">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="C52" s="5">
         <v>80</v>
       </c>
       <c r="D52" s="5">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E52" s="5">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F52" s="5">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G52" s="5">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="H52" s="5">
         <v>585</v>
@@ -3644,25 +3644,25 @@
         <v>88</v>
       </c>
       <c r="B53" s="5">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="C53" s="5">
         <v>98</v>
       </c>
       <c r="D53" s="5">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E53" s="5">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F53" s="5">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="G53" s="5">
-        <v>173</v>
+        <v>184</v>
       </c>
       <c r="H53" s="5">
-        <v>712</v>
+        <v>711</v>
       </c>
     </row>
   </sheetData>
@@ -3707,16 +3707,16 @@
         <v>72</v>
       </c>
       <c r="B5" s="6">
-        <v>0.140396210163652</v>
+        <v>0.1464254952627046</v>
       </c>
       <c r="C5" s="6">
         <v>0.141</v>
       </c>
       <c r="D5" s="4">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="E5" s="4">
-        <v>198</v>
+        <v>206</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -3741,16 +3741,16 @@
         <v>74</v>
       </c>
       <c r="B7" s="6">
-        <v>0.3118001722652886</v>
+        <v>0.3169681309216193</v>
       </c>
       <c r="C7" s="6">
         <v>0.336</v>
       </c>
       <c r="D7" s="4">
-        <v>362</v>
+        <v>368</v>
       </c>
       <c r="E7" s="4">
-        <v>436</v>
+        <v>443</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -3758,16 +3758,16 @@
         <v>75</v>
       </c>
       <c r="B8" s="6">
-        <v>0.1748492678725237</v>
+        <v>0.1791559000861326</v>
       </c>
       <c r="C8" s="6">
         <v>0.178</v>
       </c>
       <c r="D8" s="4">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="E8" s="4">
-        <v>245</v>
+        <v>251</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -3775,16 +3775,16 @@
         <v>76</v>
       </c>
       <c r="B9" s="6">
-        <v>0.06804478897502153</v>
+        <v>0.05254091300602928</v>
       </c>
       <c r="C9" s="6">
         <v>0.011</v>
       </c>
       <c r="D9" s="4">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="E9" s="4">
-        <v>97</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -3845,16 +3845,16 @@
         <v>72</v>
       </c>
       <c r="B15" s="6">
-        <v>0.2467644521138913</v>
+        <v>0.2510785159620362</v>
       </c>
       <c r="C15" s="6">
         <v>0.244</v>
       </c>
       <c r="D15" s="4">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="E15" s="4">
-        <v>346</v>
+        <v>352</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -3862,16 +3862,16 @@
         <v>73</v>
       </c>
       <c r="B16" s="6">
-        <v>0.2907679033649698</v>
+        <v>0.2881794650560828</v>
       </c>
       <c r="C16" s="6">
         <v>0.305</v>
       </c>
       <c r="D16" s="4">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="E16" s="4">
-        <v>407</v>
+        <v>403</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -3879,16 +3879,16 @@
         <v>74</v>
       </c>
       <c r="B17" s="6">
-        <v>0.181190681622088</v>
+        <v>0.17946505608283</v>
       </c>
       <c r="C17" s="6">
         <v>0.176</v>
       </c>
       <c r="D17" s="4">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E17" s="4">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -3949,16 +3949,16 @@
         <v>59</v>
       </c>
       <c r="B23" s="6">
-        <v>0.09743589743589744</v>
+        <v>0.08547008547008547</v>
       </c>
       <c r="C23" s="6">
         <v>0.09300000000000001</v>
       </c>
       <c r="D23" s="4">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="E23" s="4">
-        <v>70</v>
+        <v>62</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -3983,16 +3983,16 @@
         <v>61</v>
       </c>
       <c r="B25" s="6">
-        <v>0.1128205128205128</v>
+        <v>0.1179487179487179</v>
       </c>
       <c r="C25" s="6">
         <v>0.115</v>
       </c>
       <c r="D25" s="4">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E25" s="4">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -4000,16 +4000,16 @@
         <v>62</v>
       </c>
       <c r="B26" s="6">
-        <v>0.1931623931623932</v>
+        <v>0.1914529914529915</v>
       </c>
       <c r="C26" s="6">
         <v>0.198</v>
       </c>
       <c r="D26" s="4">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E26" s="4">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -4017,16 +4017,16 @@
         <v>63</v>
       </c>
       <c r="B27" s="6">
-        <v>0.2153846153846154</v>
+        <v>0.2085470085470086</v>
       </c>
       <c r="C27" s="6">
         <v>0.215</v>
       </c>
       <c r="D27" s="4">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E27" s="4">
-        <v>152</v>
+        <v>147</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -4034,16 +4034,16 @@
         <v>64</v>
       </c>
       <c r="B28" s="6">
-        <v>0.2444444444444444</v>
+        <v>0.2598290598290598</v>
       </c>
       <c r="C28" s="6">
         <v>0.248</v>
       </c>
       <c r="D28" s="4">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="E28" s="4">
-        <v>173</v>
+        <v>184</v>
       </c>
     </row>
     <row r="29" spans="1:5">

</xml_diff>